<commit_message>
chore: atualiza histórico de ordens 2026-09-14
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E523"/>
+  <dimension ref="A1:E552"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10746,7 +10746,7 @@
       </c>
     </row>
     <row r="495">
-      <c r="A495" s="2" t="n">
+      <c r="A495" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B495" t="inlineStr">
@@ -10767,7 +10767,7 @@
       </c>
     </row>
     <row r="496">
-      <c r="A496" s="2" t="n">
+      <c r="A496" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B496" t="inlineStr">
@@ -10788,7 +10788,7 @@
       </c>
     </row>
     <row r="497">
-      <c r="A497" s="2" t="n">
+      <c r="A497" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B497" t="inlineStr">
@@ -10809,7 +10809,7 @@
       </c>
     </row>
     <row r="498">
-      <c r="A498" s="2" t="n">
+      <c r="A498" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B498" t="inlineStr">
@@ -10830,7 +10830,7 @@
       </c>
     </row>
     <row r="499">
-      <c r="A499" s="2" t="n">
+      <c r="A499" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B499" t="inlineStr">
@@ -10851,7 +10851,7 @@
       </c>
     </row>
     <row r="500">
-      <c r="A500" s="2" t="n">
+      <c r="A500" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B500" t="inlineStr">
@@ -10872,7 +10872,7 @@
       </c>
     </row>
     <row r="501">
-      <c r="A501" s="2" t="n">
+      <c r="A501" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B501" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
     </row>
     <row r="502">
-      <c r="A502" s="2" t="n">
+      <c r="A502" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B502" t="inlineStr">
@@ -10914,7 +10914,7 @@
       </c>
     </row>
     <row r="503">
-      <c r="A503" s="2" t="n">
+      <c r="A503" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B503" t="inlineStr">
@@ -10935,7 +10935,7 @@
       </c>
     </row>
     <row r="504">
-      <c r="A504" s="2" t="n">
+      <c r="A504" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B504" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
     </row>
     <row r="505">
-      <c r="A505" s="2" t="n">
+      <c r="A505" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B505" t="inlineStr">
@@ -10977,7 +10977,7 @@
       </c>
     </row>
     <row r="506">
-      <c r="A506" s="2" t="n">
+      <c r="A506" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B506" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
     </row>
     <row r="507">
-      <c r="A507" s="2" t="n">
+      <c r="A507" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B507" t="inlineStr">
@@ -11019,7 +11019,7 @@
       </c>
     </row>
     <row r="508">
-      <c r="A508" s="2" t="n">
+      <c r="A508" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B508" t="inlineStr">
@@ -11040,7 +11040,7 @@
       </c>
     </row>
     <row r="509">
-      <c r="A509" s="2" t="n">
+      <c r="A509" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B509" t="inlineStr">
@@ -11061,7 +11061,7 @@
       </c>
     </row>
     <row r="510">
-      <c r="A510" s="2" t="n">
+      <c r="A510" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B510" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
     </row>
     <row r="511">
-      <c r="A511" s="2" t="n">
+      <c r="A511" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B511" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
     </row>
     <row r="512">
-      <c r="A512" s="2" t="n">
+      <c r="A512" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B512" t="inlineStr">
@@ -11124,7 +11124,7 @@
       </c>
     </row>
     <row r="513">
-      <c r="A513" s="2" t="n">
+      <c r="A513" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B513" t="inlineStr">
@@ -11145,7 +11145,7 @@
       </c>
     </row>
     <row r="514">
-      <c r="A514" s="2" t="n">
+      <c r="A514" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B514" t="inlineStr">
@@ -11166,7 +11166,7 @@
       </c>
     </row>
     <row r="515">
-      <c r="A515" s="2" t="n">
+      <c r="A515" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B515" t="inlineStr">
@@ -11187,7 +11187,7 @@
       </c>
     </row>
     <row r="516">
-      <c r="A516" s="2" t="n">
+      <c r="A516" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B516" t="inlineStr">
@@ -11208,7 +11208,7 @@
       </c>
     </row>
     <row r="517">
-      <c r="A517" s="2" t="n">
+      <c r="A517" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B517" t="inlineStr">
@@ -11229,7 +11229,7 @@
       </c>
     </row>
     <row r="518">
-      <c r="A518" s="2" t="n">
+      <c r="A518" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B518" t="inlineStr">
@@ -11250,7 +11250,7 @@
       </c>
     </row>
     <row r="519">
-      <c r="A519" s="2" t="n">
+      <c r="A519" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B519" t="inlineStr">
@@ -11271,7 +11271,7 @@
       </c>
     </row>
     <row r="520">
-      <c r="A520" s="2" t="n">
+      <c r="A520" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B520" t="inlineStr">
@@ -11292,7 +11292,7 @@
       </c>
     </row>
     <row r="521">
-      <c r="A521" s="2" t="n">
+      <c r="A521" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B521" t="inlineStr">
@@ -11313,7 +11313,7 @@
       </c>
     </row>
     <row r="522">
-      <c r="A522" s="2" t="n">
+      <c r="A522" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B522" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
     </row>
     <row r="523">
-      <c r="A523" s="2" t="n">
+      <c r="A523" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="B523" t="inlineStr">
@@ -11349,6 +11349,615 @@
         <v>48</v>
       </c>
       <c r="E523" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C524" t="n">
+        <v>28.44000053405762</v>
+      </c>
+      <c r="D524" t="n">
+        <v>28</v>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C525" t="n">
+        <v>13.09000015258789</v>
+      </c>
+      <c r="D525" t="n">
+        <v>31</v>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C526" t="n">
+        <v>22.20000076293945</v>
+      </c>
+      <c r="D526" t="n">
+        <v>30</v>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C527" t="n">
+        <v>4.119999885559082</v>
+      </c>
+      <c r="D527" t="n">
+        <v>16</v>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C528" t="n">
+        <v>0.7699999809265137</v>
+      </c>
+      <c r="D528" t="n">
+        <v>12</v>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C529" t="n">
+        <v>183.2700042724609</v>
+      </c>
+      <c r="D529" t="n">
+        <v>26</v>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C530" t="n">
+        <v>60.83000183105469</v>
+      </c>
+      <c r="D530" t="n">
+        <v>45</v>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C531" t="n">
+        <v>5.070000171661377</v>
+      </c>
+      <c r="D531" t="n">
+        <v>61</v>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C532" t="n">
+        <v>6.230000019073486</v>
+      </c>
+      <c r="D532" t="n">
+        <v>10</v>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C533" t="n">
+        <v>6.349999904632568</v>
+      </c>
+      <c r="D533" t="n">
+        <v>22</v>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C534" t="n">
+        <v>20.09000015258789</v>
+      </c>
+      <c r="D534" t="n">
+        <v>49</v>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C535" t="n">
+        <v>26.89999961853027</v>
+      </c>
+      <c r="D535" t="n">
+        <v>20</v>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C536" t="n">
+        <v>12.90999984741211</v>
+      </c>
+      <c r="D536" t="n">
+        <v>9</v>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C537" t="n">
+        <v>4.860000133514404</v>
+      </c>
+      <c r="D537" t="n">
+        <v>26</v>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C538" t="n">
+        <v>23.48999977111816</v>
+      </c>
+      <c r="D538" t="n">
+        <v>27</v>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C539" t="n">
+        <v>11.80000019073486</v>
+      </c>
+      <c r="D539" t="n">
+        <v>22</v>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C540" t="n">
+        <v>5.570000171661377</v>
+      </c>
+      <c r="D540" t="n">
+        <v>20</v>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C541" t="n">
+        <v>7.800000190734863</v>
+      </c>
+      <c r="D541" t="n">
+        <v>25</v>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C542" t="n">
+        <v>5.539999961853027</v>
+      </c>
+      <c r="D542" t="n">
+        <v>30</v>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C543" t="n">
+        <v>49.11000061035156</v>
+      </c>
+      <c r="D543" t="n">
+        <v>23</v>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C544" t="n">
+        <v>4.460000038146973</v>
+      </c>
+      <c r="D544" t="n">
+        <v>20</v>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C545" t="n">
+        <v>64.01000213623047</v>
+      </c>
+      <c r="D545" t="n">
+        <v>8</v>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C546" t="n">
+        <v>50.20999908447266</v>
+      </c>
+      <c r="D546" t="n">
+        <v>16</v>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C547" t="n">
+        <v>19.6299991607666</v>
+      </c>
+      <c r="D547" t="n">
+        <v>63</v>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C548" t="n">
+        <v>36.95999908447266</v>
+      </c>
+      <c r="D548" t="n">
+        <v>35</v>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C549" t="n">
+        <v>110.129997253418</v>
+      </c>
+      <c r="D549" t="n">
+        <v>31</v>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C550" t="n">
+        <v>47.34999847412109</v>
+      </c>
+      <c r="D550" t="n">
+        <v>11</v>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C551" t="n">
+        <v>7.03000020980835</v>
+      </c>
+      <c r="D551" t="n">
+        <v>11</v>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C552" t="n">
+        <v>37.81999969482422</v>
+      </c>
+      <c r="D552" t="n">
+        <v>48</v>
+      </c>
+      <c r="E552" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-15
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E552"/>
+  <dimension ref="A1:E581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11355,7 +11355,7 @@
       </c>
     </row>
     <row r="524">
-      <c r="A524" s="2" t="n">
+      <c r="A524" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B524" t="inlineStr">
@@ -11376,7 +11376,7 @@
       </c>
     </row>
     <row r="525">
-      <c r="A525" s="2" t="n">
+      <c r="A525" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B525" t="inlineStr">
@@ -11397,7 +11397,7 @@
       </c>
     </row>
     <row r="526">
-      <c r="A526" s="2" t="n">
+      <c r="A526" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B526" t="inlineStr">
@@ -11418,7 +11418,7 @@
       </c>
     </row>
     <row r="527">
-      <c r="A527" s="2" t="n">
+      <c r="A527" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B527" t="inlineStr">
@@ -11439,7 +11439,7 @@
       </c>
     </row>
     <row r="528">
-      <c r="A528" s="2" t="n">
+      <c r="A528" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B528" t="inlineStr">
@@ -11460,7 +11460,7 @@
       </c>
     </row>
     <row r="529">
-      <c r="A529" s="2" t="n">
+      <c r="A529" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B529" t="inlineStr">
@@ -11481,7 +11481,7 @@
       </c>
     </row>
     <row r="530">
-      <c r="A530" s="2" t="n">
+      <c r="A530" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B530" t="inlineStr">
@@ -11502,7 +11502,7 @@
       </c>
     </row>
     <row r="531">
-      <c r="A531" s="2" t="n">
+      <c r="A531" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B531" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
     </row>
     <row r="532">
-      <c r="A532" s="2" t="n">
+      <c r="A532" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B532" t="inlineStr">
@@ -11544,7 +11544,7 @@
       </c>
     </row>
     <row r="533">
-      <c r="A533" s="2" t="n">
+      <c r="A533" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B533" t="inlineStr">
@@ -11565,7 +11565,7 @@
       </c>
     </row>
     <row r="534">
-      <c r="A534" s="2" t="n">
+      <c r="A534" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B534" t="inlineStr">
@@ -11586,7 +11586,7 @@
       </c>
     </row>
     <row r="535">
-      <c r="A535" s="2" t="n">
+      <c r="A535" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B535" t="inlineStr">
@@ -11607,7 +11607,7 @@
       </c>
     </row>
     <row r="536">
-      <c r="A536" s="2" t="n">
+      <c r="A536" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B536" t="inlineStr">
@@ -11628,7 +11628,7 @@
       </c>
     </row>
     <row r="537">
-      <c r="A537" s="2" t="n">
+      <c r="A537" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B537" t="inlineStr">
@@ -11649,7 +11649,7 @@
       </c>
     </row>
     <row r="538">
-      <c r="A538" s="2" t="n">
+      <c r="A538" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B538" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
     </row>
     <row r="539">
-      <c r="A539" s="2" t="n">
+      <c r="A539" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B539" t="inlineStr">
@@ -11691,7 +11691,7 @@
       </c>
     </row>
     <row r="540">
-      <c r="A540" s="2" t="n">
+      <c r="A540" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B540" t="inlineStr">
@@ -11712,7 +11712,7 @@
       </c>
     </row>
     <row r="541">
-      <c r="A541" s="2" t="n">
+      <c r="A541" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B541" t="inlineStr">
@@ -11733,7 +11733,7 @@
       </c>
     </row>
     <row r="542">
-      <c r="A542" s="2" t="n">
+      <c r="A542" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B542" t="inlineStr">
@@ -11754,7 +11754,7 @@
       </c>
     </row>
     <row r="543">
-      <c r="A543" s="2" t="n">
+      <c r="A543" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B543" t="inlineStr">
@@ -11775,7 +11775,7 @@
       </c>
     </row>
     <row r="544">
-      <c r="A544" s="2" t="n">
+      <c r="A544" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B544" t="inlineStr">
@@ -11796,7 +11796,7 @@
       </c>
     </row>
     <row r="545">
-      <c r="A545" s="2" t="n">
+      <c r="A545" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B545" t="inlineStr">
@@ -11817,7 +11817,7 @@
       </c>
     </row>
     <row r="546">
-      <c r="A546" s="2" t="n">
+      <c r="A546" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B546" t="inlineStr">
@@ -11838,7 +11838,7 @@
       </c>
     </row>
     <row r="547">
-      <c r="A547" s="2" t="n">
+      <c r="A547" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B547" t="inlineStr">
@@ -11859,7 +11859,7 @@
       </c>
     </row>
     <row r="548">
-      <c r="A548" s="2" t="n">
+      <c r="A548" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B548" t="inlineStr">
@@ -11880,7 +11880,7 @@
       </c>
     </row>
     <row r="549">
-      <c r="A549" s="2" t="n">
+      <c r="A549" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B549" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
     </row>
     <row r="550">
-      <c r="A550" s="2" t="n">
+      <c r="A550" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B550" t="inlineStr">
@@ -11922,7 +11922,7 @@
       </c>
     </row>
     <row r="551">
-      <c r="A551" s="2" t="n">
+      <c r="A551" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B551" t="inlineStr">
@@ -11943,7 +11943,7 @@
       </c>
     </row>
     <row r="552">
-      <c r="A552" s="2" t="n">
+      <c r="A552" s="1" t="n">
         <v>46279</v>
       </c>
       <c r="B552" t="inlineStr">
@@ -11958,6 +11958,615 @@
         <v>48</v>
       </c>
       <c r="E552" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C553" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="D553" t="n">
+        <v>28</v>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C554" t="n">
+        <v>13.03999996185303</v>
+      </c>
+      <c r="D554" t="n">
+        <v>31</v>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C555" t="n">
+        <v>22.09000015258789</v>
+      </c>
+      <c r="D555" t="n">
+        <v>30</v>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C556" t="n">
+        <v>4.019999980926514</v>
+      </c>
+      <c r="D556" t="n">
+        <v>16</v>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C557" t="n">
+        <v>0.7599999904632568</v>
+      </c>
+      <c r="D557" t="n">
+        <v>12</v>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C558" t="n">
+        <v>183.8800048828125</v>
+      </c>
+      <c r="D558" t="n">
+        <v>26</v>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C559" t="n">
+        <v>60.43999862670898</v>
+      </c>
+      <c r="D559" t="n">
+        <v>45</v>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C560" t="n">
+        <v>5.309999942779541</v>
+      </c>
+      <c r="D560" t="n">
+        <v>61</v>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C561" t="n">
+        <v>6.21999979019165</v>
+      </c>
+      <c r="D561" t="n">
+        <v>10</v>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C562" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="D562" t="n">
+        <v>22</v>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C563" t="n">
+        <v>20.22999954223633</v>
+      </c>
+      <c r="D563" t="n">
+        <v>49</v>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C564" t="n">
+        <v>26.96999931335449</v>
+      </c>
+      <c r="D564" t="n">
+        <v>20</v>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C565" t="n">
+        <v>13.14999961853027</v>
+      </c>
+      <c r="D565" t="n">
+        <v>9</v>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C566" t="n">
+        <v>4.889999866485596</v>
+      </c>
+      <c r="D566" t="n">
+        <v>26</v>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C567" t="n">
+        <v>23.45000076293945</v>
+      </c>
+      <c r="D567" t="n">
+        <v>27</v>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C568" t="n">
+        <v>11.52999973297119</v>
+      </c>
+      <c r="D568" t="n">
+        <v>22</v>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C569" t="n">
+        <v>5.539999961853027</v>
+      </c>
+      <c r="D569" t="n">
+        <v>20</v>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C570" t="n">
+        <v>7.900000095367432</v>
+      </c>
+      <c r="D570" t="n">
+        <v>25</v>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C571" t="n">
+        <v>5.670000076293945</v>
+      </c>
+      <c r="D571" t="n">
+        <v>30</v>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C572" t="n">
+        <v>50.43000030517578</v>
+      </c>
+      <c r="D572" t="n">
+        <v>23</v>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C573" t="n">
+        <v>4.440000057220459</v>
+      </c>
+      <c r="D573" t="n">
+        <v>20</v>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C574" t="n">
+        <v>65.48999786376953</v>
+      </c>
+      <c r="D574" t="n">
+        <v>8</v>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C575" t="n">
+        <v>50.45999908447266</v>
+      </c>
+      <c r="D575" t="n">
+        <v>16</v>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C576" t="n">
+        <v>19.54000091552734</v>
+      </c>
+      <c r="D576" t="n">
+        <v>63</v>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C577" t="n">
+        <v>37.02000045776367</v>
+      </c>
+      <c r="D577" t="n">
+        <v>35</v>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C578" t="n">
+        <v>109.9400024414062</v>
+      </c>
+      <c r="D578" t="n">
+        <v>31</v>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C579" t="n">
+        <v>47.54000091552734</v>
+      </c>
+      <c r="D579" t="n">
+        <v>11</v>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C580" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="D580" t="n">
+        <v>11</v>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C581" t="n">
+        <v>38.77000045776367</v>
+      </c>
+      <c r="D581" t="n">
+        <v>48</v>
+      </c>
+      <c r="E581" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-16
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E581"/>
+  <dimension ref="A1:E610"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11964,7 +11964,7 @@
       </c>
     </row>
     <row r="553">
-      <c r="A553" s="2" t="n">
+      <c r="A553" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B553" t="inlineStr">
@@ -11985,7 +11985,7 @@
       </c>
     </row>
     <row r="554">
-      <c r="A554" s="2" t="n">
+      <c r="A554" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B554" t="inlineStr">
@@ -12006,7 +12006,7 @@
       </c>
     </row>
     <row r="555">
-      <c r="A555" s="2" t="n">
+      <c r="A555" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B555" t="inlineStr">
@@ -12027,7 +12027,7 @@
       </c>
     </row>
     <row r="556">
-      <c r="A556" s="2" t="n">
+      <c r="A556" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B556" t="inlineStr">
@@ -12048,7 +12048,7 @@
       </c>
     </row>
     <row r="557">
-      <c r="A557" s="2" t="n">
+      <c r="A557" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B557" t="inlineStr">
@@ -12069,7 +12069,7 @@
       </c>
     </row>
     <row r="558">
-      <c r="A558" s="2" t="n">
+      <c r="A558" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B558" t="inlineStr">
@@ -12090,7 +12090,7 @@
       </c>
     </row>
     <row r="559">
-      <c r="A559" s="2" t="n">
+      <c r="A559" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B559" t="inlineStr">
@@ -12111,7 +12111,7 @@
       </c>
     </row>
     <row r="560">
-      <c r="A560" s="2" t="n">
+      <c r="A560" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B560" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
     </row>
     <row r="561">
-      <c r="A561" s="2" t="n">
+      <c r="A561" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B561" t="inlineStr">
@@ -12153,7 +12153,7 @@
       </c>
     </row>
     <row r="562">
-      <c r="A562" s="2" t="n">
+      <c r="A562" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B562" t="inlineStr">
@@ -12174,7 +12174,7 @@
       </c>
     </row>
     <row r="563">
-      <c r="A563" s="2" t="n">
+      <c r="A563" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B563" t="inlineStr">
@@ -12195,7 +12195,7 @@
       </c>
     </row>
     <row r="564">
-      <c r="A564" s="2" t="n">
+      <c r="A564" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B564" t="inlineStr">
@@ -12216,7 +12216,7 @@
       </c>
     </row>
     <row r="565">
-      <c r="A565" s="2" t="n">
+      <c r="A565" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B565" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
     </row>
     <row r="566">
-      <c r="A566" s="2" t="n">
+      <c r="A566" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B566" t="inlineStr">
@@ -12258,7 +12258,7 @@
       </c>
     </row>
     <row r="567">
-      <c r="A567" s="2" t="n">
+      <c r="A567" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B567" t="inlineStr">
@@ -12279,7 +12279,7 @@
       </c>
     </row>
     <row r="568">
-      <c r="A568" s="2" t="n">
+      <c r="A568" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B568" t="inlineStr">
@@ -12300,7 +12300,7 @@
       </c>
     </row>
     <row r="569">
-      <c r="A569" s="2" t="n">
+      <c r="A569" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B569" t="inlineStr">
@@ -12321,7 +12321,7 @@
       </c>
     </row>
     <row r="570">
-      <c r="A570" s="2" t="n">
+      <c r="A570" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B570" t="inlineStr">
@@ -12342,7 +12342,7 @@
       </c>
     </row>
     <row r="571">
-      <c r="A571" s="2" t="n">
+      <c r="A571" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B571" t="inlineStr">
@@ -12363,7 +12363,7 @@
       </c>
     </row>
     <row r="572">
-      <c r="A572" s="2" t="n">
+      <c r="A572" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B572" t="inlineStr">
@@ -12384,7 +12384,7 @@
       </c>
     </row>
     <row r="573">
-      <c r="A573" s="2" t="n">
+      <c r="A573" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B573" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
     </row>
     <row r="574">
-      <c r="A574" s="2" t="n">
+      <c r="A574" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B574" t="inlineStr">
@@ -12426,7 +12426,7 @@
       </c>
     </row>
     <row r="575">
-      <c r="A575" s="2" t="n">
+      <c r="A575" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B575" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
     </row>
     <row r="576">
-      <c r="A576" s="2" t="n">
+      <c r="A576" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B576" t="inlineStr">
@@ -12468,7 +12468,7 @@
       </c>
     </row>
     <row r="577">
-      <c r="A577" s="2" t="n">
+      <c r="A577" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B577" t="inlineStr">
@@ -12489,7 +12489,7 @@
       </c>
     </row>
     <row r="578">
-      <c r="A578" s="2" t="n">
+      <c r="A578" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B578" t="inlineStr">
@@ -12510,7 +12510,7 @@
       </c>
     </row>
     <row r="579">
-      <c r="A579" s="2" t="n">
+      <c r="A579" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B579" t="inlineStr">
@@ -12531,7 +12531,7 @@
       </c>
     </row>
     <row r="580">
-      <c r="A580" s="2" t="n">
+      <c r="A580" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B580" t="inlineStr">
@@ -12552,7 +12552,7 @@
       </c>
     </row>
     <row r="581">
-      <c r="A581" s="2" t="n">
+      <c r="A581" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="B581" t="inlineStr">
@@ -12567,6 +12567,615 @@
         <v>48</v>
       </c>
       <c r="E581" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C582" t="n">
+        <v>28.45999908447266</v>
+      </c>
+      <c r="D582" t="n">
+        <v>28</v>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C583" t="n">
+        <v>13.22999954223633</v>
+      </c>
+      <c r="D583" t="n">
+        <v>31</v>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C584" t="n">
+        <v>22.69000053405762</v>
+      </c>
+      <c r="D584" t="n">
+        <v>30</v>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C585" t="n">
+        <v>4.019999980926514</v>
+      </c>
+      <c r="D585" t="n">
+        <v>16</v>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C586" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D586" t="n">
+        <v>12</v>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C587" t="n">
+        <v>183.0299987792969</v>
+      </c>
+      <c r="D587" t="n">
+        <v>26</v>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C588" t="n">
+        <v>60.61999893188477</v>
+      </c>
+      <c r="D588" t="n">
+        <v>45</v>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C589" t="n">
+        <v>4.519999980926514</v>
+      </c>
+      <c r="D589" t="n">
+        <v>61</v>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C590" t="n">
+        <v>6.070000171661377</v>
+      </c>
+      <c r="D590" t="n">
+        <v>10</v>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C591" t="n">
+        <v>6.449999809265137</v>
+      </c>
+      <c r="D591" t="n">
+        <v>22</v>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C592" t="n">
+        <v>20.45000076293945</v>
+      </c>
+      <c r="D592" t="n">
+        <v>49</v>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C593" t="n">
+        <v>27</v>
+      </c>
+      <c r="D593" t="n">
+        <v>20</v>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C594" t="n">
+        <v>13.30000019073486</v>
+      </c>
+      <c r="D594" t="n">
+        <v>9</v>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C595" t="n">
+        <v>4.949999809265137</v>
+      </c>
+      <c r="D595" t="n">
+        <v>26</v>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C596" t="n">
+        <v>23.52000045776367</v>
+      </c>
+      <c r="D596" t="n">
+        <v>27</v>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C597" t="n">
+        <v>11.80000019073486</v>
+      </c>
+      <c r="D597" t="n">
+        <v>22</v>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C598" t="n">
+        <v>5.920000076293945</v>
+      </c>
+      <c r="D598" t="n">
+        <v>20</v>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C599" t="n">
+        <v>7.949999809265137</v>
+      </c>
+      <c r="D599" t="n">
+        <v>25</v>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C600" t="n">
+        <v>5.71999979019165</v>
+      </c>
+      <c r="D600" t="n">
+        <v>30</v>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C601" t="n">
+        <v>48.70999908447266</v>
+      </c>
+      <c r="D601" t="n">
+        <v>23</v>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C602" t="n">
+        <v>4.53000020980835</v>
+      </c>
+      <c r="D602" t="n">
+        <v>20</v>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C603" t="n">
+        <v>62.83000183105469</v>
+      </c>
+      <c r="D603" t="n">
+        <v>8</v>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C604" t="n">
+        <v>49.9900016784668</v>
+      </c>
+      <c r="D604" t="n">
+        <v>16</v>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C605" t="n">
+        <v>20.11000061035156</v>
+      </c>
+      <c r="D605" t="n">
+        <v>63</v>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C606" t="n">
+        <v>37.13000106811523</v>
+      </c>
+      <c r="D606" t="n">
+        <v>35</v>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C607" t="n">
+        <v>110.25</v>
+      </c>
+      <c r="D607" t="n">
+        <v>31</v>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C608" t="n">
+        <v>46.7400016784668</v>
+      </c>
+      <c r="D608" t="n">
+        <v>11</v>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C609" t="n">
+        <v>7.010000228881836</v>
+      </c>
+      <c r="D609" t="n">
+        <v>11</v>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C610" t="n">
+        <v>39.04999923706055</v>
+      </c>
+      <c r="D610" t="n">
+        <v>48</v>
+      </c>
+      <c r="E610" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-17
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E610"/>
+  <dimension ref="A1:E639"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12573,7 +12573,7 @@
       </c>
     </row>
     <row r="582">
-      <c r="A582" s="2" t="n">
+      <c r="A582" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B582" t="inlineStr">
@@ -12594,7 +12594,7 @@
       </c>
     </row>
     <row r="583">
-      <c r="A583" s="2" t="n">
+      <c r="A583" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B583" t="inlineStr">
@@ -12615,7 +12615,7 @@
       </c>
     </row>
     <row r="584">
-      <c r="A584" s="2" t="n">
+      <c r="A584" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B584" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
     </row>
     <row r="585">
-      <c r="A585" s="2" t="n">
+      <c r="A585" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B585" t="inlineStr">
@@ -12657,7 +12657,7 @@
       </c>
     </row>
     <row r="586">
-      <c r="A586" s="2" t="n">
+      <c r="A586" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B586" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
     </row>
     <row r="587">
-      <c r="A587" s="2" t="n">
+      <c r="A587" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B587" t="inlineStr">
@@ -12699,7 +12699,7 @@
       </c>
     </row>
     <row r="588">
-      <c r="A588" s="2" t="n">
+      <c r="A588" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B588" t="inlineStr">
@@ -12720,7 +12720,7 @@
       </c>
     </row>
     <row r="589">
-      <c r="A589" s="2" t="n">
+      <c r="A589" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B589" t="inlineStr">
@@ -12741,7 +12741,7 @@
       </c>
     </row>
     <row r="590">
-      <c r="A590" s="2" t="n">
+      <c r="A590" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B590" t="inlineStr">
@@ -12762,7 +12762,7 @@
       </c>
     </row>
     <row r="591">
-      <c r="A591" s="2" t="n">
+      <c r="A591" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B591" t="inlineStr">
@@ -12783,7 +12783,7 @@
       </c>
     </row>
     <row r="592">
-      <c r="A592" s="2" t="n">
+      <c r="A592" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B592" t="inlineStr">
@@ -12804,7 +12804,7 @@
       </c>
     </row>
     <row r="593">
-      <c r="A593" s="2" t="n">
+      <c r="A593" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B593" t="inlineStr">
@@ -12825,7 +12825,7 @@
       </c>
     </row>
     <row r="594">
-      <c r="A594" s="2" t="n">
+      <c r="A594" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B594" t="inlineStr">
@@ -12846,7 +12846,7 @@
       </c>
     </row>
     <row r="595">
-      <c r="A595" s="2" t="n">
+      <c r="A595" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B595" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
     </row>
     <row r="596">
-      <c r="A596" s="2" t="n">
+      <c r="A596" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B596" t="inlineStr">
@@ -12888,7 +12888,7 @@
       </c>
     </row>
     <row r="597">
-      <c r="A597" s="2" t="n">
+      <c r="A597" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B597" t="inlineStr">
@@ -12909,7 +12909,7 @@
       </c>
     </row>
     <row r="598">
-      <c r="A598" s="2" t="n">
+      <c r="A598" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B598" t="inlineStr">
@@ -12930,7 +12930,7 @@
       </c>
     </row>
     <row r="599">
-      <c r="A599" s="2" t="n">
+      <c r="A599" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B599" t="inlineStr">
@@ -12951,7 +12951,7 @@
       </c>
     </row>
     <row r="600">
-      <c r="A600" s="2" t="n">
+      <c r="A600" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B600" t="inlineStr">
@@ -12972,7 +12972,7 @@
       </c>
     </row>
     <row r="601">
-      <c r="A601" s="2" t="n">
+      <c r="A601" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B601" t="inlineStr">
@@ -12993,7 +12993,7 @@
       </c>
     </row>
     <row r="602">
-      <c r="A602" s="2" t="n">
+      <c r="A602" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B602" t="inlineStr">
@@ -13014,7 +13014,7 @@
       </c>
     </row>
     <row r="603">
-      <c r="A603" s="2" t="n">
+      <c r="A603" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B603" t="inlineStr">
@@ -13035,7 +13035,7 @@
       </c>
     </row>
     <row r="604">
-      <c r="A604" s="2" t="n">
+      <c r="A604" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B604" t="inlineStr">
@@ -13056,7 +13056,7 @@
       </c>
     </row>
     <row r="605">
-      <c r="A605" s="2" t="n">
+      <c r="A605" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B605" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
     </row>
     <row r="606">
-      <c r="A606" s="2" t="n">
+      <c r="A606" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B606" t="inlineStr">
@@ -13098,7 +13098,7 @@
       </c>
     </row>
     <row r="607">
-      <c r="A607" s="2" t="n">
+      <c r="A607" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B607" t="inlineStr">
@@ -13119,7 +13119,7 @@
       </c>
     </row>
     <row r="608">
-      <c r="A608" s="2" t="n">
+      <c r="A608" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B608" t="inlineStr">
@@ -13140,7 +13140,7 @@
       </c>
     </row>
     <row r="609">
-      <c r="A609" s="2" t="n">
+      <c r="A609" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B609" t="inlineStr">
@@ -13161,7 +13161,7 @@
       </c>
     </row>
     <row r="610">
-      <c r="A610" s="2" t="n">
+      <c r="A610" s="1" t="n">
         <v>46281</v>
       </c>
       <c r="B610" t="inlineStr">
@@ -13176,6 +13176,615 @@
         <v>48</v>
       </c>
       <c r="E610" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C611" t="n">
+        <v>28.29999923706055</v>
+      </c>
+      <c r="D611" t="n">
+        <v>28</v>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C612" t="n">
+        <v>12.86999988555908</v>
+      </c>
+      <c r="D612" t="n">
+        <v>31</v>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C613" t="n">
+        <v>22.77000045776367</v>
+      </c>
+      <c r="D613" t="n">
+        <v>30</v>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C614" t="n">
+        <v>3.819999933242798</v>
+      </c>
+      <c r="D614" t="n">
+        <v>16</v>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C615" t="n">
+        <v>0.8199999928474426</v>
+      </c>
+      <c r="D615" t="n">
+        <v>12</v>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C616" t="n">
+        <v>183.3300018310547</v>
+      </c>
+      <c r="D616" t="n">
+        <v>26</v>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C617" t="n">
+        <v>61.11000061035156</v>
+      </c>
+      <c r="D617" t="n">
+        <v>45</v>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C618" t="n">
+        <v>4.519999980926514</v>
+      </c>
+      <c r="D618" t="n">
+        <v>61</v>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C619" t="n">
+        <v>5.710000038146973</v>
+      </c>
+      <c r="D619" t="n">
+        <v>10</v>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C620" t="n">
+        <v>6.210000038146973</v>
+      </c>
+      <c r="D620" t="n">
+        <v>22</v>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C621" t="n">
+        <v>20.53000068664551</v>
+      </c>
+      <c r="D621" t="n">
+        <v>49</v>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C622" t="n">
+        <v>27.34000015258789</v>
+      </c>
+      <c r="D622" t="n">
+        <v>20</v>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C623" t="n">
+        <v>13</v>
+      </c>
+      <c r="D623" t="n">
+        <v>9</v>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C624" t="n">
+        <v>4.929999828338623</v>
+      </c>
+      <c r="D624" t="n">
+        <v>26</v>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C625" t="n">
+        <v>23.54000091552734</v>
+      </c>
+      <c r="D625" t="n">
+        <v>27</v>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C626" t="n">
+        <v>11.38000011444092</v>
+      </c>
+      <c r="D626" t="n">
+        <v>22</v>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C627" t="n">
+        <v>5.769999980926514</v>
+      </c>
+      <c r="D627" t="n">
+        <v>20</v>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C628" t="n">
+        <v>8.010000228881836</v>
+      </c>
+      <c r="D628" t="n">
+        <v>25</v>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C629" t="n">
+        <v>5.409999847412109</v>
+      </c>
+      <c r="D629" t="n">
+        <v>30</v>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C630" t="n">
+        <v>48.75</v>
+      </c>
+      <c r="D630" t="n">
+        <v>23</v>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C631" t="n">
+        <v>4.320000171661377</v>
+      </c>
+      <c r="D631" t="n">
+        <v>20</v>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C632" t="n">
+        <v>63.47999954223633</v>
+      </c>
+      <c r="D632" t="n">
+        <v>8</v>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C633" t="n">
+        <v>49.47000122070312</v>
+      </c>
+      <c r="D633" t="n">
+        <v>16</v>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C634" t="n">
+        <v>20.29999923706055</v>
+      </c>
+      <c r="D634" t="n">
+        <v>63</v>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C635" t="n">
+        <v>37.06000137329102</v>
+      </c>
+      <c r="D635" t="n">
+        <v>35</v>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C636" t="n">
+        <v>109.7900009155273</v>
+      </c>
+      <c r="D636" t="n">
+        <v>31</v>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C637" t="n">
+        <v>47.59000015258789</v>
+      </c>
+      <c r="D637" t="n">
+        <v>11</v>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C638" t="n">
+        <v>7.059999942779541</v>
+      </c>
+      <c r="D638" t="n">
+        <v>11</v>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C639" t="n">
+        <v>39.34999847412109</v>
+      </c>
+      <c r="D639" t="n">
+        <v>48</v>
+      </c>
+      <c r="E639" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-18
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E639"/>
+  <dimension ref="A1:E668"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13182,7 +13182,7 @@
       </c>
     </row>
     <row r="611">
-      <c r="A611" s="2" t="n">
+      <c r="A611" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B611" t="inlineStr">
@@ -13203,7 +13203,7 @@
       </c>
     </row>
     <row r="612">
-      <c r="A612" s="2" t="n">
+      <c r="A612" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B612" t="inlineStr">
@@ -13224,7 +13224,7 @@
       </c>
     </row>
     <row r="613">
-      <c r="A613" s="2" t="n">
+      <c r="A613" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B613" t="inlineStr">
@@ -13245,7 +13245,7 @@
       </c>
     </row>
     <row r="614">
-      <c r="A614" s="2" t="n">
+      <c r="A614" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B614" t="inlineStr">
@@ -13266,7 +13266,7 @@
       </c>
     </row>
     <row r="615">
-      <c r="A615" s="2" t="n">
+      <c r="A615" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B615" t="inlineStr">
@@ -13287,7 +13287,7 @@
       </c>
     </row>
     <row r="616">
-      <c r="A616" s="2" t="n">
+      <c r="A616" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B616" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
     </row>
     <row r="617">
-      <c r="A617" s="2" t="n">
+      <c r="A617" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B617" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
     </row>
     <row r="618">
-      <c r="A618" s="2" t="n">
+      <c r="A618" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B618" t="inlineStr">
@@ -13350,7 +13350,7 @@
       </c>
     </row>
     <row r="619">
-      <c r="A619" s="2" t="n">
+      <c r="A619" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B619" t="inlineStr">
@@ -13371,7 +13371,7 @@
       </c>
     </row>
     <row r="620">
-      <c r="A620" s="2" t="n">
+      <c r="A620" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B620" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
     </row>
     <row r="621">
-      <c r="A621" s="2" t="n">
+      <c r="A621" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B621" t="inlineStr">
@@ -13413,7 +13413,7 @@
       </c>
     </row>
     <row r="622">
-      <c r="A622" s="2" t="n">
+      <c r="A622" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B622" t="inlineStr">
@@ -13434,7 +13434,7 @@
       </c>
     </row>
     <row r="623">
-      <c r="A623" s="2" t="n">
+      <c r="A623" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B623" t="inlineStr">
@@ -13455,7 +13455,7 @@
       </c>
     </row>
     <row r="624">
-      <c r="A624" s="2" t="n">
+      <c r="A624" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B624" t="inlineStr">
@@ -13476,7 +13476,7 @@
       </c>
     </row>
     <row r="625">
-      <c r="A625" s="2" t="n">
+      <c r="A625" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B625" t="inlineStr">
@@ -13497,7 +13497,7 @@
       </c>
     </row>
     <row r="626">
-      <c r="A626" s="2" t="n">
+      <c r="A626" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B626" t="inlineStr">
@@ -13518,7 +13518,7 @@
       </c>
     </row>
     <row r="627">
-      <c r="A627" s="2" t="n">
+      <c r="A627" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B627" t="inlineStr">
@@ -13539,7 +13539,7 @@
       </c>
     </row>
     <row r="628">
-      <c r="A628" s="2" t="n">
+      <c r="A628" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B628" t="inlineStr">
@@ -13560,7 +13560,7 @@
       </c>
     </row>
     <row r="629">
-      <c r="A629" s="2" t="n">
+      <c r="A629" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B629" t="inlineStr">
@@ -13581,7 +13581,7 @@
       </c>
     </row>
     <row r="630">
-      <c r="A630" s="2" t="n">
+      <c r="A630" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B630" t="inlineStr">
@@ -13602,7 +13602,7 @@
       </c>
     </row>
     <row r="631">
-      <c r="A631" s="2" t="n">
+      <c r="A631" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B631" t="inlineStr">
@@ -13623,7 +13623,7 @@
       </c>
     </row>
     <row r="632">
-      <c r="A632" s="2" t="n">
+      <c r="A632" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B632" t="inlineStr">
@@ -13644,7 +13644,7 @@
       </c>
     </row>
     <row r="633">
-      <c r="A633" s="2" t="n">
+      <c r="A633" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B633" t="inlineStr">
@@ -13665,7 +13665,7 @@
       </c>
     </row>
     <row r="634">
-      <c r="A634" s="2" t="n">
+      <c r="A634" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B634" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
     </row>
     <row r="635">
-      <c r="A635" s="2" t="n">
+      <c r="A635" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B635" t="inlineStr">
@@ -13707,7 +13707,7 @@
       </c>
     </row>
     <row r="636">
-      <c r="A636" s="2" t="n">
+      <c r="A636" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B636" t="inlineStr">
@@ -13728,7 +13728,7 @@
       </c>
     </row>
     <row r="637">
-      <c r="A637" s="2" t="n">
+      <c r="A637" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B637" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
     </row>
     <row r="638">
-      <c r="A638" s="2" t="n">
+      <c r="A638" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B638" t="inlineStr">
@@ -13770,7 +13770,7 @@
       </c>
     </row>
     <row r="639">
-      <c r="A639" s="2" t="n">
+      <c r="A639" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="B639" t="inlineStr">
@@ -13785,6 +13785,615 @@
         <v>48</v>
       </c>
       <c r="E639" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C640" t="n">
+        <v>28.71999931335449</v>
+      </c>
+      <c r="D640" t="n">
+        <v>28</v>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C641" t="n">
+        <v>12.98999977111816</v>
+      </c>
+      <c r="D641" t="n">
+        <v>31</v>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C642" t="n">
+        <v>23.04999923706055</v>
+      </c>
+      <c r="D642" t="n">
+        <v>30</v>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C643" t="n">
+        <v>3.970000028610229</v>
+      </c>
+      <c r="D643" t="n">
+        <v>16</v>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C644" t="n">
+        <v>0.8299999833106995</v>
+      </c>
+      <c r="D644" t="n">
+        <v>12</v>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C645" t="n">
+        <v>182.3699951171875</v>
+      </c>
+      <c r="D645" t="n">
+        <v>26</v>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C646" t="n">
+        <v>61.38999938964844</v>
+      </c>
+      <c r="D646" t="n">
+        <v>45</v>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C647" t="n">
+        <v>4.409999847412109</v>
+      </c>
+      <c r="D647" t="n">
+        <v>61</v>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C648" t="n">
+        <v>5.510000228881836</v>
+      </c>
+      <c r="D648" t="n">
+        <v>10</v>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C649" t="n">
+        <v>5.78000020980835</v>
+      </c>
+      <c r="D649" t="n">
+        <v>22</v>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C650" t="n">
+        <v>20.6299991607666</v>
+      </c>
+      <c r="D650" t="n">
+        <v>49</v>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C651" t="n">
+        <v>27.13999938964844</v>
+      </c>
+      <c r="D651" t="n">
+        <v>20</v>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C652" t="n">
+        <v>13.42000007629395</v>
+      </c>
+      <c r="D652" t="n">
+        <v>9</v>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C653" t="n">
+        <v>4.869999885559082</v>
+      </c>
+      <c r="D653" t="n">
+        <v>26</v>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C654" t="n">
+        <v>23.77000045776367</v>
+      </c>
+      <c r="D654" t="n">
+        <v>27</v>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C655" t="n">
+        <v>11.44999980926514</v>
+      </c>
+      <c r="D655" t="n">
+        <v>22</v>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C656" t="n">
+        <v>5.869999885559082</v>
+      </c>
+      <c r="D656" t="n">
+        <v>20</v>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C657" t="n">
+        <v>7.949999809265137</v>
+      </c>
+      <c r="D657" t="n">
+        <v>25</v>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C658" t="n">
+        <v>5.239999771118164</v>
+      </c>
+      <c r="D658" t="n">
+        <v>30</v>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C659" t="n">
+        <v>48.45000076293945</v>
+      </c>
+      <c r="D659" t="n">
+        <v>23</v>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C660" t="n">
+        <v>4.289999961853027</v>
+      </c>
+      <c r="D660" t="n">
+        <v>20</v>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C661" t="n">
+        <v>63.31999969482422</v>
+      </c>
+      <c r="D661" t="n">
+        <v>8</v>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C662" t="n">
+        <v>49</v>
+      </c>
+      <c r="D662" t="n">
+        <v>16</v>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C663" t="n">
+        <v>20.26000022888184</v>
+      </c>
+      <c r="D663" t="n">
+        <v>63</v>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C664" t="n">
+        <v>37.25</v>
+      </c>
+      <c r="D664" t="n">
+        <v>35</v>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C665" t="n">
+        <v>109.4800033569336</v>
+      </c>
+      <c r="D665" t="n">
+        <v>31</v>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C666" t="n">
+        <v>47.7599983215332</v>
+      </c>
+      <c r="D666" t="n">
+        <v>11</v>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C667" t="n">
+        <v>6.900000095367432</v>
+      </c>
+      <c r="D667" t="n">
+        <v>11</v>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C668" t="n">
+        <v>39.83000183105469</v>
+      </c>
+      <c r="D668" t="n">
+        <v>48</v>
+      </c>
+      <c r="E668" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-21
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E668"/>
+  <dimension ref="A1:E697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13791,7 +13791,7 @@
       </c>
     </row>
     <row r="640">
-      <c r="A640" s="2" t="n">
+      <c r="A640" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B640" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
     </row>
     <row r="641">
-      <c r="A641" s="2" t="n">
+      <c r="A641" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B641" t="inlineStr">
@@ -13833,7 +13833,7 @@
       </c>
     </row>
     <row r="642">
-      <c r="A642" s="2" t="n">
+      <c r="A642" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B642" t="inlineStr">
@@ -13854,7 +13854,7 @@
       </c>
     </row>
     <row r="643">
-      <c r="A643" s="2" t="n">
+      <c r="A643" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B643" t="inlineStr">
@@ -13875,7 +13875,7 @@
       </c>
     </row>
     <row r="644">
-      <c r="A644" s="2" t="n">
+      <c r="A644" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B644" t="inlineStr">
@@ -13896,7 +13896,7 @@
       </c>
     </row>
     <row r="645">
-      <c r="A645" s="2" t="n">
+      <c r="A645" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B645" t="inlineStr">
@@ -13917,7 +13917,7 @@
       </c>
     </row>
     <row r="646">
-      <c r="A646" s="2" t="n">
+      <c r="A646" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B646" t="inlineStr">
@@ -13938,7 +13938,7 @@
       </c>
     </row>
     <row r="647">
-      <c r="A647" s="2" t="n">
+      <c r="A647" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B647" t="inlineStr">
@@ -13959,7 +13959,7 @@
       </c>
     </row>
     <row r="648">
-      <c r="A648" s="2" t="n">
+      <c r="A648" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B648" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
     </row>
     <row r="649">
-      <c r="A649" s="2" t="n">
+      <c r="A649" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B649" t="inlineStr">
@@ -14001,7 +14001,7 @@
       </c>
     </row>
     <row r="650">
-      <c r="A650" s="2" t="n">
+      <c r="A650" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B650" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
     </row>
     <row r="651">
-      <c r="A651" s="2" t="n">
+      <c r="A651" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B651" t="inlineStr">
@@ -14043,7 +14043,7 @@
       </c>
     </row>
     <row r="652">
-      <c r="A652" s="2" t="n">
+      <c r="A652" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B652" t="inlineStr">
@@ -14064,7 +14064,7 @@
       </c>
     </row>
     <row r="653">
-      <c r="A653" s="2" t="n">
+      <c r="A653" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B653" t="inlineStr">
@@ -14085,7 +14085,7 @@
       </c>
     </row>
     <row r="654">
-      <c r="A654" s="2" t="n">
+      <c r="A654" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B654" t="inlineStr">
@@ -14106,7 +14106,7 @@
       </c>
     </row>
     <row r="655">
-      <c r="A655" s="2" t="n">
+      <c r="A655" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B655" t="inlineStr">
@@ -14127,7 +14127,7 @@
       </c>
     </row>
     <row r="656">
-      <c r="A656" s="2" t="n">
+      <c r="A656" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B656" t="inlineStr">
@@ -14148,7 +14148,7 @@
       </c>
     </row>
     <row r="657">
-      <c r="A657" s="2" t="n">
+      <c r="A657" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B657" t="inlineStr">
@@ -14169,7 +14169,7 @@
       </c>
     </row>
     <row r="658">
-      <c r="A658" s="2" t="n">
+      <c r="A658" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B658" t="inlineStr">
@@ -14190,7 +14190,7 @@
       </c>
     </row>
     <row r="659">
-      <c r="A659" s="2" t="n">
+      <c r="A659" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B659" t="inlineStr">
@@ -14211,7 +14211,7 @@
       </c>
     </row>
     <row r="660">
-      <c r="A660" s="2" t="n">
+      <c r="A660" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B660" t="inlineStr">
@@ -14232,7 +14232,7 @@
       </c>
     </row>
     <row r="661">
-      <c r="A661" s="2" t="n">
+      <c r="A661" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B661" t="inlineStr">
@@ -14253,7 +14253,7 @@
       </c>
     </row>
     <row r="662">
-      <c r="A662" s="2" t="n">
+      <c r="A662" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B662" t="inlineStr">
@@ -14274,7 +14274,7 @@
       </c>
     </row>
     <row r="663">
-      <c r="A663" s="2" t="n">
+      <c r="A663" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B663" t="inlineStr">
@@ -14295,7 +14295,7 @@
       </c>
     </row>
     <row r="664">
-      <c r="A664" s="2" t="n">
+      <c r="A664" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B664" t="inlineStr">
@@ -14316,7 +14316,7 @@
       </c>
     </row>
     <row r="665">
-      <c r="A665" s="2" t="n">
+      <c r="A665" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B665" t="inlineStr">
@@ -14337,7 +14337,7 @@
       </c>
     </row>
     <row r="666">
-      <c r="A666" s="2" t="n">
+      <c r="A666" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B666" t="inlineStr">
@@ -14358,7 +14358,7 @@
       </c>
     </row>
     <row r="667">
-      <c r="A667" s="2" t="n">
+      <c r="A667" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B667" t="inlineStr">
@@ -14379,7 +14379,7 @@
       </c>
     </row>
     <row r="668">
-      <c r="A668" s="2" t="n">
+      <c r="A668" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="B668" t="inlineStr">
@@ -14394,6 +14394,615 @@
         <v>48</v>
       </c>
       <c r="E668" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C669" t="n">
+        <v>29.81999969482422</v>
+      </c>
+      <c r="D669" t="n">
+        <v>28</v>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C670" t="n">
+        <v>13.13000011444092</v>
+      </c>
+      <c r="D670" t="n">
+        <v>31</v>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C671" t="n">
+        <v>23.11000061035156</v>
+      </c>
+      <c r="D671" t="n">
+        <v>30</v>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C672" t="n">
+        <v>3.900000095367432</v>
+      </c>
+      <c r="D672" t="n">
+        <v>16</v>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C673" t="n">
+        <v>0.8999999761581421</v>
+      </c>
+      <c r="D673" t="n">
+        <v>12</v>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C674" t="n">
+        <v>184.1999969482422</v>
+      </c>
+      <c r="D674" t="n">
+        <v>26</v>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C675" t="n">
+        <v>63.56999969482422</v>
+      </c>
+      <c r="D675" t="n">
+        <v>45</v>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C676" t="n">
+        <v>4.429999828338623</v>
+      </c>
+      <c r="D676" t="n">
+        <v>61</v>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C677" t="n">
+        <v>5.400000095367432</v>
+      </c>
+      <c r="D677" t="n">
+        <v>10</v>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C678" t="n">
+        <v>6.170000076293945</v>
+      </c>
+      <c r="D678" t="n">
+        <v>22</v>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C679" t="n">
+        <v>20.6200008392334</v>
+      </c>
+      <c r="D679" t="n">
+        <v>49</v>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C680" t="n">
+        <v>28.03000068664551</v>
+      </c>
+      <c r="D680" t="n">
+        <v>20</v>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C681" t="n">
+        <v>13.88000011444092</v>
+      </c>
+      <c r="D681" t="n">
+        <v>9</v>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C682" t="n">
+        <v>4.909999847412109</v>
+      </c>
+      <c r="D682" t="n">
+        <v>26</v>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C683" t="n">
+        <v>23.97999954223633</v>
+      </c>
+      <c r="D683" t="n">
+        <v>27</v>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C684" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="D684" t="n">
+        <v>22</v>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C685" t="n">
+        <v>5.96999979019165</v>
+      </c>
+      <c r="D685" t="n">
+        <v>20</v>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C686" t="n">
+        <v>8.479999542236328</v>
+      </c>
+      <c r="D686" t="n">
+        <v>25</v>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C687" t="n">
+        <v>5.28000020980835</v>
+      </c>
+      <c r="D687" t="n">
+        <v>30</v>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C688" t="n">
+        <v>48.0099983215332</v>
+      </c>
+      <c r="D688" t="n">
+        <v>23</v>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C689" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="D689" t="n">
+        <v>20</v>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C690" t="n">
+        <v>60.79999923706055</v>
+      </c>
+      <c r="D690" t="n">
+        <v>8</v>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C691" t="n">
+        <v>49.41999816894531</v>
+      </c>
+      <c r="D691" t="n">
+        <v>16</v>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C692" t="n">
+        <v>20.71999931335449</v>
+      </c>
+      <c r="D692" t="n">
+        <v>63</v>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C693" t="n">
+        <v>38.34000015258789</v>
+      </c>
+      <c r="D693" t="n">
+        <v>35</v>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C694" t="n">
+        <v>111.9700012207031</v>
+      </c>
+      <c r="D694" t="n">
+        <v>31</v>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C695" t="n">
+        <v>47.29000091552734</v>
+      </c>
+      <c r="D695" t="n">
+        <v>11</v>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C696" t="n">
+        <v>6.940000057220459</v>
+      </c>
+      <c r="D696" t="n">
+        <v>11</v>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C697" t="n">
+        <v>39.56000137329102</v>
+      </c>
+      <c r="D697" t="n">
+        <v>48</v>
+      </c>
+      <c r="E697" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-22
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E697"/>
+  <dimension ref="A1:E726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14400,7 +14400,7 @@
       </c>
     </row>
     <row r="669">
-      <c r="A669" s="2" t="n">
+      <c r="A669" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B669" t="inlineStr">
@@ -14421,7 +14421,7 @@
       </c>
     </row>
     <row r="670">
-      <c r="A670" s="2" t="n">
+      <c r="A670" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B670" t="inlineStr">
@@ -14442,7 +14442,7 @@
       </c>
     </row>
     <row r="671">
-      <c r="A671" s="2" t="n">
+      <c r="A671" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B671" t="inlineStr">
@@ -14463,7 +14463,7 @@
       </c>
     </row>
     <row r="672">
-      <c r="A672" s="2" t="n">
+      <c r="A672" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B672" t="inlineStr">
@@ -14484,7 +14484,7 @@
       </c>
     </row>
     <row r="673">
-      <c r="A673" s="2" t="n">
+      <c r="A673" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B673" t="inlineStr">
@@ -14505,7 +14505,7 @@
       </c>
     </row>
     <row r="674">
-      <c r="A674" s="2" t="n">
+      <c r="A674" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B674" t="inlineStr">
@@ -14526,7 +14526,7 @@
       </c>
     </row>
     <row r="675">
-      <c r="A675" s="2" t="n">
+      <c r="A675" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B675" t="inlineStr">
@@ -14547,7 +14547,7 @@
       </c>
     </row>
     <row r="676">
-      <c r="A676" s="2" t="n">
+      <c r="A676" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B676" t="inlineStr">
@@ -14568,7 +14568,7 @@
       </c>
     </row>
     <row r="677">
-      <c r="A677" s="2" t="n">
+      <c r="A677" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B677" t="inlineStr">
@@ -14589,7 +14589,7 @@
       </c>
     </row>
     <row r="678">
-      <c r="A678" s="2" t="n">
+      <c r="A678" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B678" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
     </row>
     <row r="679">
-      <c r="A679" s="2" t="n">
+      <c r="A679" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B679" t="inlineStr">
@@ -14631,7 +14631,7 @@
       </c>
     </row>
     <row r="680">
-      <c r="A680" s="2" t="n">
+      <c r="A680" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B680" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
     </row>
     <row r="681">
-      <c r="A681" s="2" t="n">
+      <c r="A681" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B681" t="inlineStr">
@@ -14673,7 +14673,7 @@
       </c>
     </row>
     <row r="682">
-      <c r="A682" s="2" t="n">
+      <c r="A682" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B682" t="inlineStr">
@@ -14694,7 +14694,7 @@
       </c>
     </row>
     <row r="683">
-      <c r="A683" s="2" t="n">
+      <c r="A683" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B683" t="inlineStr">
@@ -14715,7 +14715,7 @@
       </c>
     </row>
     <row r="684">
-      <c r="A684" s="2" t="n">
+      <c r="A684" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B684" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
     </row>
     <row r="685">
-      <c r="A685" s="2" t="n">
+      <c r="A685" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B685" t="inlineStr">
@@ -14757,7 +14757,7 @@
       </c>
     </row>
     <row r="686">
-      <c r="A686" s="2" t="n">
+      <c r="A686" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B686" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
     </row>
     <row r="687">
-      <c r="A687" s="2" t="n">
+      <c r="A687" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B687" t="inlineStr">
@@ -14799,7 +14799,7 @@
       </c>
     </row>
     <row r="688">
-      <c r="A688" s="2" t="n">
+      <c r="A688" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B688" t="inlineStr">
@@ -14820,7 +14820,7 @@
       </c>
     </row>
     <row r="689">
-      <c r="A689" s="2" t="n">
+      <c r="A689" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B689" t="inlineStr">
@@ -14841,7 +14841,7 @@
       </c>
     </row>
     <row r="690">
-      <c r="A690" s="2" t="n">
+      <c r="A690" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B690" t="inlineStr">
@@ -14862,7 +14862,7 @@
       </c>
     </row>
     <row r="691">
-      <c r="A691" s="2" t="n">
+      <c r="A691" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B691" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
     </row>
     <row r="692">
-      <c r="A692" s="2" t="n">
+      <c r="A692" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B692" t="inlineStr">
@@ -14904,7 +14904,7 @@
       </c>
     </row>
     <row r="693">
-      <c r="A693" s="2" t="n">
+      <c r="A693" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B693" t="inlineStr">
@@ -14925,7 +14925,7 @@
       </c>
     </row>
     <row r="694">
-      <c r="A694" s="2" t="n">
+      <c r="A694" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B694" t="inlineStr">
@@ -14946,7 +14946,7 @@
       </c>
     </row>
     <row r="695">
-      <c r="A695" s="2" t="n">
+      <c r="A695" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B695" t="inlineStr">
@@ -14967,7 +14967,7 @@
       </c>
     </row>
     <row r="696">
-      <c r="A696" s="2" t="n">
+      <c r="A696" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B696" t="inlineStr">
@@ -14988,7 +14988,7 @@
       </c>
     </row>
     <row r="697">
-      <c r="A697" s="2" t="n">
+      <c r="A697" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="B697" t="inlineStr">
@@ -15003,6 +15003,615 @@
         <v>48</v>
       </c>
       <c r="E697" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C698" t="n">
+        <v>29.81999969482422</v>
+      </c>
+      <c r="D698" t="n">
+        <v>28</v>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C699" t="n">
+        <v>13.77999973297119</v>
+      </c>
+      <c r="D699" t="n">
+        <v>31</v>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C700" t="n">
+        <v>22.6200008392334</v>
+      </c>
+      <c r="D700" t="n">
+        <v>30</v>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C701" t="n">
+        <v>3.990000009536743</v>
+      </c>
+      <c r="D701" t="n">
+        <v>16</v>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C702" t="n">
+        <v>0.9700000286102295</v>
+      </c>
+      <c r="D702" t="n">
+        <v>12</v>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C703" t="n">
+        <v>184.5399932861328</v>
+      </c>
+      <c r="D703" t="n">
+        <v>26</v>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C704" t="n">
+        <v>63.93000030517578</v>
+      </c>
+      <c r="D704" t="n">
+        <v>45</v>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C705" t="n">
+        <v>4.300000190734863</v>
+      </c>
+      <c r="D705" t="n">
+        <v>61</v>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C706" t="n">
+        <v>5.300000190734863</v>
+      </c>
+      <c r="D706" t="n">
+        <v>10</v>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C707" t="n">
+        <v>6.300000190734863</v>
+      </c>
+      <c r="D707" t="n">
+        <v>22</v>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C708" t="n">
+        <v>20.42000007629395</v>
+      </c>
+      <c r="D708" t="n">
+        <v>49</v>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C709" t="n">
+        <v>27.71999931335449</v>
+      </c>
+      <c r="D709" t="n">
+        <v>20</v>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C710" t="n">
+        <v>13.81999969482422</v>
+      </c>
+      <c r="D710" t="n">
+        <v>9</v>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C711" t="n">
+        <v>5.019999980926514</v>
+      </c>
+      <c r="D711" t="n">
+        <v>26</v>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C712" t="n">
+        <v>24.89999961853027</v>
+      </c>
+      <c r="D712" t="n">
+        <v>27</v>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C713" t="n">
+        <v>11.86999988555908</v>
+      </c>
+      <c r="D713" t="n">
+        <v>22</v>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C714" t="n">
+        <v>5.900000095367432</v>
+      </c>
+      <c r="D714" t="n">
+        <v>20</v>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C715" t="n">
+        <v>8.460000038146973</v>
+      </c>
+      <c r="D715" t="n">
+        <v>25</v>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C716" t="n">
+        <v>5.309999942779541</v>
+      </c>
+      <c r="D716" t="n">
+        <v>30</v>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C717" t="n">
+        <v>48.36999893188477</v>
+      </c>
+      <c r="D717" t="n">
+        <v>23</v>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C718" t="n">
+        <v>4.190000057220459</v>
+      </c>
+      <c r="D718" t="n">
+        <v>20</v>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C719" t="n">
+        <v>60.38999938964844</v>
+      </c>
+      <c r="D719" t="n">
+        <v>8</v>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C720" t="n">
+        <v>48.38000106811523</v>
+      </c>
+      <c r="D720" t="n">
+        <v>16</v>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C721" t="n">
+        <v>20.17000007629395</v>
+      </c>
+      <c r="D721" t="n">
+        <v>63</v>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C722" t="n">
+        <v>38.33000183105469</v>
+      </c>
+      <c r="D722" t="n">
+        <v>35</v>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C723" t="n">
+        <v>112.2300033569336</v>
+      </c>
+      <c r="D723" t="n">
+        <v>31</v>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C724" t="n">
+        <v>48.65999984741211</v>
+      </c>
+      <c r="D724" t="n">
+        <v>11</v>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C725" t="n">
+        <v>7.099999904632568</v>
+      </c>
+      <c r="D725" t="n">
+        <v>11</v>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C726" t="n">
+        <v>39.61000061035156</v>
+      </c>
+      <c r="D726" t="n">
+        <v>48</v>
+      </c>
+      <c r="E726" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-23
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E726"/>
+  <dimension ref="A1:E755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15009,7 +15009,7 @@
       </c>
     </row>
     <row r="698">
-      <c r="A698" s="2" t="n">
+      <c r="A698" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B698" t="inlineStr">
@@ -15030,7 +15030,7 @@
       </c>
     </row>
     <row r="699">
-      <c r="A699" s="2" t="n">
+      <c r="A699" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B699" t="inlineStr">
@@ -15051,7 +15051,7 @@
       </c>
     </row>
     <row r="700">
-      <c r="A700" s="2" t="n">
+      <c r="A700" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B700" t="inlineStr">
@@ -15072,7 +15072,7 @@
       </c>
     </row>
     <row r="701">
-      <c r="A701" s="2" t="n">
+      <c r="A701" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B701" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
     </row>
     <row r="702">
-      <c r="A702" s="2" t="n">
+      <c r="A702" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B702" t="inlineStr">
@@ -15114,7 +15114,7 @@
       </c>
     </row>
     <row r="703">
-      <c r="A703" s="2" t="n">
+      <c r="A703" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B703" t="inlineStr">
@@ -15135,7 +15135,7 @@
       </c>
     </row>
     <row r="704">
-      <c r="A704" s="2" t="n">
+      <c r="A704" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B704" t="inlineStr">
@@ -15156,7 +15156,7 @@
       </c>
     </row>
     <row r="705">
-      <c r="A705" s="2" t="n">
+      <c r="A705" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B705" t="inlineStr">
@@ -15177,7 +15177,7 @@
       </c>
     </row>
     <row r="706">
-      <c r="A706" s="2" t="n">
+      <c r="A706" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B706" t="inlineStr">
@@ -15198,7 +15198,7 @@
       </c>
     </row>
     <row r="707">
-      <c r="A707" s="2" t="n">
+      <c r="A707" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B707" t="inlineStr">
@@ -15219,7 +15219,7 @@
       </c>
     </row>
     <row r="708">
-      <c r="A708" s="2" t="n">
+      <c r="A708" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B708" t="inlineStr">
@@ -15240,7 +15240,7 @@
       </c>
     </row>
     <row r="709">
-      <c r="A709" s="2" t="n">
+      <c r="A709" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B709" t="inlineStr">
@@ -15261,7 +15261,7 @@
       </c>
     </row>
     <row r="710">
-      <c r="A710" s="2" t="n">
+      <c r="A710" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B710" t="inlineStr">
@@ -15282,7 +15282,7 @@
       </c>
     </row>
     <row r="711">
-      <c r="A711" s="2" t="n">
+      <c r="A711" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B711" t="inlineStr">
@@ -15303,7 +15303,7 @@
       </c>
     </row>
     <row r="712">
-      <c r="A712" s="2" t="n">
+      <c r="A712" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B712" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
     </row>
     <row r="713">
-      <c r="A713" s="2" t="n">
+      <c r="A713" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B713" t="inlineStr">
@@ -15345,7 +15345,7 @@
       </c>
     </row>
     <row r="714">
-      <c r="A714" s="2" t="n">
+      <c r="A714" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B714" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
     </row>
     <row r="715">
-      <c r="A715" s="2" t="n">
+      <c r="A715" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B715" t="inlineStr">
@@ -15387,7 +15387,7 @@
       </c>
     </row>
     <row r="716">
-      <c r="A716" s="2" t="n">
+      <c r="A716" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B716" t="inlineStr">
@@ -15408,7 +15408,7 @@
       </c>
     </row>
     <row r="717">
-      <c r="A717" s="2" t="n">
+      <c r="A717" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B717" t="inlineStr">
@@ -15429,7 +15429,7 @@
       </c>
     </row>
     <row r="718">
-      <c r="A718" s="2" t="n">
+      <c r="A718" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B718" t="inlineStr">
@@ -15450,7 +15450,7 @@
       </c>
     </row>
     <row r="719">
-      <c r="A719" s="2" t="n">
+      <c r="A719" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B719" t="inlineStr">
@@ -15471,7 +15471,7 @@
       </c>
     </row>
     <row r="720">
-      <c r="A720" s="2" t="n">
+      <c r="A720" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B720" t="inlineStr">
@@ -15492,7 +15492,7 @@
       </c>
     </row>
     <row r="721">
-      <c r="A721" s="2" t="n">
+      <c r="A721" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B721" t="inlineStr">
@@ -15513,7 +15513,7 @@
       </c>
     </row>
     <row r="722">
-      <c r="A722" s="2" t="n">
+      <c r="A722" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B722" t="inlineStr">
@@ -15534,7 +15534,7 @@
       </c>
     </row>
     <row r="723">
-      <c r="A723" s="2" t="n">
+      <c r="A723" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B723" t="inlineStr">
@@ -15555,7 +15555,7 @@
       </c>
     </row>
     <row r="724">
-      <c r="A724" s="2" t="n">
+      <c r="A724" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B724" t="inlineStr">
@@ -15576,7 +15576,7 @@
       </c>
     </row>
     <row r="725">
-      <c r="A725" s="2" t="n">
+      <c r="A725" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B725" t="inlineStr">
@@ -15597,7 +15597,7 @@
       </c>
     </row>
     <row r="726">
-      <c r="A726" s="2" t="n">
+      <c r="A726" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="B726" t="inlineStr">
@@ -15612,6 +15612,615 @@
         <v>48</v>
       </c>
       <c r="E726" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C727" t="n">
+        <v>29.34000015258789</v>
+      </c>
+      <c r="D727" t="n">
+        <v>28</v>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C728" t="n">
+        <v>13.22000026702881</v>
+      </c>
+      <c r="D728" t="n">
+        <v>31</v>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C729" t="n">
+        <v>22.21999931335449</v>
+      </c>
+      <c r="D729" t="n">
+        <v>30</v>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C730" t="n">
+        <v>4</v>
+      </c>
+      <c r="D730" t="n">
+        <v>16</v>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C731" t="n">
+        <v>0.9300000071525574</v>
+      </c>
+      <c r="D731" t="n">
+        <v>12</v>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C732" t="n">
+        <v>182.7899932861328</v>
+      </c>
+      <c r="D732" t="n">
+        <v>26</v>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C733" t="n">
+        <v>63.72000122070312</v>
+      </c>
+      <c r="D733" t="n">
+        <v>45</v>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C734" t="n">
+        <v>4</v>
+      </c>
+      <c r="D734" t="n">
+        <v>61</v>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C735" t="n">
+        <v>5.139999866485596</v>
+      </c>
+      <c r="D735" t="n">
+        <v>10</v>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C736" t="n">
+        <v>6.059999942779541</v>
+      </c>
+      <c r="D736" t="n">
+        <v>22</v>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C737" t="n">
+        <v>20.04000091552734</v>
+      </c>
+      <c r="D737" t="n">
+        <v>49</v>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C738" t="n">
+        <v>27.77000045776367</v>
+      </c>
+      <c r="D738" t="n">
+        <v>20</v>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C739" t="n">
+        <v>13.8100004196167</v>
+      </c>
+      <c r="D739" t="n">
+        <v>9</v>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C740" t="n">
+        <v>4.929999828338623</v>
+      </c>
+      <c r="D740" t="n">
+        <v>26</v>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C741" t="n">
+        <v>24.48999977111816</v>
+      </c>
+      <c r="D741" t="n">
+        <v>27</v>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C742" t="n">
+        <v>11.81999969482422</v>
+      </c>
+      <c r="D742" t="n">
+        <v>22</v>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C743" t="n">
+        <v>6.099999904632568</v>
+      </c>
+      <c r="D743" t="n">
+        <v>20</v>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C744" t="n">
+        <v>8.609999656677246</v>
+      </c>
+      <c r="D744" t="n">
+        <v>25</v>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C745" t="n">
+        <v>5.230000019073486</v>
+      </c>
+      <c r="D745" t="n">
+        <v>30</v>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C746" t="n">
+        <v>49.72000122070312</v>
+      </c>
+      <c r="D746" t="n">
+        <v>23</v>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C747" t="n">
+        <v>4.150000095367432</v>
+      </c>
+      <c r="D747" t="n">
+        <v>20</v>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C748" t="n">
+        <v>60.88000106811523</v>
+      </c>
+      <c r="D748" t="n">
+        <v>8</v>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C749" t="n">
+        <v>47.95999908447266</v>
+      </c>
+      <c r="D749" t="n">
+        <v>16</v>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C750" t="n">
+        <v>19.3799991607666</v>
+      </c>
+      <c r="D750" t="n">
+        <v>63</v>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C751" t="n">
+        <v>38.09999847412109</v>
+      </c>
+      <c r="D751" t="n">
+        <v>35</v>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C752" t="n">
+        <v>110.9899978637695</v>
+      </c>
+      <c r="D752" t="n">
+        <v>31</v>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C753" t="n">
+        <v>47.5099983215332</v>
+      </c>
+      <c r="D753" t="n">
+        <v>11</v>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C754" t="n">
+        <v>7.03000020980835</v>
+      </c>
+      <c r="D754" t="n">
+        <v>11</v>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C755" t="n">
+        <v>39.83000183105469</v>
+      </c>
+      <c r="D755" t="n">
+        <v>48</v>
+      </c>
+      <c r="E755" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-24
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E755"/>
+  <dimension ref="A1:E784"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15618,7 +15618,7 @@
       </c>
     </row>
     <row r="727">
-      <c r="A727" s="2" t="n">
+      <c r="A727" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B727" t="inlineStr">
@@ -15639,7 +15639,7 @@
       </c>
     </row>
     <row r="728">
-      <c r="A728" s="2" t="n">
+      <c r="A728" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B728" t="inlineStr">
@@ -15660,7 +15660,7 @@
       </c>
     </row>
     <row r="729">
-      <c r="A729" s="2" t="n">
+      <c r="A729" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B729" t="inlineStr">
@@ -15681,7 +15681,7 @@
       </c>
     </row>
     <row r="730">
-      <c r="A730" s="2" t="n">
+      <c r="A730" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B730" t="inlineStr">
@@ -15702,7 +15702,7 @@
       </c>
     </row>
     <row r="731">
-      <c r="A731" s="2" t="n">
+      <c r="A731" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B731" t="inlineStr">
@@ -15723,7 +15723,7 @@
       </c>
     </row>
     <row r="732">
-      <c r="A732" s="2" t="n">
+      <c r="A732" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B732" t="inlineStr">
@@ -15744,7 +15744,7 @@
       </c>
     </row>
     <row r="733">
-      <c r="A733" s="2" t="n">
+      <c r="A733" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B733" t="inlineStr">
@@ -15765,7 +15765,7 @@
       </c>
     </row>
     <row r="734">
-      <c r="A734" s="2" t="n">
+      <c r="A734" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B734" t="inlineStr">
@@ -15786,7 +15786,7 @@
       </c>
     </row>
     <row r="735">
-      <c r="A735" s="2" t="n">
+      <c r="A735" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B735" t="inlineStr">
@@ -15807,7 +15807,7 @@
       </c>
     </row>
     <row r="736">
-      <c r="A736" s="2" t="n">
+      <c r="A736" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B736" t="inlineStr">
@@ -15828,7 +15828,7 @@
       </c>
     </row>
     <row r="737">
-      <c r="A737" s="2" t="n">
+      <c r="A737" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B737" t="inlineStr">
@@ -15849,7 +15849,7 @@
       </c>
     </row>
     <row r="738">
-      <c r="A738" s="2" t="n">
+      <c r="A738" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B738" t="inlineStr">
@@ -15870,7 +15870,7 @@
       </c>
     </row>
     <row r="739">
-      <c r="A739" s="2" t="n">
+      <c r="A739" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B739" t="inlineStr">
@@ -15891,7 +15891,7 @@
       </c>
     </row>
     <row r="740">
-      <c r="A740" s="2" t="n">
+      <c r="A740" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B740" t="inlineStr">
@@ -15912,7 +15912,7 @@
       </c>
     </row>
     <row r="741">
-      <c r="A741" s="2" t="n">
+      <c r="A741" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B741" t="inlineStr">
@@ -15933,7 +15933,7 @@
       </c>
     </row>
     <row r="742">
-      <c r="A742" s="2" t="n">
+      <c r="A742" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B742" t="inlineStr">
@@ -15954,7 +15954,7 @@
       </c>
     </row>
     <row r="743">
-      <c r="A743" s="2" t="n">
+      <c r="A743" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B743" t="inlineStr">
@@ -15975,7 +15975,7 @@
       </c>
     </row>
     <row r="744">
-      <c r="A744" s="2" t="n">
+      <c r="A744" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B744" t="inlineStr">
@@ -15996,7 +15996,7 @@
       </c>
     </row>
     <row r="745">
-      <c r="A745" s="2" t="n">
+      <c r="A745" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B745" t="inlineStr">
@@ -16017,7 +16017,7 @@
       </c>
     </row>
     <row r="746">
-      <c r="A746" s="2" t="n">
+      <c r="A746" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B746" t="inlineStr">
@@ -16038,7 +16038,7 @@
       </c>
     </row>
     <row r="747">
-      <c r="A747" s="2" t="n">
+      <c r="A747" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B747" t="inlineStr">
@@ -16059,7 +16059,7 @@
       </c>
     </row>
     <row r="748">
-      <c r="A748" s="2" t="n">
+      <c r="A748" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B748" t="inlineStr">
@@ -16080,7 +16080,7 @@
       </c>
     </row>
     <row r="749">
-      <c r="A749" s="2" t="n">
+      <c r="A749" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B749" t="inlineStr">
@@ -16101,7 +16101,7 @@
       </c>
     </row>
     <row r="750">
-      <c r="A750" s="2" t="n">
+      <c r="A750" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B750" t="inlineStr">
@@ -16122,7 +16122,7 @@
       </c>
     </row>
     <row r="751">
-      <c r="A751" s="2" t="n">
+      <c r="A751" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B751" t="inlineStr">
@@ -16143,7 +16143,7 @@
       </c>
     </row>
     <row r="752">
-      <c r="A752" s="2" t="n">
+      <c r="A752" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B752" t="inlineStr">
@@ -16164,7 +16164,7 @@
       </c>
     </row>
     <row r="753">
-      <c r="A753" s="2" t="n">
+      <c r="A753" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B753" t="inlineStr">
@@ -16185,7 +16185,7 @@
       </c>
     </row>
     <row r="754">
-      <c r="A754" s="2" t="n">
+      <c r="A754" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B754" t="inlineStr">
@@ -16206,7 +16206,7 @@
       </c>
     </row>
     <row r="755">
-      <c r="A755" s="2" t="n">
+      <c r="A755" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="B755" t="inlineStr">
@@ -16221,6 +16221,615 @@
         <v>48</v>
       </c>
       <c r="E755" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C756" t="n">
+        <v>29.1299991607666</v>
+      </c>
+      <c r="D756" t="n">
+        <v>28</v>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C757" t="n">
+        <v>13.27999973297119</v>
+      </c>
+      <c r="D757" t="n">
+        <v>31</v>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C758" t="n">
+        <v>21.56999969482422</v>
+      </c>
+      <c r="D758" t="n">
+        <v>30</v>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C759" t="n">
+        <v>4.070000171661377</v>
+      </c>
+      <c r="D759" t="n">
+        <v>16</v>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C760" t="n">
+        <v>0.9200000166893005</v>
+      </c>
+      <c r="D760" t="n">
+        <v>12</v>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C761" t="n">
+        <v>181.3699951171875</v>
+      </c>
+      <c r="D761" t="n">
+        <v>26</v>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C762" t="n">
+        <v>62.91999816894531</v>
+      </c>
+      <c r="D762" t="n">
+        <v>45</v>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C763" t="n">
+        <v>3.960000038146973</v>
+      </c>
+      <c r="D763" t="n">
+        <v>61</v>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C764" t="n">
+        <v>5.010000228881836</v>
+      </c>
+      <c r="D764" t="n">
+        <v>10</v>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C765" t="n">
+        <v>5.940000057220459</v>
+      </c>
+      <c r="D765" t="n">
+        <v>22</v>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C766" t="n">
+        <v>20.38999938964844</v>
+      </c>
+      <c r="D766" t="n">
+        <v>49</v>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C767" t="n">
+        <v>27.25</v>
+      </c>
+      <c r="D767" t="n">
+        <v>20</v>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C768" t="n">
+        <v>13.63000011444092</v>
+      </c>
+      <c r="D768" t="n">
+        <v>9</v>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C769" t="n">
+        <v>4.900000095367432</v>
+      </c>
+      <c r="D769" t="n">
+        <v>26</v>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C770" t="n">
+        <v>24.48999977111816</v>
+      </c>
+      <c r="D770" t="n">
+        <v>27</v>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C771" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="D771" t="n">
+        <v>22</v>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C772" t="n">
+        <v>6.289999961853027</v>
+      </c>
+      <c r="D772" t="n">
+        <v>20</v>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C773" t="n">
+        <v>8.869999885559082</v>
+      </c>
+      <c r="D773" t="n">
+        <v>25</v>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C774" t="n">
+        <v>5.199999809265137</v>
+      </c>
+      <c r="D774" t="n">
+        <v>30</v>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C775" t="n">
+        <v>49.33000183105469</v>
+      </c>
+      <c r="D775" t="n">
+        <v>23</v>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C776" t="n">
+        <v>4.130000114440918</v>
+      </c>
+      <c r="D776" t="n">
+        <v>20</v>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C777" t="n">
+        <v>60.90000152587891</v>
+      </c>
+      <c r="D777" t="n">
+        <v>8</v>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C778" t="n">
+        <v>47.02000045776367</v>
+      </c>
+      <c r="D778" t="n">
+        <v>16</v>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C779" t="n">
+        <v>18.42000007629395</v>
+      </c>
+      <c r="D779" t="n">
+        <v>63</v>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C780" t="n">
+        <v>37.77999877929688</v>
+      </c>
+      <c r="D780" t="n">
+        <v>35</v>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C781" t="n">
+        <v>110.2300033569336</v>
+      </c>
+      <c r="D781" t="n">
+        <v>31</v>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C782" t="n">
+        <v>45.52999877929688</v>
+      </c>
+      <c r="D782" t="n">
+        <v>11</v>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C783" t="n">
+        <v>6.840000152587891</v>
+      </c>
+      <c r="D783" t="n">
+        <v>11</v>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C784" t="n">
+        <v>39.04999923706055</v>
+      </c>
+      <c r="D784" t="n">
+        <v>48</v>
+      </c>
+      <c r="E784" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-25
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E784"/>
+  <dimension ref="A1:E813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16227,7 +16227,7 @@
       </c>
     </row>
     <row r="756">
-      <c r="A756" s="2" t="n">
+      <c r="A756" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B756" t="inlineStr">
@@ -16248,7 +16248,7 @@
       </c>
     </row>
     <row r="757">
-      <c r="A757" s="2" t="n">
+      <c r="A757" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B757" t="inlineStr">
@@ -16269,7 +16269,7 @@
       </c>
     </row>
     <row r="758">
-      <c r="A758" s="2" t="n">
+      <c r="A758" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B758" t="inlineStr">
@@ -16290,7 +16290,7 @@
       </c>
     </row>
     <row r="759">
-      <c r="A759" s="2" t="n">
+      <c r="A759" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B759" t="inlineStr">
@@ -16311,7 +16311,7 @@
       </c>
     </row>
     <row r="760">
-      <c r="A760" s="2" t="n">
+      <c r="A760" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B760" t="inlineStr">
@@ -16332,7 +16332,7 @@
       </c>
     </row>
     <row r="761">
-      <c r="A761" s="2" t="n">
+      <c r="A761" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B761" t="inlineStr">
@@ -16353,7 +16353,7 @@
       </c>
     </row>
     <row r="762">
-      <c r="A762" s="2" t="n">
+      <c r="A762" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B762" t="inlineStr">
@@ -16374,7 +16374,7 @@
       </c>
     </row>
     <row r="763">
-      <c r="A763" s="2" t="n">
+      <c r="A763" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B763" t="inlineStr">
@@ -16395,7 +16395,7 @@
       </c>
     </row>
     <row r="764">
-      <c r="A764" s="2" t="n">
+      <c r="A764" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B764" t="inlineStr">
@@ -16416,7 +16416,7 @@
       </c>
     </row>
     <row r="765">
-      <c r="A765" s="2" t="n">
+      <c r="A765" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B765" t="inlineStr">
@@ -16437,7 +16437,7 @@
       </c>
     </row>
     <row r="766">
-      <c r="A766" s="2" t="n">
+      <c r="A766" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B766" t="inlineStr">
@@ -16458,7 +16458,7 @@
       </c>
     </row>
     <row r="767">
-      <c r="A767" s="2" t="n">
+      <c r="A767" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B767" t="inlineStr">
@@ -16479,7 +16479,7 @@
       </c>
     </row>
     <row r="768">
-      <c r="A768" s="2" t="n">
+      <c r="A768" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B768" t="inlineStr">
@@ -16500,7 +16500,7 @@
       </c>
     </row>
     <row r="769">
-      <c r="A769" s="2" t="n">
+      <c r="A769" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B769" t="inlineStr">
@@ -16521,7 +16521,7 @@
       </c>
     </row>
     <row r="770">
-      <c r="A770" s="2" t="n">
+      <c r="A770" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B770" t="inlineStr">
@@ -16542,7 +16542,7 @@
       </c>
     </row>
     <row r="771">
-      <c r="A771" s="2" t="n">
+      <c r="A771" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B771" t="inlineStr">
@@ -16563,7 +16563,7 @@
       </c>
     </row>
     <row r="772">
-      <c r="A772" s="2" t="n">
+      <c r="A772" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B772" t="inlineStr">
@@ -16584,7 +16584,7 @@
       </c>
     </row>
     <row r="773">
-      <c r="A773" s="2" t="n">
+      <c r="A773" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B773" t="inlineStr">
@@ -16605,7 +16605,7 @@
       </c>
     </row>
     <row r="774">
-      <c r="A774" s="2" t="n">
+      <c r="A774" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B774" t="inlineStr">
@@ -16626,7 +16626,7 @@
       </c>
     </row>
     <row r="775">
-      <c r="A775" s="2" t="n">
+      <c r="A775" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B775" t="inlineStr">
@@ -16647,7 +16647,7 @@
       </c>
     </row>
     <row r="776">
-      <c r="A776" s="2" t="n">
+      <c r="A776" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B776" t="inlineStr">
@@ -16668,7 +16668,7 @@
       </c>
     </row>
     <row r="777">
-      <c r="A777" s="2" t="n">
+      <c r="A777" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B777" t="inlineStr">
@@ -16689,7 +16689,7 @@
       </c>
     </row>
     <row r="778">
-      <c r="A778" s="2" t="n">
+      <c r="A778" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B778" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
     </row>
     <row r="779">
-      <c r="A779" s="2" t="n">
+      <c r="A779" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B779" t="inlineStr">
@@ -16731,7 +16731,7 @@
       </c>
     </row>
     <row r="780">
-      <c r="A780" s="2" t="n">
+      <c r="A780" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B780" t="inlineStr">
@@ -16752,7 +16752,7 @@
       </c>
     </row>
     <row r="781">
-      <c r="A781" s="2" t="n">
+      <c r="A781" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B781" t="inlineStr">
@@ -16773,7 +16773,7 @@
       </c>
     </row>
     <row r="782">
-      <c r="A782" s="2" t="n">
+      <c r="A782" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B782" t="inlineStr">
@@ -16794,7 +16794,7 @@
       </c>
     </row>
     <row r="783">
-      <c r="A783" s="2" t="n">
+      <c r="A783" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B783" t="inlineStr">
@@ -16815,7 +16815,7 @@
       </c>
     </row>
     <row r="784">
-      <c r="A784" s="2" t="n">
+      <c r="A784" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="B784" t="inlineStr">
@@ -16830,6 +16830,615 @@
         <v>48</v>
       </c>
       <c r="E784" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C785" t="n">
+        <v>29.10000038146973</v>
+      </c>
+      <c r="D785" t="n">
+        <v>28</v>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C786" t="n">
+        <v>13.89999961853027</v>
+      </c>
+      <c r="D786" t="n">
+        <v>31</v>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C787" t="n">
+        <v>21.63999938964844</v>
+      </c>
+      <c r="D787" t="n">
+        <v>30</v>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C788" t="n">
+        <v>4.119999885559082</v>
+      </c>
+      <c r="D788" t="n">
+        <v>16</v>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C789" t="n">
+        <v>1.009999990463257</v>
+      </c>
+      <c r="D789" t="n">
+        <v>12</v>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C790" t="n">
+        <v>180.6300048828125</v>
+      </c>
+      <c r="D790" t="n">
+        <v>26</v>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C791" t="n">
+        <v>62.68000030517578</v>
+      </c>
+      <c r="D791" t="n">
+        <v>45</v>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C792" t="n">
+        <v>4.03000020980835</v>
+      </c>
+      <c r="D792" t="n">
+        <v>61</v>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C793" t="n">
+        <v>5</v>
+      </c>
+      <c r="D793" t="n">
+        <v>10</v>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C794" t="n">
+        <v>5.989999771118164</v>
+      </c>
+      <c r="D794" t="n">
+        <v>22</v>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C795" t="n">
+        <v>20.52000045776367</v>
+      </c>
+      <c r="D795" t="n">
+        <v>49</v>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C796" t="n">
+        <v>27.44000053405762</v>
+      </c>
+      <c r="D796" t="n">
+        <v>20</v>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C797" t="n">
+        <v>13.6899995803833</v>
+      </c>
+      <c r="D797" t="n">
+        <v>9</v>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C798" t="n">
+        <v>4.900000095367432</v>
+      </c>
+      <c r="D798" t="n">
+        <v>26</v>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C799" t="n">
+        <v>24.64999961853027</v>
+      </c>
+      <c r="D799" t="n">
+        <v>27</v>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C800" t="n">
+        <v>11.77000045776367</v>
+      </c>
+      <c r="D800" t="n">
+        <v>22</v>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C801" t="n">
+        <v>6.71999979019165</v>
+      </c>
+      <c r="D801" t="n">
+        <v>20</v>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C802" t="n">
+        <v>9.020000457763672</v>
+      </c>
+      <c r="D802" t="n">
+        <v>25</v>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C803" t="n">
+        <v>5.199999809265137</v>
+      </c>
+      <c r="D803" t="n">
+        <v>30</v>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C804" t="n">
+        <v>48.04000091552734</v>
+      </c>
+      <c r="D804" t="n">
+        <v>23</v>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C805" t="n">
+        <v>4.119999885559082</v>
+      </c>
+      <c r="D805" t="n">
+        <v>20</v>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C806" t="n">
+        <v>59.52999877929688</v>
+      </c>
+      <c r="D806" t="n">
+        <v>8</v>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C807" t="n">
+        <v>47.22000122070312</v>
+      </c>
+      <c r="D807" t="n">
+        <v>16</v>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C808" t="n">
+        <v>18.13999938964844</v>
+      </c>
+      <c r="D808" t="n">
+        <v>63</v>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C809" t="n">
+        <v>37.36999893188477</v>
+      </c>
+      <c r="D809" t="n">
+        <v>35</v>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C810" t="n">
+        <v>110.4300003051758</v>
+      </c>
+      <c r="D810" t="n">
+        <v>31</v>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C811" t="n">
+        <v>45.04999923706055</v>
+      </c>
+      <c r="D811" t="n">
+        <v>11</v>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C812" t="n">
+        <v>6.900000095367432</v>
+      </c>
+      <c r="D812" t="n">
+        <v>11</v>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C813" t="n">
+        <v>37.41999816894531</v>
+      </c>
+      <c r="D813" t="n">
+        <v>48</v>
+      </c>
+      <c r="E813" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-28
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E813"/>
+  <dimension ref="A1:E842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16836,7 +16836,7 @@
       </c>
     </row>
     <row r="785">
-      <c r="A785" s="2" t="n">
+      <c r="A785" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B785" t="inlineStr">
@@ -16857,7 +16857,7 @@
       </c>
     </row>
     <row r="786">
-      <c r="A786" s="2" t="n">
+      <c r="A786" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B786" t="inlineStr">
@@ -16878,7 +16878,7 @@
       </c>
     </row>
     <row r="787">
-      <c r="A787" s="2" t="n">
+      <c r="A787" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B787" t="inlineStr">
@@ -16899,7 +16899,7 @@
       </c>
     </row>
     <row r="788">
-      <c r="A788" s="2" t="n">
+      <c r="A788" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B788" t="inlineStr">
@@ -16920,7 +16920,7 @@
       </c>
     </row>
     <row r="789">
-      <c r="A789" s="2" t="n">
+      <c r="A789" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B789" t="inlineStr">
@@ -16941,7 +16941,7 @@
       </c>
     </row>
     <row r="790">
-      <c r="A790" s="2" t="n">
+      <c r="A790" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B790" t="inlineStr">
@@ -16962,7 +16962,7 @@
       </c>
     </row>
     <row r="791">
-      <c r="A791" s="2" t="n">
+      <c r="A791" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B791" t="inlineStr">
@@ -16983,7 +16983,7 @@
       </c>
     </row>
     <row r="792">
-      <c r="A792" s="2" t="n">
+      <c r="A792" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B792" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
     </row>
     <row r="793">
-      <c r="A793" s="2" t="n">
+      <c r="A793" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B793" t="inlineStr">
@@ -17025,7 +17025,7 @@
       </c>
     </row>
     <row r="794">
-      <c r="A794" s="2" t="n">
+      <c r="A794" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B794" t="inlineStr">
@@ -17046,7 +17046,7 @@
       </c>
     </row>
     <row r="795">
-      <c r="A795" s="2" t="n">
+      <c r="A795" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B795" t="inlineStr">
@@ -17067,7 +17067,7 @@
       </c>
     </row>
     <row r="796">
-      <c r="A796" s="2" t="n">
+      <c r="A796" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B796" t="inlineStr">
@@ -17088,7 +17088,7 @@
       </c>
     </row>
     <row r="797">
-      <c r="A797" s="2" t="n">
+      <c r="A797" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B797" t="inlineStr">
@@ -17109,7 +17109,7 @@
       </c>
     </row>
     <row r="798">
-      <c r="A798" s="2" t="n">
+      <c r="A798" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B798" t="inlineStr">
@@ -17130,7 +17130,7 @@
       </c>
     </row>
     <row r="799">
-      <c r="A799" s="2" t="n">
+      <c r="A799" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B799" t="inlineStr">
@@ -17151,7 +17151,7 @@
       </c>
     </row>
     <row r="800">
-      <c r="A800" s="2" t="n">
+      <c r="A800" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B800" t="inlineStr">
@@ -17172,7 +17172,7 @@
       </c>
     </row>
     <row r="801">
-      <c r="A801" s="2" t="n">
+      <c r="A801" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B801" t="inlineStr">
@@ -17193,7 +17193,7 @@
       </c>
     </row>
     <row r="802">
-      <c r="A802" s="2" t="n">
+      <c r="A802" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B802" t="inlineStr">
@@ -17214,7 +17214,7 @@
       </c>
     </row>
     <row r="803">
-      <c r="A803" s="2" t="n">
+      <c r="A803" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B803" t="inlineStr">
@@ -17235,7 +17235,7 @@
       </c>
     </row>
     <row r="804">
-      <c r="A804" s="2" t="n">
+      <c r="A804" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B804" t="inlineStr">
@@ -17256,7 +17256,7 @@
       </c>
     </row>
     <row r="805">
-      <c r="A805" s="2" t="n">
+      <c r="A805" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B805" t="inlineStr">
@@ -17277,7 +17277,7 @@
       </c>
     </row>
     <row r="806">
-      <c r="A806" s="2" t="n">
+      <c r="A806" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B806" t="inlineStr">
@@ -17298,7 +17298,7 @@
       </c>
     </row>
     <row r="807">
-      <c r="A807" s="2" t="n">
+      <c r="A807" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B807" t="inlineStr">
@@ -17319,7 +17319,7 @@
       </c>
     </row>
     <row r="808">
-      <c r="A808" s="2" t="n">
+      <c r="A808" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B808" t="inlineStr">
@@ -17340,7 +17340,7 @@
       </c>
     </row>
     <row r="809">
-      <c r="A809" s="2" t="n">
+      <c r="A809" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B809" t="inlineStr">
@@ -17361,7 +17361,7 @@
       </c>
     </row>
     <row r="810">
-      <c r="A810" s="2" t="n">
+      <c r="A810" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B810" t="inlineStr">
@@ -17382,7 +17382,7 @@
       </c>
     </row>
     <row r="811">
-      <c r="A811" s="2" t="n">
+      <c r="A811" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B811" t="inlineStr">
@@ -17403,7 +17403,7 @@
       </c>
     </row>
     <row r="812">
-      <c r="A812" s="2" t="n">
+      <c r="A812" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B812" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
     </row>
     <row r="813">
-      <c r="A813" s="2" t="n">
+      <c r="A813" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="B813" t="inlineStr">
@@ -17439,6 +17439,615 @@
         <v>48</v>
       </c>
       <c r="E813" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C814" t="n">
+        <v>28.45999908447266</v>
+      </c>
+      <c r="D814" t="n">
+        <v>28</v>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C815" t="n">
+        <v>14.23999977111816</v>
+      </c>
+      <c r="D815" t="n">
+        <v>31</v>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C816" t="n">
+        <v>21.54999923706055</v>
+      </c>
+      <c r="D816" t="n">
+        <v>30</v>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C817" t="n">
+        <v>4.019999980926514</v>
+      </c>
+      <c r="D817" t="n">
+        <v>16</v>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C818" t="n">
+        <v>1.039999961853027</v>
+      </c>
+      <c r="D818" t="n">
+        <v>12</v>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C819" t="n">
+        <v>180.3200073242188</v>
+      </c>
+      <c r="D819" t="n">
+        <v>26</v>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C820" t="n">
+        <v>62.40999984741211</v>
+      </c>
+      <c r="D820" t="n">
+        <v>45</v>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C821" t="n">
+        <v>3.920000076293945</v>
+      </c>
+      <c r="D821" t="n">
+        <v>61</v>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C822" t="n">
+        <v>5.039999961853027</v>
+      </c>
+      <c r="D822" t="n">
+        <v>10</v>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C823" t="n">
+        <v>5.980000019073486</v>
+      </c>
+      <c r="D823" t="n">
+        <v>22</v>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C824" t="n">
+        <v>20.1200008392334</v>
+      </c>
+      <c r="D824" t="n">
+        <v>49</v>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C825" t="n">
+        <v>26.79000091552734</v>
+      </c>
+      <c r="D825" t="n">
+        <v>20</v>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C826" t="n">
+        <v>13.3100004196167</v>
+      </c>
+      <c r="D826" t="n">
+        <v>9</v>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C827" t="n">
+        <v>4.829999923706055</v>
+      </c>
+      <c r="D827" t="n">
+        <v>26</v>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C828" t="n">
+        <v>24.61000061035156</v>
+      </c>
+      <c r="D828" t="n">
+        <v>27</v>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C829" t="n">
+        <v>11.35999965667725</v>
+      </c>
+      <c r="D829" t="n">
+        <v>22</v>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C830" t="n">
+        <v>6.619999885559082</v>
+      </c>
+      <c r="D830" t="n">
+        <v>20</v>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C831" t="n">
+        <v>8.939999580383301</v>
+      </c>
+      <c r="D831" t="n">
+        <v>25</v>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C832" t="n">
+        <v>5.230000019073486</v>
+      </c>
+      <c r="D832" t="n">
+        <v>30</v>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C833" t="n">
+        <v>48.86999893188477</v>
+      </c>
+      <c r="D833" t="n">
+        <v>23</v>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C834" t="n">
+        <v>4.199999809265137</v>
+      </c>
+      <c r="D834" t="n">
+        <v>20</v>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C835" t="n">
+        <v>61.70999908447266</v>
+      </c>
+      <c r="D835" t="n">
+        <v>8</v>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C836" t="n">
+        <v>46.90999984741211</v>
+      </c>
+      <c r="D836" t="n">
+        <v>16</v>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C837" t="n">
+        <v>17.70000076293945</v>
+      </c>
+      <c r="D837" t="n">
+        <v>63</v>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C838" t="n">
+        <v>37.54000091552734</v>
+      </c>
+      <c r="D838" t="n">
+        <v>35</v>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C839" t="n">
+        <v>109.1900024414062</v>
+      </c>
+      <c r="D839" t="n">
+        <v>31</v>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C840" t="n">
+        <v>44.75</v>
+      </c>
+      <c r="D840" t="n">
+        <v>11</v>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C841" t="n">
+        <v>6.989999771118164</v>
+      </c>
+      <c r="D841" t="n">
+        <v>11</v>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C842" t="n">
+        <v>37.95000076293945</v>
+      </c>
+      <c r="D842" t="n">
+        <v>48</v>
+      </c>
+      <c r="E842" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-29
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E842"/>
+  <dimension ref="A1:E871"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17445,7 +17445,7 @@
       </c>
     </row>
     <row r="814">
-      <c r="A814" s="2" t="n">
+      <c r="A814" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B814" t="inlineStr">
@@ -17466,7 +17466,7 @@
       </c>
     </row>
     <row r="815">
-      <c r="A815" s="2" t="n">
+      <c r="A815" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B815" t="inlineStr">
@@ -17487,7 +17487,7 @@
       </c>
     </row>
     <row r="816">
-      <c r="A816" s="2" t="n">
+      <c r="A816" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B816" t="inlineStr">
@@ -17508,7 +17508,7 @@
       </c>
     </row>
     <row r="817">
-      <c r="A817" s="2" t="n">
+      <c r="A817" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B817" t="inlineStr">
@@ -17529,7 +17529,7 @@
       </c>
     </row>
     <row r="818">
-      <c r="A818" s="2" t="n">
+      <c r="A818" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B818" t="inlineStr">
@@ -17550,7 +17550,7 @@
       </c>
     </row>
     <row r="819">
-      <c r="A819" s="2" t="n">
+      <c r="A819" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B819" t="inlineStr">
@@ -17571,7 +17571,7 @@
       </c>
     </row>
     <row r="820">
-      <c r="A820" s="2" t="n">
+      <c r="A820" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B820" t="inlineStr">
@@ -17592,7 +17592,7 @@
       </c>
     </row>
     <row r="821">
-      <c r="A821" s="2" t="n">
+      <c r="A821" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B821" t="inlineStr">
@@ -17613,7 +17613,7 @@
       </c>
     </row>
     <row r="822">
-      <c r="A822" s="2" t="n">
+      <c r="A822" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B822" t="inlineStr">
@@ -17634,7 +17634,7 @@
       </c>
     </row>
     <row r="823">
-      <c r="A823" s="2" t="n">
+      <c r="A823" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B823" t="inlineStr">
@@ -17655,7 +17655,7 @@
       </c>
     </row>
     <row r="824">
-      <c r="A824" s="2" t="n">
+      <c r="A824" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B824" t="inlineStr">
@@ -17676,7 +17676,7 @@
       </c>
     </row>
     <row r="825">
-      <c r="A825" s="2" t="n">
+      <c r="A825" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B825" t="inlineStr">
@@ -17697,7 +17697,7 @@
       </c>
     </row>
     <row r="826">
-      <c r="A826" s="2" t="n">
+      <c r="A826" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B826" t="inlineStr">
@@ -17718,7 +17718,7 @@
       </c>
     </row>
     <row r="827">
-      <c r="A827" s="2" t="n">
+      <c r="A827" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B827" t="inlineStr">
@@ -17739,7 +17739,7 @@
       </c>
     </row>
     <row r="828">
-      <c r="A828" s="2" t="n">
+      <c r="A828" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B828" t="inlineStr">
@@ -17760,7 +17760,7 @@
       </c>
     </row>
     <row r="829">
-      <c r="A829" s="2" t="n">
+      <c r="A829" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B829" t="inlineStr">
@@ -17781,7 +17781,7 @@
       </c>
     </row>
     <row r="830">
-      <c r="A830" s="2" t="n">
+      <c r="A830" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B830" t="inlineStr">
@@ -17802,7 +17802,7 @@
       </c>
     </row>
     <row r="831">
-      <c r="A831" s="2" t="n">
+      <c r="A831" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B831" t="inlineStr">
@@ -17823,7 +17823,7 @@
       </c>
     </row>
     <row r="832">
-      <c r="A832" s="2" t="n">
+      <c r="A832" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B832" t="inlineStr">
@@ -17844,7 +17844,7 @@
       </c>
     </row>
     <row r="833">
-      <c r="A833" s="2" t="n">
+      <c r="A833" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B833" t="inlineStr">
@@ -17865,7 +17865,7 @@
       </c>
     </row>
     <row r="834">
-      <c r="A834" s="2" t="n">
+      <c r="A834" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B834" t="inlineStr">
@@ -17886,7 +17886,7 @@
       </c>
     </row>
     <row r="835">
-      <c r="A835" s="2" t="n">
+      <c r="A835" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B835" t="inlineStr">
@@ -17907,7 +17907,7 @@
       </c>
     </row>
     <row r="836">
-      <c r="A836" s="2" t="n">
+      <c r="A836" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B836" t="inlineStr">
@@ -17928,7 +17928,7 @@
       </c>
     </row>
     <row r="837">
-      <c r="A837" s="2" t="n">
+      <c r="A837" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B837" t="inlineStr">
@@ -17949,7 +17949,7 @@
       </c>
     </row>
     <row r="838">
-      <c r="A838" s="2" t="n">
+      <c r="A838" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B838" t="inlineStr">
@@ -17970,7 +17970,7 @@
       </c>
     </row>
     <row r="839">
-      <c r="A839" s="2" t="n">
+      <c r="A839" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B839" t="inlineStr">
@@ -17991,7 +17991,7 @@
       </c>
     </row>
     <row r="840">
-      <c r="A840" s="2" t="n">
+      <c r="A840" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B840" t="inlineStr">
@@ -18012,7 +18012,7 @@
       </c>
     </row>
     <row r="841">
-      <c r="A841" s="2" t="n">
+      <c r="A841" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B841" t="inlineStr">
@@ -18033,7 +18033,7 @@
       </c>
     </row>
     <row r="842">
-      <c r="A842" s="2" t="n">
+      <c r="A842" s="1" t="n">
         <v>46293</v>
       </c>
       <c r="B842" t="inlineStr">
@@ -18048,6 +18048,615 @@
         <v>48</v>
       </c>
       <c r="E842" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C843" t="n">
+        <v>28.77000045776367</v>
+      </c>
+      <c r="D843" t="n">
+        <v>28</v>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C844" t="n">
+        <v>14</v>
+      </c>
+      <c r="D844" t="n">
+        <v>31</v>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C845" t="n">
+        <v>22.06999969482422</v>
+      </c>
+      <c r="D845" t="n">
+        <v>30</v>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C846" t="n">
+        <v>3.910000085830688</v>
+      </c>
+      <c r="D846" t="n">
+        <v>16</v>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C847" t="n">
+        <v>1.070000052452087</v>
+      </c>
+      <c r="D847" t="n">
+        <v>12</v>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C848" t="n">
+        <v>180.8999938964844</v>
+      </c>
+      <c r="D848" t="n">
+        <v>26</v>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C849" t="n">
+        <v>62.77000045776367</v>
+      </c>
+      <c r="D849" t="n">
+        <v>45</v>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C850" t="n">
+        <v>3.690000057220459</v>
+      </c>
+      <c r="D850" t="n">
+        <v>61</v>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C851" t="n">
+        <v>4.739999771118164</v>
+      </c>
+      <c r="D851" t="n">
+        <v>10</v>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C852" t="n">
+        <v>5.380000114440918</v>
+      </c>
+      <c r="D852" t="n">
+        <v>22</v>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C853" t="n">
+        <v>20.10000038146973</v>
+      </c>
+      <c r="D853" t="n">
+        <v>49</v>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C854" t="n">
+        <v>27.11000061035156</v>
+      </c>
+      <c r="D854" t="n">
+        <v>20</v>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C855" t="n">
+        <v>13.47000026702881</v>
+      </c>
+      <c r="D855" t="n">
+        <v>9</v>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C856" t="n">
+        <v>5.059999942779541</v>
+      </c>
+      <c r="D856" t="n">
+        <v>26</v>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C857" t="n">
+        <v>23.70000076293945</v>
+      </c>
+      <c r="D857" t="n">
+        <v>27</v>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C858" t="n">
+        <v>11.61999988555908</v>
+      </c>
+      <c r="D858" t="n">
+        <v>22</v>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C859" t="n">
+        <v>6.559999942779541</v>
+      </c>
+      <c r="D859" t="n">
+        <v>20</v>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C860" t="n">
+        <v>9.279999732971191</v>
+      </c>
+      <c r="D860" t="n">
+        <v>25</v>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C861" t="n">
+        <v>5.369999885559082</v>
+      </c>
+      <c r="D861" t="n">
+        <v>30</v>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C862" t="n">
+        <v>49.02999877929688</v>
+      </c>
+      <c r="D862" t="n">
+        <v>23</v>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C863" t="n">
+        <v>4.119999885559082</v>
+      </c>
+      <c r="D863" t="n">
+        <v>20</v>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C864" t="n">
+        <v>61.58000183105469</v>
+      </c>
+      <c r="D864" t="n">
+        <v>8</v>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C865" t="n">
+        <v>47.08000183105469</v>
+      </c>
+      <c r="D865" t="n">
+        <v>16</v>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C866" t="n">
+        <v>18.15999984741211</v>
+      </c>
+      <c r="D866" t="n">
+        <v>63</v>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C867" t="n">
+        <v>37.54000091552734</v>
+      </c>
+      <c r="D867" t="n">
+        <v>35</v>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C868" t="n">
+        <v>109.9199981689453</v>
+      </c>
+      <c r="D868" t="n">
+        <v>31</v>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C869" t="n">
+        <v>44.38999938964844</v>
+      </c>
+      <c r="D869" t="n">
+        <v>11</v>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C870" t="n">
+        <v>6.929999828338623</v>
+      </c>
+      <c r="D870" t="n">
+        <v>11</v>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C871" t="n">
+        <v>37.93999862670898</v>
+      </c>
+      <c r="D871" t="n">
+        <v>48</v>
+      </c>
+      <c r="E871" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-30
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E871"/>
+  <dimension ref="A1:E900"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18054,7 +18054,7 @@
       </c>
     </row>
     <row r="843">
-      <c r="A843" s="2" t="n">
+      <c r="A843" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B843" t="inlineStr">
@@ -18075,7 +18075,7 @@
       </c>
     </row>
     <row r="844">
-      <c r="A844" s="2" t="n">
+      <c r="A844" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B844" t="inlineStr">
@@ -18096,7 +18096,7 @@
       </c>
     </row>
     <row r="845">
-      <c r="A845" s="2" t="n">
+      <c r="A845" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B845" t="inlineStr">
@@ -18117,7 +18117,7 @@
       </c>
     </row>
     <row r="846">
-      <c r="A846" s="2" t="n">
+      <c r="A846" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B846" t="inlineStr">
@@ -18138,7 +18138,7 @@
       </c>
     </row>
     <row r="847">
-      <c r="A847" s="2" t="n">
+      <c r="A847" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B847" t="inlineStr">
@@ -18159,7 +18159,7 @@
       </c>
     </row>
     <row r="848">
-      <c r="A848" s="2" t="n">
+      <c r="A848" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B848" t="inlineStr">
@@ -18180,7 +18180,7 @@
       </c>
     </row>
     <row r="849">
-      <c r="A849" s="2" t="n">
+      <c r="A849" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B849" t="inlineStr">
@@ -18201,7 +18201,7 @@
       </c>
     </row>
     <row r="850">
-      <c r="A850" s="2" t="n">
+      <c r="A850" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B850" t="inlineStr">
@@ -18222,7 +18222,7 @@
       </c>
     </row>
     <row r="851">
-      <c r="A851" s="2" t="n">
+      <c r="A851" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B851" t="inlineStr">
@@ -18243,7 +18243,7 @@
       </c>
     </row>
     <row r="852">
-      <c r="A852" s="2" t="n">
+      <c r="A852" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B852" t="inlineStr">
@@ -18264,7 +18264,7 @@
       </c>
     </row>
     <row r="853">
-      <c r="A853" s="2" t="n">
+      <c r="A853" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B853" t="inlineStr">
@@ -18285,7 +18285,7 @@
       </c>
     </row>
     <row r="854">
-      <c r="A854" s="2" t="n">
+      <c r="A854" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B854" t="inlineStr">
@@ -18306,7 +18306,7 @@
       </c>
     </row>
     <row r="855">
-      <c r="A855" s="2" t="n">
+      <c r="A855" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B855" t="inlineStr">
@@ -18327,7 +18327,7 @@
       </c>
     </row>
     <row r="856">
-      <c r="A856" s="2" t="n">
+      <c r="A856" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B856" t="inlineStr">
@@ -18348,7 +18348,7 @@
       </c>
     </row>
     <row r="857">
-      <c r="A857" s="2" t="n">
+      <c r="A857" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B857" t="inlineStr">
@@ -18369,7 +18369,7 @@
       </c>
     </row>
     <row r="858">
-      <c r="A858" s="2" t="n">
+      <c r="A858" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B858" t="inlineStr">
@@ -18390,7 +18390,7 @@
       </c>
     </row>
     <row r="859">
-      <c r="A859" s="2" t="n">
+      <c r="A859" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B859" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
     </row>
     <row r="860">
-      <c r="A860" s="2" t="n">
+      <c r="A860" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B860" t="inlineStr">
@@ -18432,7 +18432,7 @@
       </c>
     </row>
     <row r="861">
-      <c r="A861" s="2" t="n">
+      <c r="A861" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B861" t="inlineStr">
@@ -18453,7 +18453,7 @@
       </c>
     </row>
     <row r="862">
-      <c r="A862" s="2" t="n">
+      <c r="A862" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B862" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
     </row>
     <row r="863">
-      <c r="A863" s="2" t="n">
+      <c r="A863" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B863" t="inlineStr">
@@ -18495,7 +18495,7 @@
       </c>
     </row>
     <row r="864">
-      <c r="A864" s="2" t="n">
+      <c r="A864" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B864" t="inlineStr">
@@ -18516,7 +18516,7 @@
       </c>
     </row>
     <row r="865">
-      <c r="A865" s="2" t="n">
+      <c r="A865" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B865" t="inlineStr">
@@ -18537,7 +18537,7 @@
       </c>
     </row>
     <row r="866">
-      <c r="A866" s="2" t="n">
+      <c r="A866" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B866" t="inlineStr">
@@ -18558,7 +18558,7 @@
       </c>
     </row>
     <row r="867">
-      <c r="A867" s="2" t="n">
+      <c r="A867" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B867" t="inlineStr">
@@ -18579,7 +18579,7 @@
       </c>
     </row>
     <row r="868">
-      <c r="A868" s="2" t="n">
+      <c r="A868" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B868" t="inlineStr">
@@ -18600,7 +18600,7 @@
       </c>
     </row>
     <row r="869">
-      <c r="A869" s="2" t="n">
+      <c r="A869" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B869" t="inlineStr">
@@ -18621,7 +18621,7 @@
       </c>
     </row>
     <row r="870">
-      <c r="A870" s="2" t="n">
+      <c r="A870" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B870" t="inlineStr">
@@ -18642,7 +18642,7 @@
       </c>
     </row>
     <row r="871">
-      <c r="A871" s="2" t="n">
+      <c r="A871" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="B871" t="inlineStr">
@@ -18657,6 +18657,615 @@
         <v>48</v>
       </c>
       <c r="E871" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C872" t="n">
+        <v>29.53000068664551</v>
+      </c>
+      <c r="D872" t="n">
+        <v>28</v>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C873" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="D873" t="n">
+        <v>31</v>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C874" t="n">
+        <v>22.96999931335449</v>
+      </c>
+      <c r="D874" t="n">
+        <v>30</v>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C875" t="n">
+        <v>3.960000038146973</v>
+      </c>
+      <c r="D875" t="n">
+        <v>16</v>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C876" t="n">
+        <v>1.230000019073486</v>
+      </c>
+      <c r="D876" t="n">
+        <v>12</v>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C877" t="n">
+        <v>183.8200073242188</v>
+      </c>
+      <c r="D877" t="n">
+        <v>26</v>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C878" t="n">
+        <v>64.20999908447266</v>
+      </c>
+      <c r="D878" t="n">
+        <v>45</v>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C879" t="n">
+        <v>3.730000019073486</v>
+      </c>
+      <c r="D879" t="n">
+        <v>61</v>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C880" t="n">
+        <v>5.050000190734863</v>
+      </c>
+      <c r="D880" t="n">
+        <v>10</v>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C881" t="n">
+        <v>5.670000076293945</v>
+      </c>
+      <c r="D881" t="n">
+        <v>22</v>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C882" t="n">
+        <v>19.93000030517578</v>
+      </c>
+      <c r="D882" t="n">
+        <v>49</v>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C883" t="n">
+        <v>27.95000076293945</v>
+      </c>
+      <c r="D883" t="n">
+        <v>20</v>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C884" t="n">
+        <v>14.05000019073486</v>
+      </c>
+      <c r="D884" t="n">
+        <v>9</v>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C885" t="n">
+        <v>5.059999942779541</v>
+      </c>
+      <c r="D885" t="n">
+        <v>26</v>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C886" t="n">
+        <v>24.59000015258789</v>
+      </c>
+      <c r="D886" t="n">
+        <v>27</v>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C887" t="n">
+        <v>11.78999996185303</v>
+      </c>
+      <c r="D887" t="n">
+        <v>22</v>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C888" t="n">
+        <v>7.369999885559082</v>
+      </c>
+      <c r="D888" t="n">
+        <v>20</v>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C889" t="n">
+        <v>9.970000267028809</v>
+      </c>
+      <c r="D889" t="n">
+        <v>25</v>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C890" t="n">
+        <v>5.510000228881836</v>
+      </c>
+      <c r="D890" t="n">
+        <v>30</v>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C891" t="n">
+        <v>49.27000045776367</v>
+      </c>
+      <c r="D891" t="n">
+        <v>23</v>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C892" t="n">
+        <v>4.179999828338623</v>
+      </c>
+      <c r="D892" t="n">
+        <v>20</v>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C893" t="n">
+        <v>61.13000106811523</v>
+      </c>
+      <c r="D893" t="n">
+        <v>8</v>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C894" t="n">
+        <v>47.29000091552734</v>
+      </c>
+      <c r="D894" t="n">
+        <v>16</v>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C895" t="n">
+        <v>18.47999954223633</v>
+      </c>
+      <c r="D895" t="n">
+        <v>63</v>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C896" t="n">
+        <v>38.11999893188477</v>
+      </c>
+      <c r="D896" t="n">
+        <v>35</v>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C897" t="n">
+        <v>112.120002746582</v>
+      </c>
+      <c r="D897" t="n">
+        <v>31</v>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C898" t="n">
+        <v>44.34000015258789</v>
+      </c>
+      <c r="D898" t="n">
+        <v>11</v>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C899" t="n">
+        <v>6.989999771118164</v>
+      </c>
+      <c r="D899" t="n">
+        <v>11</v>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C900" t="n">
+        <v>37.02999877929688</v>
+      </c>
+      <c r="D900" t="n">
+        <v>48</v>
+      </c>
+      <c r="E900" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-01
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E900"/>
+  <dimension ref="A1:E929"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18663,7 +18663,7 @@
       </c>
     </row>
     <row r="872">
-      <c r="A872" s="2" t="n">
+      <c r="A872" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B872" t="inlineStr">
@@ -18684,7 +18684,7 @@
       </c>
     </row>
     <row r="873">
-      <c r="A873" s="2" t="n">
+      <c r="A873" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B873" t="inlineStr">
@@ -18705,7 +18705,7 @@
       </c>
     </row>
     <row r="874">
-      <c r="A874" s="2" t="n">
+      <c r="A874" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B874" t="inlineStr">
@@ -18726,7 +18726,7 @@
       </c>
     </row>
     <row r="875">
-      <c r="A875" s="2" t="n">
+      <c r="A875" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B875" t="inlineStr">
@@ -18747,7 +18747,7 @@
       </c>
     </row>
     <row r="876">
-      <c r="A876" s="2" t="n">
+      <c r="A876" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B876" t="inlineStr">
@@ -18768,7 +18768,7 @@
       </c>
     </row>
     <row r="877">
-      <c r="A877" s="2" t="n">
+      <c r="A877" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B877" t="inlineStr">
@@ -18789,7 +18789,7 @@
       </c>
     </row>
     <row r="878">
-      <c r="A878" s="2" t="n">
+      <c r="A878" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B878" t="inlineStr">
@@ -18810,7 +18810,7 @@
       </c>
     </row>
     <row r="879">
-      <c r="A879" s="2" t="n">
+      <c r="A879" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B879" t="inlineStr">
@@ -18831,7 +18831,7 @@
       </c>
     </row>
     <row r="880">
-      <c r="A880" s="2" t="n">
+      <c r="A880" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B880" t="inlineStr">
@@ -18852,7 +18852,7 @@
       </c>
     </row>
     <row r="881">
-      <c r="A881" s="2" t="n">
+      <c r="A881" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B881" t="inlineStr">
@@ -18873,7 +18873,7 @@
       </c>
     </row>
     <row r="882">
-      <c r="A882" s="2" t="n">
+      <c r="A882" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B882" t="inlineStr">
@@ -18894,7 +18894,7 @@
       </c>
     </row>
     <row r="883">
-      <c r="A883" s="2" t="n">
+      <c r="A883" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B883" t="inlineStr">
@@ -18915,7 +18915,7 @@
       </c>
     </row>
     <row r="884">
-      <c r="A884" s="2" t="n">
+      <c r="A884" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B884" t="inlineStr">
@@ -18936,7 +18936,7 @@
       </c>
     </row>
     <row r="885">
-      <c r="A885" s="2" t="n">
+      <c r="A885" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B885" t="inlineStr">
@@ -18957,7 +18957,7 @@
       </c>
     </row>
     <row r="886">
-      <c r="A886" s="2" t="n">
+      <c r="A886" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B886" t="inlineStr">
@@ -18978,7 +18978,7 @@
       </c>
     </row>
     <row r="887">
-      <c r="A887" s="2" t="n">
+      <c r="A887" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B887" t="inlineStr">
@@ -18999,7 +18999,7 @@
       </c>
     </row>
     <row r="888">
-      <c r="A888" s="2" t="n">
+      <c r="A888" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B888" t="inlineStr">
@@ -19020,7 +19020,7 @@
       </c>
     </row>
     <row r="889">
-      <c r="A889" s="2" t="n">
+      <c r="A889" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B889" t="inlineStr">
@@ -19041,7 +19041,7 @@
       </c>
     </row>
     <row r="890">
-      <c r="A890" s="2" t="n">
+      <c r="A890" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B890" t="inlineStr">
@@ -19062,7 +19062,7 @@
       </c>
     </row>
     <row r="891">
-      <c r="A891" s="2" t="n">
+      <c r="A891" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B891" t="inlineStr">
@@ -19083,7 +19083,7 @@
       </c>
     </row>
     <row r="892">
-      <c r="A892" s="2" t="n">
+      <c r="A892" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B892" t="inlineStr">
@@ -19104,7 +19104,7 @@
       </c>
     </row>
     <row r="893">
-      <c r="A893" s="2" t="n">
+      <c r="A893" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B893" t="inlineStr">
@@ -19125,7 +19125,7 @@
       </c>
     </row>
     <row r="894">
-      <c r="A894" s="2" t="n">
+      <c r="A894" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B894" t="inlineStr">
@@ -19146,7 +19146,7 @@
       </c>
     </row>
     <row r="895">
-      <c r="A895" s="2" t="n">
+      <c r="A895" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B895" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
     </row>
     <row r="896">
-      <c r="A896" s="2" t="n">
+      <c r="A896" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B896" t="inlineStr">
@@ -19188,7 +19188,7 @@
       </c>
     </row>
     <row r="897">
-      <c r="A897" s="2" t="n">
+      <c r="A897" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B897" t="inlineStr">
@@ -19209,7 +19209,7 @@
       </c>
     </row>
     <row r="898">
-      <c r="A898" s="2" t="n">
+      <c r="A898" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B898" t="inlineStr">
@@ -19230,7 +19230,7 @@
       </c>
     </row>
     <row r="899">
-      <c r="A899" s="2" t="n">
+      <c r="A899" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B899" t="inlineStr">
@@ -19251,7 +19251,7 @@
       </c>
     </row>
     <row r="900">
-      <c r="A900" s="2" t="n">
+      <c r="A900" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B900" t="inlineStr">
@@ -19266,6 +19266,615 @@
         <v>48</v>
       </c>
       <c r="E900" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C901" t="n">
+        <v>29.64999961853027</v>
+      </c>
+      <c r="D901" t="n">
+        <v>28</v>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C902" t="n">
+        <v>14.56999969482422</v>
+      </c>
+      <c r="D902" t="n">
+        <v>31</v>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C903" t="n">
+        <v>23.07999992370605</v>
+      </c>
+      <c r="D903" t="n">
+        <v>30</v>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C904" t="n">
+        <v>3.920000076293945</v>
+      </c>
+      <c r="D904" t="n">
+        <v>16</v>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C905" t="n">
+        <v>1.330000042915344</v>
+      </c>
+      <c r="D905" t="n">
+        <v>12</v>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C906" t="n">
+        <v>184.4100036621094</v>
+      </c>
+      <c r="D906" t="n">
+        <v>26</v>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C907" t="n">
+        <v>63.72000122070312</v>
+      </c>
+      <c r="D907" t="n">
+        <v>45</v>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C908" t="n">
+        <v>4.070000171661377</v>
+      </c>
+      <c r="D908" t="n">
+        <v>61</v>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C909" t="n">
+        <v>4.929999828338623</v>
+      </c>
+      <c r="D909" t="n">
+        <v>10</v>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C910" t="n">
+        <v>6.010000228881836</v>
+      </c>
+      <c r="D910" t="n">
+        <v>22</v>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C911" t="n">
+        <v>19.90999984741211</v>
+      </c>
+      <c r="D911" t="n">
+        <v>49</v>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C912" t="n">
+        <v>28.09000015258789</v>
+      </c>
+      <c r="D912" t="n">
+        <v>20</v>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C913" t="n">
+        <v>14.02000045776367</v>
+      </c>
+      <c r="D913" t="n">
+        <v>9</v>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C914" t="n">
+        <v>5.079999923706055</v>
+      </c>
+      <c r="D914" t="n">
+        <v>26</v>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C915" t="n">
+        <v>24.63999938964844</v>
+      </c>
+      <c r="D915" t="n">
+        <v>27</v>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C916" t="n">
+        <v>11.72000026702881</v>
+      </c>
+      <c r="D916" t="n">
+        <v>22</v>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C917" t="n">
+        <v>7.630000114440918</v>
+      </c>
+      <c r="D917" t="n">
+        <v>20</v>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C918" t="n">
+        <v>10.14000034332275</v>
+      </c>
+      <c r="D918" t="n">
+        <v>25</v>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C919" t="n">
+        <v>5.440000057220459</v>
+      </c>
+      <c r="D919" t="n">
+        <v>30</v>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C920" t="n">
+        <v>49.90000152587891</v>
+      </c>
+      <c r="D920" t="n">
+        <v>23</v>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C921" t="n">
+        <v>4.179999828338623</v>
+      </c>
+      <c r="D921" t="n">
+        <v>20</v>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C922" t="n">
+        <v>61.45999908447266</v>
+      </c>
+      <c r="D922" t="n">
+        <v>8</v>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C923" t="n">
+        <v>47.68000030517578</v>
+      </c>
+      <c r="D923" t="n">
+        <v>16</v>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C924" t="n">
+        <v>18.72999954223633</v>
+      </c>
+      <c r="D924" t="n">
+        <v>63</v>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C925" t="n">
+        <v>38.34999847412109</v>
+      </c>
+      <c r="D925" t="n">
+        <v>35</v>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C926" t="n">
+        <v>113.0199966430664</v>
+      </c>
+      <c r="D926" t="n">
+        <v>31</v>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C927" t="n">
+        <v>43.2599983215332</v>
+      </c>
+      <c r="D927" t="n">
+        <v>11</v>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C928" t="n">
+        <v>7.130000114440918</v>
+      </c>
+      <c r="D928" t="n">
+        <v>11</v>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C929" t="n">
+        <v>37.79999923706055</v>
+      </c>
+      <c r="D929" t="n">
+        <v>48</v>
+      </c>
+      <c r="E929" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-02
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E929"/>
+  <dimension ref="A1:E958"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19272,7 +19272,7 @@
       </c>
     </row>
     <row r="901">
-      <c r="A901" s="2" t="n">
+      <c r="A901" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B901" t="inlineStr">
@@ -19293,7 +19293,7 @@
       </c>
     </row>
     <row r="902">
-      <c r="A902" s="2" t="n">
+      <c r="A902" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B902" t="inlineStr">
@@ -19314,7 +19314,7 @@
       </c>
     </row>
     <row r="903">
-      <c r="A903" s="2" t="n">
+      <c r="A903" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B903" t="inlineStr">
@@ -19335,7 +19335,7 @@
       </c>
     </row>
     <row r="904">
-      <c r="A904" s="2" t="n">
+      <c r="A904" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B904" t="inlineStr">
@@ -19356,7 +19356,7 @@
       </c>
     </row>
     <row r="905">
-      <c r="A905" s="2" t="n">
+      <c r="A905" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B905" t="inlineStr">
@@ -19377,7 +19377,7 @@
       </c>
     </row>
     <row r="906">
-      <c r="A906" s="2" t="n">
+      <c r="A906" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B906" t="inlineStr">
@@ -19398,7 +19398,7 @@
       </c>
     </row>
     <row r="907">
-      <c r="A907" s="2" t="n">
+      <c r="A907" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B907" t="inlineStr">
@@ -19419,7 +19419,7 @@
       </c>
     </row>
     <row r="908">
-      <c r="A908" s="2" t="n">
+      <c r="A908" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B908" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
     </row>
     <row r="909">
-      <c r="A909" s="2" t="n">
+      <c r="A909" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B909" t="inlineStr">
@@ -19461,7 +19461,7 @@
       </c>
     </row>
     <row r="910">
-      <c r="A910" s="2" t="n">
+      <c r="A910" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B910" t="inlineStr">
@@ -19482,7 +19482,7 @@
       </c>
     </row>
     <row r="911">
-      <c r="A911" s="2" t="n">
+      <c r="A911" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B911" t="inlineStr">
@@ -19503,7 +19503,7 @@
       </c>
     </row>
     <row r="912">
-      <c r="A912" s="2" t="n">
+      <c r="A912" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B912" t="inlineStr">
@@ -19524,7 +19524,7 @@
       </c>
     </row>
     <row r="913">
-      <c r="A913" s="2" t="n">
+      <c r="A913" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B913" t="inlineStr">
@@ -19545,7 +19545,7 @@
       </c>
     </row>
     <row r="914">
-      <c r="A914" s="2" t="n">
+      <c r="A914" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B914" t="inlineStr">
@@ -19566,7 +19566,7 @@
       </c>
     </row>
     <row r="915">
-      <c r="A915" s="2" t="n">
+      <c r="A915" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B915" t="inlineStr">
@@ -19587,7 +19587,7 @@
       </c>
     </row>
     <row r="916">
-      <c r="A916" s="2" t="n">
+      <c r="A916" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B916" t="inlineStr">
@@ -19608,7 +19608,7 @@
       </c>
     </row>
     <row r="917">
-      <c r="A917" s="2" t="n">
+      <c r="A917" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B917" t="inlineStr">
@@ -19629,7 +19629,7 @@
       </c>
     </row>
     <row r="918">
-      <c r="A918" s="2" t="n">
+      <c r="A918" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B918" t="inlineStr">
@@ -19650,7 +19650,7 @@
       </c>
     </row>
     <row r="919">
-      <c r="A919" s="2" t="n">
+      <c r="A919" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B919" t="inlineStr">
@@ -19671,7 +19671,7 @@
       </c>
     </row>
     <row r="920">
-      <c r="A920" s="2" t="n">
+      <c r="A920" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B920" t="inlineStr">
@@ -19692,7 +19692,7 @@
       </c>
     </row>
     <row r="921">
-      <c r="A921" s="2" t="n">
+      <c r="A921" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B921" t="inlineStr">
@@ -19713,7 +19713,7 @@
       </c>
     </row>
     <row r="922">
-      <c r="A922" s="2" t="n">
+      <c r="A922" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B922" t="inlineStr">
@@ -19734,7 +19734,7 @@
       </c>
     </row>
     <row r="923">
-      <c r="A923" s="2" t="n">
+      <c r="A923" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B923" t="inlineStr">
@@ -19755,7 +19755,7 @@
       </c>
     </row>
     <row r="924">
-      <c r="A924" s="2" t="n">
+      <c r="A924" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B924" t="inlineStr">
@@ -19776,7 +19776,7 @@
       </c>
     </row>
     <row r="925">
-      <c r="A925" s="2" t="n">
+      <c r="A925" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B925" t="inlineStr">
@@ -19797,7 +19797,7 @@
       </c>
     </row>
     <row r="926">
-      <c r="A926" s="2" t="n">
+      <c r="A926" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B926" t="inlineStr">
@@ -19818,7 +19818,7 @@
       </c>
     </row>
     <row r="927">
-      <c r="A927" s="2" t="n">
+      <c r="A927" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B927" t="inlineStr">
@@ -19839,7 +19839,7 @@
       </c>
     </row>
     <row r="928">
-      <c r="A928" s="2" t="n">
+      <c r="A928" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B928" t="inlineStr">
@@ -19860,7 +19860,7 @@
       </c>
     </row>
     <row r="929">
-      <c r="A929" s="2" t="n">
+      <c r="A929" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B929" t="inlineStr">
@@ -19875,6 +19875,615 @@
         <v>48</v>
       </c>
       <c r="E929" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C930" t="n">
+        <v>30.46999931335449</v>
+      </c>
+      <c r="D930" t="n">
+        <v>28</v>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C931" t="n">
+        <v>15.28999996185303</v>
+      </c>
+      <c r="D931" t="n">
+        <v>31</v>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C932" t="n">
+        <v>23.71999931335449</v>
+      </c>
+      <c r="D932" t="n">
+        <v>30</v>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C933" t="n">
+        <v>3.880000114440918</v>
+      </c>
+      <c r="D933" t="n">
+        <v>16</v>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C934" t="n">
+        <v>1.389999985694885</v>
+      </c>
+      <c r="D934" t="n">
+        <v>12</v>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C935" t="n">
+        <v>189.0700073242188</v>
+      </c>
+      <c r="D935" t="n">
+        <v>26</v>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C936" t="n">
+        <v>65.73999786376953</v>
+      </c>
+      <c r="D936" t="n">
+        <v>45</v>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C937" t="n">
+        <v>4.03000020980835</v>
+      </c>
+      <c r="D937" t="n">
+        <v>61</v>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C938" t="n">
+        <v>4.989999771118164</v>
+      </c>
+      <c r="D938" t="n">
+        <v>10</v>
+      </c>
+      <c r="E938" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C939" t="n">
+        <v>6.190000057220459</v>
+      </c>
+      <c r="D939" t="n">
+        <v>22</v>
+      </c>
+      <c r="E939" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C940" t="n">
+        <v>20.51000022888184</v>
+      </c>
+      <c r="D940" t="n">
+        <v>49</v>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C941" t="n">
+        <v>28.70000076293945</v>
+      </c>
+      <c r="D941" t="n">
+        <v>20</v>
+      </c>
+      <c r="E941" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C942" t="n">
+        <v>14.60999965667725</v>
+      </c>
+      <c r="D942" t="n">
+        <v>9</v>
+      </c>
+      <c r="E942" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C943" t="n">
+        <v>4.96999979019165</v>
+      </c>
+      <c r="D943" t="n">
+        <v>26</v>
+      </c>
+      <c r="E943" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C944" t="n">
+        <v>25.11000061035156</v>
+      </c>
+      <c r="D944" t="n">
+        <v>27</v>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C945" t="n">
+        <v>12.05000019073486</v>
+      </c>
+      <c r="D945" t="n">
+        <v>22</v>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C946" t="n">
+        <v>7.619999885559082</v>
+      </c>
+      <c r="D946" t="n">
+        <v>20</v>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C947" t="n">
+        <v>10.85000038146973</v>
+      </c>
+      <c r="D947" t="n">
+        <v>25</v>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C948" t="n">
+        <v>5.610000133514404</v>
+      </c>
+      <c r="D948" t="n">
+        <v>30</v>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C949" t="n">
+        <v>51.15000152587891</v>
+      </c>
+      <c r="D949" t="n">
+        <v>23</v>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C950" t="n">
+        <v>4.320000171661377</v>
+      </c>
+      <c r="D950" t="n">
+        <v>20</v>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C951" t="n">
+        <v>63.04000091552734</v>
+      </c>
+      <c r="D951" t="n">
+        <v>8</v>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C952" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="D952" t="n">
+        <v>16</v>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C953" t="n">
+        <v>19</v>
+      </c>
+      <c r="D953" t="n">
+        <v>63</v>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C954" t="n">
+        <v>39.79000091552734</v>
+      </c>
+      <c r="D954" t="n">
+        <v>35</v>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C955" t="n">
+        <v>116.120002746582</v>
+      </c>
+      <c r="D955" t="n">
+        <v>31</v>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C956" t="n">
+        <v>44.27999877929688</v>
+      </c>
+      <c r="D956" t="n">
+        <v>11</v>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C957" t="n">
+        <v>7.460000038146973</v>
+      </c>
+      <c r="D957" t="n">
+        <v>11</v>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C958" t="n">
+        <v>37.91999816894531</v>
+      </c>
+      <c r="D958" t="n">
+        <v>48</v>
+      </c>
+      <c r="E958" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-05
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E958"/>
+  <dimension ref="A1:E987"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19881,7 +19881,7 @@
       </c>
     </row>
     <row r="930">
-      <c r="A930" s="2" t="n">
+      <c r="A930" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B930" t="inlineStr">
@@ -19902,7 +19902,7 @@
       </c>
     </row>
     <row r="931">
-      <c r="A931" s="2" t="n">
+      <c r="A931" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B931" t="inlineStr">
@@ -19923,7 +19923,7 @@
       </c>
     </row>
     <row r="932">
-      <c r="A932" s="2" t="n">
+      <c r="A932" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B932" t="inlineStr">
@@ -19944,7 +19944,7 @@
       </c>
     </row>
     <row r="933">
-      <c r="A933" s="2" t="n">
+      <c r="A933" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B933" t="inlineStr">
@@ -19965,7 +19965,7 @@
       </c>
     </row>
     <row r="934">
-      <c r="A934" s="2" t="n">
+      <c r="A934" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B934" t="inlineStr">
@@ -19986,7 +19986,7 @@
       </c>
     </row>
     <row r="935">
-      <c r="A935" s="2" t="n">
+      <c r="A935" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B935" t="inlineStr">
@@ -20007,7 +20007,7 @@
       </c>
     </row>
     <row r="936">
-      <c r="A936" s="2" t="n">
+      <c r="A936" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B936" t="inlineStr">
@@ -20028,7 +20028,7 @@
       </c>
     </row>
     <row r="937">
-      <c r="A937" s="2" t="n">
+      <c r="A937" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B937" t="inlineStr">
@@ -20049,7 +20049,7 @@
       </c>
     </row>
     <row r="938">
-      <c r="A938" s="2" t="n">
+      <c r="A938" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B938" t="inlineStr">
@@ -20070,7 +20070,7 @@
       </c>
     </row>
     <row r="939">
-      <c r="A939" s="2" t="n">
+      <c r="A939" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B939" t="inlineStr">
@@ -20091,7 +20091,7 @@
       </c>
     </row>
     <row r="940">
-      <c r="A940" s="2" t="n">
+      <c r="A940" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B940" t="inlineStr">
@@ -20112,7 +20112,7 @@
       </c>
     </row>
     <row r="941">
-      <c r="A941" s="2" t="n">
+      <c r="A941" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B941" t="inlineStr">
@@ -20133,7 +20133,7 @@
       </c>
     </row>
     <row r="942">
-      <c r="A942" s="2" t="n">
+      <c r="A942" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B942" t="inlineStr">
@@ -20154,7 +20154,7 @@
       </c>
     </row>
     <row r="943">
-      <c r="A943" s="2" t="n">
+      <c r="A943" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B943" t="inlineStr">
@@ -20175,7 +20175,7 @@
       </c>
     </row>
     <row r="944">
-      <c r="A944" s="2" t="n">
+      <c r="A944" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B944" t="inlineStr">
@@ -20196,7 +20196,7 @@
       </c>
     </row>
     <row r="945">
-      <c r="A945" s="2" t="n">
+      <c r="A945" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B945" t="inlineStr">
@@ -20217,7 +20217,7 @@
       </c>
     </row>
     <row r="946">
-      <c r="A946" s="2" t="n">
+      <c r="A946" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B946" t="inlineStr">
@@ -20238,7 +20238,7 @@
       </c>
     </row>
     <row r="947">
-      <c r="A947" s="2" t="n">
+      <c r="A947" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B947" t="inlineStr">
@@ -20259,7 +20259,7 @@
       </c>
     </row>
     <row r="948">
-      <c r="A948" s="2" t="n">
+      <c r="A948" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B948" t="inlineStr">
@@ -20280,7 +20280,7 @@
       </c>
     </row>
     <row r="949">
-      <c r="A949" s="2" t="n">
+      <c r="A949" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B949" t="inlineStr">
@@ -20301,7 +20301,7 @@
       </c>
     </row>
     <row r="950">
-      <c r="A950" s="2" t="n">
+      <c r="A950" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B950" t="inlineStr">
@@ -20322,7 +20322,7 @@
       </c>
     </row>
     <row r="951">
-      <c r="A951" s="2" t="n">
+      <c r="A951" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B951" t="inlineStr">
@@ -20343,7 +20343,7 @@
       </c>
     </row>
     <row r="952">
-      <c r="A952" s="2" t="n">
+      <c r="A952" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B952" t="inlineStr">
@@ -20364,7 +20364,7 @@
       </c>
     </row>
     <row r="953">
-      <c r="A953" s="2" t="n">
+      <c r="A953" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B953" t="inlineStr">
@@ -20385,7 +20385,7 @@
       </c>
     </row>
     <row r="954">
-      <c r="A954" s="2" t="n">
+      <c r="A954" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B954" t="inlineStr">
@@ -20406,7 +20406,7 @@
       </c>
     </row>
     <row r="955">
-      <c r="A955" s="2" t="n">
+      <c r="A955" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B955" t="inlineStr">
@@ -20427,7 +20427,7 @@
       </c>
     </row>
     <row r="956">
-      <c r="A956" s="2" t="n">
+      <c r="A956" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B956" t="inlineStr">
@@ -20448,7 +20448,7 @@
       </c>
     </row>
     <row r="957">
-      <c r="A957" s="2" t="n">
+      <c r="A957" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B957" t="inlineStr">
@@ -20469,7 +20469,7 @@
       </c>
     </row>
     <row r="958">
-      <c r="A958" s="2" t="n">
+      <c r="A958" s="1" t="n">
         <v>46297</v>
       </c>
       <c r="B958" t="inlineStr">
@@ -20484,6 +20484,615 @@
         <v>48</v>
       </c>
       <c r="E958" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C959" t="n">
+        <v>33.18999862670898</v>
+      </c>
+      <c r="D959" t="n">
+        <v>28</v>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C960" t="n">
+        <v>15.88000011444092</v>
+      </c>
+      <c r="D960" t="n">
+        <v>31</v>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C961" t="n">
+        <v>26.44000053405762</v>
+      </c>
+      <c r="D961" t="n">
+        <v>30</v>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C962" t="n">
+        <v>4.190000057220459</v>
+      </c>
+      <c r="D962" t="n">
+        <v>16</v>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C963" t="n">
+        <v>1.429999947547913</v>
+      </c>
+      <c r="D963" t="n">
+        <v>12</v>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C964" t="n">
+        <v>204.3600006103516</v>
+      </c>
+      <c r="D964" t="n">
+        <v>26</v>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C965" t="n">
+        <v>80.73000335693359</v>
+      </c>
+      <c r="D965" t="n">
+        <v>45</v>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C966" t="n">
+        <v>4.119999885559082</v>
+      </c>
+      <c r="D966" t="n">
+        <v>61</v>
+      </c>
+      <c r="E966" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C967" t="n">
+        <v>5.039999961853027</v>
+      </c>
+      <c r="D967" t="n">
+        <v>10</v>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C968" t="n">
+        <v>6.420000076293945</v>
+      </c>
+      <c r="D968" t="n">
+        <v>22</v>
+      </c>
+      <c r="E968" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C969" t="n">
+        <v>20.77000045776367</v>
+      </c>
+      <c r="D969" t="n">
+        <v>49</v>
+      </c>
+      <c r="E969" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C970" t="n">
+        <v>30.29000091552734</v>
+      </c>
+      <c r="D970" t="n">
+        <v>20</v>
+      </c>
+      <c r="E970" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C971" t="n">
+        <v>17.20000076293945</v>
+      </c>
+      <c r="D971" t="n">
+        <v>9</v>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C972" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D972" t="n">
+        <v>26</v>
+      </c>
+      <c r="E972" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C973" t="n">
+        <v>27.15999984741211</v>
+      </c>
+      <c r="D973" t="n">
+        <v>27</v>
+      </c>
+      <c r="E973" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C974" t="n">
+        <v>12.85000038146973</v>
+      </c>
+      <c r="D974" t="n">
+        <v>22</v>
+      </c>
+      <c r="E974" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C975" t="n">
+        <v>9.409999847412109</v>
+      </c>
+      <c r="D975" t="n">
+        <v>20</v>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C976" t="n">
+        <v>13.59000015258789</v>
+      </c>
+      <c r="D976" t="n">
+        <v>25</v>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C977" t="n">
+        <v>6.28000020980835</v>
+      </c>
+      <c r="D977" t="n">
+        <v>30</v>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C978" t="n">
+        <v>55.31000137329102</v>
+      </c>
+      <c r="D978" t="n">
+        <v>23</v>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C979" t="n">
+        <v>4.699999809265137</v>
+      </c>
+      <c r="D979" t="n">
+        <v>20</v>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C980" t="n">
+        <v>64.05000305175781</v>
+      </c>
+      <c r="D980" t="n">
+        <v>8</v>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C981" t="n">
+        <v>51.68999862670898</v>
+      </c>
+      <c r="D981" t="n">
+        <v>16</v>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C982" t="n">
+        <v>21.04999923706055</v>
+      </c>
+      <c r="D982" t="n">
+        <v>63</v>
+      </c>
+      <c r="E982" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C983" t="n">
+        <v>43.86999893188477</v>
+      </c>
+      <c r="D983" t="n">
+        <v>35</v>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C984" t="n">
+        <v>126.9400024414062</v>
+      </c>
+      <c r="D984" t="n">
+        <v>31</v>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C985" t="n">
+        <v>41.9900016784668</v>
+      </c>
+      <c r="D985" t="n">
+        <v>11</v>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C986" t="n">
+        <v>7.460000038146973</v>
+      </c>
+      <c r="D986" t="n">
+        <v>11</v>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C987" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="D987" t="n">
+        <v>48</v>
+      </c>
+      <c r="E987" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-06
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E987"/>
+  <dimension ref="A1:E1016"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20490,7 +20490,7 @@
       </c>
     </row>
     <row r="959">
-      <c r="A959" s="2" t="n">
+      <c r="A959" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B959" t="inlineStr">
@@ -20511,7 +20511,7 @@
       </c>
     </row>
     <row r="960">
-      <c r="A960" s="2" t="n">
+      <c r="A960" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B960" t="inlineStr">
@@ -20532,7 +20532,7 @@
       </c>
     </row>
     <row r="961">
-      <c r="A961" s="2" t="n">
+      <c r="A961" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B961" t="inlineStr">
@@ -20553,7 +20553,7 @@
       </c>
     </row>
     <row r="962">
-      <c r="A962" s="2" t="n">
+      <c r="A962" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B962" t="inlineStr">
@@ -20574,7 +20574,7 @@
       </c>
     </row>
     <row r="963">
-      <c r="A963" s="2" t="n">
+      <c r="A963" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B963" t="inlineStr">
@@ -20595,7 +20595,7 @@
       </c>
     </row>
     <row r="964">
-      <c r="A964" s="2" t="n">
+      <c r="A964" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B964" t="inlineStr">
@@ -20616,7 +20616,7 @@
       </c>
     </row>
     <row r="965">
-      <c r="A965" s="2" t="n">
+      <c r="A965" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B965" t="inlineStr">
@@ -20637,7 +20637,7 @@
       </c>
     </row>
     <row r="966">
-      <c r="A966" s="2" t="n">
+      <c r="A966" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B966" t="inlineStr">
@@ -20658,7 +20658,7 @@
       </c>
     </row>
     <row r="967">
-      <c r="A967" s="2" t="n">
+      <c r="A967" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B967" t="inlineStr">
@@ -20679,7 +20679,7 @@
       </c>
     </row>
     <row r="968">
-      <c r="A968" s="2" t="n">
+      <c r="A968" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B968" t="inlineStr">
@@ -20700,7 +20700,7 @@
       </c>
     </row>
     <row r="969">
-      <c r="A969" s="2" t="n">
+      <c r="A969" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B969" t="inlineStr">
@@ -20721,7 +20721,7 @@
       </c>
     </row>
     <row r="970">
-      <c r="A970" s="2" t="n">
+      <c r="A970" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B970" t="inlineStr">
@@ -20742,7 +20742,7 @@
       </c>
     </row>
     <row r="971">
-      <c r="A971" s="2" t="n">
+      <c r="A971" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B971" t="inlineStr">
@@ -20763,7 +20763,7 @@
       </c>
     </row>
     <row r="972">
-      <c r="A972" s="2" t="n">
+      <c r="A972" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B972" t="inlineStr">
@@ -20784,7 +20784,7 @@
       </c>
     </row>
     <row r="973">
-      <c r="A973" s="2" t="n">
+      <c r="A973" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B973" t="inlineStr">
@@ -20805,7 +20805,7 @@
       </c>
     </row>
     <row r="974">
-      <c r="A974" s="2" t="n">
+      <c r="A974" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B974" t="inlineStr">
@@ -20826,7 +20826,7 @@
       </c>
     </row>
     <row r="975">
-      <c r="A975" s="2" t="n">
+      <c r="A975" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B975" t="inlineStr">
@@ -20847,7 +20847,7 @@
       </c>
     </row>
     <row r="976">
-      <c r="A976" s="2" t="n">
+      <c r="A976" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B976" t="inlineStr">
@@ -20868,7 +20868,7 @@
       </c>
     </row>
     <row r="977">
-      <c r="A977" s="2" t="n">
+      <c r="A977" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B977" t="inlineStr">
@@ -20889,7 +20889,7 @@
       </c>
     </row>
     <row r="978">
-      <c r="A978" s="2" t="n">
+      <c r="A978" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B978" t="inlineStr">
@@ -20910,7 +20910,7 @@
       </c>
     </row>
     <row r="979">
-      <c r="A979" s="2" t="n">
+      <c r="A979" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B979" t="inlineStr">
@@ -20931,7 +20931,7 @@
       </c>
     </row>
     <row r="980">
-      <c r="A980" s="2" t="n">
+      <c r="A980" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B980" t="inlineStr">
@@ -20952,7 +20952,7 @@
       </c>
     </row>
     <row r="981">
-      <c r="A981" s="2" t="n">
+      <c r="A981" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B981" t="inlineStr">
@@ -20973,7 +20973,7 @@
       </c>
     </row>
     <row r="982">
-      <c r="A982" s="2" t="n">
+      <c r="A982" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B982" t="inlineStr">
@@ -20994,7 +20994,7 @@
       </c>
     </row>
     <row r="983">
-      <c r="A983" s="2" t="n">
+      <c r="A983" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B983" t="inlineStr">
@@ -21015,7 +21015,7 @@
       </c>
     </row>
     <row r="984">
-      <c r="A984" s="2" t="n">
+      <c r="A984" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B984" t="inlineStr">
@@ -21036,7 +21036,7 @@
       </c>
     </row>
     <row r="985">
-      <c r="A985" s="2" t="n">
+      <c r="A985" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B985" t="inlineStr">
@@ -21057,7 +21057,7 @@
       </c>
     </row>
     <row r="986">
-      <c r="A986" s="2" t="n">
+      <c r="A986" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B986" t="inlineStr">
@@ -21078,7 +21078,7 @@
       </c>
     </row>
     <row r="987">
-      <c r="A987" s="2" t="n">
+      <c r="A987" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="B987" t="inlineStr">
@@ -21093,6 +21093,615 @@
         <v>48</v>
       </c>
       <c r="E987" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C988" t="n">
+        <v>34.31999969482422</v>
+      </c>
+      <c r="D988" t="n">
+        <v>28</v>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C989" t="n">
+        <v>15.94999980926514</v>
+      </c>
+      <c r="D989" t="n">
+        <v>31</v>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C990" t="n">
+        <v>24.60000038146973</v>
+      </c>
+      <c r="D990" t="n">
+        <v>30</v>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C991" t="n">
+        <v>4.46999979019165</v>
+      </c>
+      <c r="D991" t="n">
+        <v>16</v>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C992" t="n">
+        <v>1.440000057220459</v>
+      </c>
+      <c r="D992" t="n">
+        <v>12</v>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C993" t="n">
+        <v>202.6600036621094</v>
+      </c>
+      <c r="D993" t="n">
+        <v>26</v>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C994" t="n">
+        <v>78.29000091552734</v>
+      </c>
+      <c r="D994" t="n">
+        <v>45</v>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C995" t="n">
+        <v>4.150000095367432</v>
+      </c>
+      <c r="D995" t="n">
+        <v>61</v>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C996" t="n">
+        <v>4.949999809265137</v>
+      </c>
+      <c r="D996" t="n">
+        <v>10</v>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C997" t="n">
+        <v>6.369999885559082</v>
+      </c>
+      <c r="D997" t="n">
+        <v>22</v>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C998" t="n">
+        <v>20.69000053405762</v>
+      </c>
+      <c r="D998" t="n">
+        <v>49</v>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C999" t="n">
+        <v>30.1200008392334</v>
+      </c>
+      <c r="D999" t="n">
+        <v>20</v>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1000" t="n">
+        <v>17.60000038146973</v>
+      </c>
+      <c r="D1000" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1001" t="n">
+        <v>5.230000019073486</v>
+      </c>
+      <c r="D1001" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1002" t="n">
+        <v>26.97999954223633</v>
+      </c>
+      <c r="D1002" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1003" t="n">
+        <v>12.97999954223633</v>
+      </c>
+      <c r="D1003" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1004" t="n">
+        <v>9.210000038146973</v>
+      </c>
+      <c r="D1004" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1005" t="n">
+        <v>14.55000019073486</v>
+      </c>
+      <c r="D1005" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1006" t="n">
+        <v>6.329999923706055</v>
+      </c>
+      <c r="D1006" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1007" t="n">
+        <v>53.86999893188477</v>
+      </c>
+      <c r="D1007" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1008" t="n">
+        <v>4.710000038146973</v>
+      </c>
+      <c r="D1008" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1009" t="n">
+        <v>62.04000091552734</v>
+      </c>
+      <c r="D1009" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1010" t="n">
+        <v>52.68999862670898</v>
+      </c>
+      <c r="D1010" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1011" t="n">
+        <v>21.29999923706055</v>
+      </c>
+      <c r="D1011" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1012" t="n">
+        <v>44.84000015258789</v>
+      </c>
+      <c r="D1012" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1013" t="n">
+        <v>129.0899963378906</v>
+      </c>
+      <c r="D1013" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1014" t="n">
+        <v>41.65000152587891</v>
+      </c>
+      <c r="D1014" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1015" t="n">
+        <v>7.289999961853027</v>
+      </c>
+      <c r="D1015" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1016" t="n">
+        <v>37.70000076293945</v>
+      </c>
+      <c r="D1016" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1016" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-07
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1016"/>
+  <dimension ref="A1:E1045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21099,7 +21099,7 @@
       </c>
     </row>
     <row r="988">
-      <c r="A988" s="2" t="n">
+      <c r="A988" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B988" t="inlineStr">
@@ -21120,7 +21120,7 @@
       </c>
     </row>
     <row r="989">
-      <c r="A989" s="2" t="n">
+      <c r="A989" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B989" t="inlineStr">
@@ -21141,7 +21141,7 @@
       </c>
     </row>
     <row r="990">
-      <c r="A990" s="2" t="n">
+      <c r="A990" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B990" t="inlineStr">
@@ -21162,7 +21162,7 @@
       </c>
     </row>
     <row r="991">
-      <c r="A991" s="2" t="n">
+      <c r="A991" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B991" t="inlineStr">
@@ -21183,7 +21183,7 @@
       </c>
     </row>
     <row r="992">
-      <c r="A992" s="2" t="n">
+      <c r="A992" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B992" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
     </row>
     <row r="993">
-      <c r="A993" s="2" t="n">
+      <c r="A993" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B993" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
     </row>
     <row r="994">
-      <c r="A994" s="2" t="n">
+      <c r="A994" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B994" t="inlineStr">
@@ -21246,7 +21246,7 @@
       </c>
     </row>
     <row r="995">
-      <c r="A995" s="2" t="n">
+      <c r="A995" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B995" t="inlineStr">
@@ -21267,7 +21267,7 @@
       </c>
     </row>
     <row r="996">
-      <c r="A996" s="2" t="n">
+      <c r="A996" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B996" t="inlineStr">
@@ -21288,7 +21288,7 @@
       </c>
     </row>
     <row r="997">
-      <c r="A997" s="2" t="n">
+      <c r="A997" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B997" t="inlineStr">
@@ -21309,7 +21309,7 @@
       </c>
     </row>
     <row r="998">
-      <c r="A998" s="2" t="n">
+      <c r="A998" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B998" t="inlineStr">
@@ -21330,7 +21330,7 @@
       </c>
     </row>
     <row r="999">
-      <c r="A999" s="2" t="n">
+      <c r="A999" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B999" t="inlineStr">
@@ -21351,7 +21351,7 @@
       </c>
     </row>
     <row r="1000">
-      <c r="A1000" s="2" t="n">
+      <c r="A1000" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1000" t="inlineStr">
@@ -21372,7 +21372,7 @@
       </c>
     </row>
     <row r="1001">
-      <c r="A1001" s="2" t="n">
+      <c r="A1001" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1001" t="inlineStr">
@@ -21393,7 +21393,7 @@
       </c>
     </row>
     <row r="1002">
-      <c r="A1002" s="2" t="n">
+      <c r="A1002" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1002" t="inlineStr">
@@ -21414,7 +21414,7 @@
       </c>
     </row>
     <row r="1003">
-      <c r="A1003" s="2" t="n">
+      <c r="A1003" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1003" t="inlineStr">
@@ -21435,7 +21435,7 @@
       </c>
     </row>
     <row r="1004">
-      <c r="A1004" s="2" t="n">
+      <c r="A1004" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1004" t="inlineStr">
@@ -21456,7 +21456,7 @@
       </c>
     </row>
     <row r="1005">
-      <c r="A1005" s="2" t="n">
+      <c r="A1005" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1005" t="inlineStr">
@@ -21477,7 +21477,7 @@
       </c>
     </row>
     <row r="1006">
-      <c r="A1006" s="2" t="n">
+      <c r="A1006" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1006" t="inlineStr">
@@ -21498,7 +21498,7 @@
       </c>
     </row>
     <row r="1007">
-      <c r="A1007" s="2" t="n">
+      <c r="A1007" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1007" t="inlineStr">
@@ -21519,7 +21519,7 @@
       </c>
     </row>
     <row r="1008">
-      <c r="A1008" s="2" t="n">
+      <c r="A1008" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1008" t="inlineStr">
@@ -21540,7 +21540,7 @@
       </c>
     </row>
     <row r="1009">
-      <c r="A1009" s="2" t="n">
+      <c r="A1009" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1009" t="inlineStr">
@@ -21561,7 +21561,7 @@
       </c>
     </row>
     <row r="1010">
-      <c r="A1010" s="2" t="n">
+      <c r="A1010" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1010" t="inlineStr">
@@ -21582,7 +21582,7 @@
       </c>
     </row>
     <row r="1011">
-      <c r="A1011" s="2" t="n">
+      <c r="A1011" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1011" t="inlineStr">
@@ -21603,7 +21603,7 @@
       </c>
     </row>
     <row r="1012">
-      <c r="A1012" s="2" t="n">
+      <c r="A1012" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1012" t="inlineStr">
@@ -21624,7 +21624,7 @@
       </c>
     </row>
     <row r="1013">
-      <c r="A1013" s="2" t="n">
+      <c r="A1013" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1013" t="inlineStr">
@@ -21645,7 +21645,7 @@
       </c>
     </row>
     <row r="1014">
-      <c r="A1014" s="2" t="n">
+      <c r="A1014" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1014" t="inlineStr">
@@ -21666,7 +21666,7 @@
       </c>
     </row>
     <row r="1015">
-      <c r="A1015" s="2" t="n">
+      <c r="A1015" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1015" t="inlineStr">
@@ -21687,7 +21687,7 @@
       </c>
     </row>
     <row r="1016">
-      <c r="A1016" s="2" t="n">
+      <c r="A1016" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="B1016" t="inlineStr">
@@ -21702,6 +21702,615 @@
         <v>48</v>
       </c>
       <c r="E1016" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1017" t="n">
+        <v>34.58000183105469</v>
+      </c>
+      <c r="D1017" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1018" t="n">
+        <v>15.39999961853027</v>
+      </c>
+      <c r="D1018" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1019" t="n">
+        <v>24.18000030517578</v>
+      </c>
+      <c r="D1019" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1020" t="n">
+        <v>4.619999885559082</v>
+      </c>
+      <c r="D1020" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1021" t="n">
+        <v>1.440000057220459</v>
+      </c>
+      <c r="D1021" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1022" t="n">
+        <v>201.3000030517578</v>
+      </c>
+      <c r="D1022" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1023" t="n">
+        <v>76.62000274658203</v>
+      </c>
+      <c r="D1023" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1024" t="n">
+        <v>4.260000228881836</v>
+      </c>
+      <c r="D1024" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1025" t="n">
+        <v>4.980000019073486</v>
+      </c>
+      <c r="D1025" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1026" t="n">
+        <v>6.389999866485596</v>
+      </c>
+      <c r="D1026" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1026" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1027" t="n">
+        <v>20.97999954223633</v>
+      </c>
+      <c r="D1027" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1028" t="n">
+        <v>30.35000038146973</v>
+      </c>
+      <c r="D1028" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1028" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1029" t="n">
+        <v>18.02000045776367</v>
+      </c>
+      <c r="D1029" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1029" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1030" t="n">
+        <v>5.159999847412109</v>
+      </c>
+      <c r="D1030" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1030" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1031" t="n">
+        <v>27.19000053405762</v>
+      </c>
+      <c r="D1031" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1032" t="n">
+        <v>12.80000019073486</v>
+      </c>
+      <c r="D1032" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1033" t="n">
+        <v>9.680000305175781</v>
+      </c>
+      <c r="D1033" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1034" t="n">
+        <v>14.90999984741211</v>
+      </c>
+      <c r="D1034" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1035" t="n">
+        <v>6.389999866485596</v>
+      </c>
+      <c r="D1035" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1036" t="n">
+        <v>54.47999954223633</v>
+      </c>
+      <c r="D1036" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1037" t="n">
+        <v>4.760000228881836</v>
+      </c>
+      <c r="D1037" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1038" t="n">
+        <v>62.95999908447266</v>
+      </c>
+      <c r="D1038" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1039" t="n">
+        <v>52.90000152587891</v>
+      </c>
+      <c r="D1039" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1040" t="n">
+        <v>21.07999992370605</v>
+      </c>
+      <c r="D1040" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1041" t="n">
+        <v>44.38999938964844</v>
+      </c>
+      <c r="D1041" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1042" t="n">
+        <v>130.5200042724609</v>
+      </c>
+      <c r="D1042" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1043" t="n">
+        <v>42.18000030517578</v>
+      </c>
+      <c r="D1043" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1044" t="n">
+        <v>7.230000019073486</v>
+      </c>
+      <c r="D1044" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1045" t="n">
+        <v>37.5099983215332</v>
+      </c>
+      <c r="D1045" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1045" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-08
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1045"/>
+  <dimension ref="A1:E1074"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21708,7 +21708,7 @@
       </c>
     </row>
     <row r="1017">
-      <c r="A1017" s="2" t="n">
+      <c r="A1017" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1017" t="inlineStr">
@@ -21729,7 +21729,7 @@
       </c>
     </row>
     <row r="1018">
-      <c r="A1018" s="2" t="n">
+      <c r="A1018" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1018" t="inlineStr">
@@ -21750,7 +21750,7 @@
       </c>
     </row>
     <row r="1019">
-      <c r="A1019" s="2" t="n">
+      <c r="A1019" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1019" t="inlineStr">
@@ -21771,7 +21771,7 @@
       </c>
     </row>
     <row r="1020">
-      <c r="A1020" s="2" t="n">
+      <c r="A1020" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1020" t="inlineStr">
@@ -21792,7 +21792,7 @@
       </c>
     </row>
     <row r="1021">
-      <c r="A1021" s="2" t="n">
+      <c r="A1021" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1021" t="inlineStr">
@@ -21813,7 +21813,7 @@
       </c>
     </row>
     <row r="1022">
-      <c r="A1022" s="2" t="n">
+      <c r="A1022" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1022" t="inlineStr">
@@ -21834,7 +21834,7 @@
       </c>
     </row>
     <row r="1023">
-      <c r="A1023" s="2" t="n">
+      <c r="A1023" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1023" t="inlineStr">
@@ -21855,7 +21855,7 @@
       </c>
     </row>
     <row r="1024">
-      <c r="A1024" s="2" t="n">
+      <c r="A1024" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1024" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
     </row>
     <row r="1025">
-      <c r="A1025" s="2" t="n">
+      <c r="A1025" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1025" t="inlineStr">
@@ -21897,7 +21897,7 @@
       </c>
     </row>
     <row r="1026">
-      <c r="A1026" s="2" t="n">
+      <c r="A1026" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1026" t="inlineStr">
@@ -21918,7 +21918,7 @@
       </c>
     </row>
     <row r="1027">
-      <c r="A1027" s="2" t="n">
+      <c r="A1027" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1027" t="inlineStr">
@@ -21939,7 +21939,7 @@
       </c>
     </row>
     <row r="1028">
-      <c r="A1028" s="2" t="n">
+      <c r="A1028" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1028" t="inlineStr">
@@ -21960,7 +21960,7 @@
       </c>
     </row>
     <row r="1029">
-      <c r="A1029" s="2" t="n">
+      <c r="A1029" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1029" t="inlineStr">
@@ -21981,7 +21981,7 @@
       </c>
     </row>
     <row r="1030">
-      <c r="A1030" s="2" t="n">
+      <c r="A1030" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1030" t="inlineStr">
@@ -22002,7 +22002,7 @@
       </c>
     </row>
     <row r="1031">
-      <c r="A1031" s="2" t="n">
+      <c r="A1031" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1031" t="inlineStr">
@@ -22023,7 +22023,7 @@
       </c>
     </row>
     <row r="1032">
-      <c r="A1032" s="2" t="n">
+      <c r="A1032" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1032" t="inlineStr">
@@ -22044,7 +22044,7 @@
       </c>
     </row>
     <row r="1033">
-      <c r="A1033" s="2" t="n">
+      <c r="A1033" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1033" t="inlineStr">
@@ -22065,7 +22065,7 @@
       </c>
     </row>
     <row r="1034">
-      <c r="A1034" s="2" t="n">
+      <c r="A1034" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1034" t="inlineStr">
@@ -22086,7 +22086,7 @@
       </c>
     </row>
     <row r="1035">
-      <c r="A1035" s="2" t="n">
+      <c r="A1035" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1035" t="inlineStr">
@@ -22107,7 +22107,7 @@
       </c>
     </row>
     <row r="1036">
-      <c r="A1036" s="2" t="n">
+      <c r="A1036" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1036" t="inlineStr">
@@ -22128,7 +22128,7 @@
       </c>
     </row>
     <row r="1037">
-      <c r="A1037" s="2" t="n">
+      <c r="A1037" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1037" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
     </row>
     <row r="1038">
-      <c r="A1038" s="2" t="n">
+      <c r="A1038" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1038" t="inlineStr">
@@ -22170,7 +22170,7 @@
       </c>
     </row>
     <row r="1039">
-      <c r="A1039" s="2" t="n">
+      <c r="A1039" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1039" t="inlineStr">
@@ -22191,7 +22191,7 @@
       </c>
     </row>
     <row r="1040">
-      <c r="A1040" s="2" t="n">
+      <c r="A1040" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1040" t="inlineStr">
@@ -22212,7 +22212,7 @@
       </c>
     </row>
     <row r="1041">
-      <c r="A1041" s="2" t="n">
+      <c r="A1041" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1041" t="inlineStr">
@@ -22233,7 +22233,7 @@
       </c>
     </row>
     <row r="1042">
-      <c r="A1042" s="2" t="n">
+      <c r="A1042" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1042" t="inlineStr">
@@ -22254,7 +22254,7 @@
       </c>
     </row>
     <row r="1043">
-      <c r="A1043" s="2" t="n">
+      <c r="A1043" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1043" t="inlineStr">
@@ -22275,7 +22275,7 @@
       </c>
     </row>
     <row r="1044">
-      <c r="A1044" s="2" t="n">
+      <c r="A1044" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1044" t="inlineStr">
@@ -22296,7 +22296,7 @@
       </c>
     </row>
     <row r="1045">
-      <c r="A1045" s="2" t="n">
+      <c r="A1045" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="B1045" t="inlineStr">
@@ -22311,6 +22311,615 @@
         <v>48</v>
       </c>
       <c r="E1045" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1046" t="n">
+        <v>35.18000030517578</v>
+      </c>
+      <c r="D1046" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1047" t="n">
+        <v>15.94999980926514</v>
+      </c>
+      <c r="D1047" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1048" t="n">
+        <v>24.26000022888184</v>
+      </c>
+      <c r="D1048" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1049" t="n">
+        <v>4.449999809265137</v>
+      </c>
+      <c r="D1049" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1050" t="n">
+        <v>1.460000038146973</v>
+      </c>
+      <c r="D1050" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1051" t="n">
+        <v>203.2700042724609</v>
+      </c>
+      <c r="D1051" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1052" t="n">
+        <v>77.36000061035156</v>
+      </c>
+      <c r="D1052" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1053" t="n">
+        <v>4.46999979019165</v>
+      </c>
+      <c r="D1053" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1053" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1054" t="n">
+        <v>5.110000133514404</v>
+      </c>
+      <c r="D1054" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1054" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1055" t="n">
+        <v>6.400000095367432</v>
+      </c>
+      <c r="D1055" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1056" t="n">
+        <v>21.38999938964844</v>
+      </c>
+      <c r="D1056" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1056" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1057" t="n">
+        <v>30.81999969482422</v>
+      </c>
+      <c r="D1057" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1058" t="n">
+        <v>18.36000061035156</v>
+      </c>
+      <c r="D1058" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1058" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1059" t="n">
+        <v>5.570000171661377</v>
+      </c>
+      <c r="D1059" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1059" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1060" t="n">
+        <v>26.77000045776367</v>
+      </c>
+      <c r="D1060" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1060" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1061" t="n">
+        <v>13.35000038146973</v>
+      </c>
+      <c r="D1061" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1062" t="n">
+        <v>10.28999996185303</v>
+      </c>
+      <c r="D1062" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1063" t="n">
+        <v>16.88999938964844</v>
+      </c>
+      <c r="D1063" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1064" t="n">
+        <v>6.460000038146973</v>
+      </c>
+      <c r="D1064" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1065" t="n">
+        <v>55.70000076293945</v>
+      </c>
+      <c r="D1065" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1066" t="n">
+        <v>4.840000152587891</v>
+      </c>
+      <c r="D1066" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1067" t="n">
+        <v>63.79999923706055</v>
+      </c>
+      <c r="D1067" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1068" t="n">
+        <v>53.56999969482422</v>
+      </c>
+      <c r="D1068" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1069" t="n">
+        <v>20.89999961853027</v>
+      </c>
+      <c r="D1069" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1070" t="n">
+        <v>45.56000137329102</v>
+      </c>
+      <c r="D1070" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1071" t="n">
+        <v>133.9400024414062</v>
+      </c>
+      <c r="D1071" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1072" t="n">
+        <v>42.65999984741211</v>
+      </c>
+      <c r="D1072" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1073" t="n">
+        <v>7.210000038146973</v>
+      </c>
+      <c r="D1073" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1074" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="D1074" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1074" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-09
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1074"/>
+  <dimension ref="A1:E1103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22317,7 +22317,7 @@
       </c>
     </row>
     <row r="1046">
-      <c r="A1046" s="2" t="n">
+      <c r="A1046" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1046" t="inlineStr">
@@ -22338,7 +22338,7 @@
       </c>
     </row>
     <row r="1047">
-      <c r="A1047" s="2" t="n">
+      <c r="A1047" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1047" t="inlineStr">
@@ -22359,7 +22359,7 @@
       </c>
     </row>
     <row r="1048">
-      <c r="A1048" s="2" t="n">
+      <c r="A1048" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1048" t="inlineStr">
@@ -22380,7 +22380,7 @@
       </c>
     </row>
     <row r="1049">
-      <c r="A1049" s="2" t="n">
+      <c r="A1049" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1049" t="inlineStr">
@@ -22401,7 +22401,7 @@
       </c>
     </row>
     <row r="1050">
-      <c r="A1050" s="2" t="n">
+      <c r="A1050" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1050" t="inlineStr">
@@ -22422,7 +22422,7 @@
       </c>
     </row>
     <row r="1051">
-      <c r="A1051" s="2" t="n">
+      <c r="A1051" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1051" t="inlineStr">
@@ -22443,7 +22443,7 @@
       </c>
     </row>
     <row r="1052">
-      <c r="A1052" s="2" t="n">
+      <c r="A1052" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1052" t="inlineStr">
@@ -22464,7 +22464,7 @@
       </c>
     </row>
     <row r="1053">
-      <c r="A1053" s="2" t="n">
+      <c r="A1053" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1053" t="inlineStr">
@@ -22485,7 +22485,7 @@
       </c>
     </row>
     <row r="1054">
-      <c r="A1054" s="2" t="n">
+      <c r="A1054" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1054" t="inlineStr">
@@ -22506,7 +22506,7 @@
       </c>
     </row>
     <row r="1055">
-      <c r="A1055" s="2" t="n">
+      <c r="A1055" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1055" t="inlineStr">
@@ -22527,7 +22527,7 @@
       </c>
     </row>
     <row r="1056">
-      <c r="A1056" s="2" t="n">
+      <c r="A1056" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1056" t="inlineStr">
@@ -22548,7 +22548,7 @@
       </c>
     </row>
     <row r="1057">
-      <c r="A1057" s="2" t="n">
+      <c r="A1057" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1057" t="inlineStr">
@@ -22569,7 +22569,7 @@
       </c>
     </row>
     <row r="1058">
-      <c r="A1058" s="2" t="n">
+      <c r="A1058" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1058" t="inlineStr">
@@ -22590,7 +22590,7 @@
       </c>
     </row>
     <row r="1059">
-      <c r="A1059" s="2" t="n">
+      <c r="A1059" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1059" t="inlineStr">
@@ -22611,7 +22611,7 @@
       </c>
     </row>
     <row r="1060">
-      <c r="A1060" s="2" t="n">
+      <c r="A1060" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1060" t="inlineStr">
@@ -22632,7 +22632,7 @@
       </c>
     </row>
     <row r="1061">
-      <c r="A1061" s="2" t="n">
+      <c r="A1061" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1061" t="inlineStr">
@@ -22653,7 +22653,7 @@
       </c>
     </row>
     <row r="1062">
-      <c r="A1062" s="2" t="n">
+      <c r="A1062" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1062" t="inlineStr">
@@ -22674,7 +22674,7 @@
       </c>
     </row>
     <row r="1063">
-      <c r="A1063" s="2" t="n">
+      <c r="A1063" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1063" t="inlineStr">
@@ -22695,7 +22695,7 @@
       </c>
     </row>
     <row r="1064">
-      <c r="A1064" s="2" t="n">
+      <c r="A1064" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1064" t="inlineStr">
@@ -22716,7 +22716,7 @@
       </c>
     </row>
     <row r="1065">
-      <c r="A1065" s="2" t="n">
+      <c r="A1065" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1065" t="inlineStr">
@@ -22737,7 +22737,7 @@
       </c>
     </row>
     <row r="1066">
-      <c r="A1066" s="2" t="n">
+      <c r="A1066" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1066" t="inlineStr">
@@ -22758,7 +22758,7 @@
       </c>
     </row>
     <row r="1067">
-      <c r="A1067" s="2" t="n">
+      <c r="A1067" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1067" t="inlineStr">
@@ -22779,7 +22779,7 @@
       </c>
     </row>
     <row r="1068">
-      <c r="A1068" s="2" t="n">
+      <c r="A1068" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1068" t="inlineStr">
@@ -22800,7 +22800,7 @@
       </c>
     </row>
     <row r="1069">
-      <c r="A1069" s="2" t="n">
+      <c r="A1069" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1069" t="inlineStr">
@@ -22821,7 +22821,7 @@
       </c>
     </row>
     <row r="1070">
-      <c r="A1070" s="2" t="n">
+      <c r="A1070" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1070" t="inlineStr">
@@ -22842,7 +22842,7 @@
       </c>
     </row>
     <row r="1071">
-      <c r="A1071" s="2" t="n">
+      <c r="A1071" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1071" t="inlineStr">
@@ -22863,7 +22863,7 @@
       </c>
     </row>
     <row r="1072">
-      <c r="A1072" s="2" t="n">
+      <c r="A1072" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1072" t="inlineStr">
@@ -22884,7 +22884,7 @@
       </c>
     </row>
     <row r="1073">
-      <c r="A1073" s="2" t="n">
+      <c r="A1073" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1073" t="inlineStr">
@@ -22905,7 +22905,7 @@
       </c>
     </row>
     <row r="1074">
-      <c r="A1074" s="2" t="n">
+      <c r="A1074" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="B1074" t="inlineStr">
@@ -22920,6 +22920,615 @@
         <v>48</v>
       </c>
       <c r="E1074" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1075" t="n">
+        <v>35.93000030517578</v>
+      </c>
+      <c r="D1075" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1076" t="n">
+        <v>16.65999984741211</v>
+      </c>
+      <c r="D1076" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1077" t="n">
+        <v>24.63999938964844</v>
+      </c>
+      <c r="D1077" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1078" t="n">
+        <v>4.460000038146973</v>
+      </c>
+      <c r="D1078" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1079" t="n">
+        <v>1.570000052452087</v>
+      </c>
+      <c r="D1079" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1080" t="n">
+        <v>205.7899932861328</v>
+      </c>
+      <c r="D1080" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1081" t="n">
+        <v>81.37999725341797</v>
+      </c>
+      <c r="D1081" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1082" t="n">
+        <v>4.389999866485596</v>
+      </c>
+      <c r="D1082" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1083" t="n">
+        <v>5.039999961853027</v>
+      </c>
+      <c r="D1083" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1084" t="n">
+        <v>6.570000171661377</v>
+      </c>
+      <c r="D1084" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1085" t="n">
+        <v>20.70999908447266</v>
+      </c>
+      <c r="D1085" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1085" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1086" t="n">
+        <v>31.53000068664551</v>
+      </c>
+      <c r="D1086" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1087" t="n">
+        <v>20.02000045776367</v>
+      </c>
+      <c r="D1087" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1088" t="n">
+        <v>5.739999771118164</v>
+      </c>
+      <c r="D1088" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1088" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1089" t="n">
+        <v>26.93000030517578</v>
+      </c>
+      <c r="D1089" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1089" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1090" t="n">
+        <v>14.68000030517578</v>
+      </c>
+      <c r="D1090" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1090" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1091" t="n">
+        <v>12.22000026702881</v>
+      </c>
+      <c r="D1091" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1091" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1092" t="n">
+        <v>19.19000053405762</v>
+      </c>
+      <c r="D1092" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1093" t="n">
+        <v>7.929999828338623</v>
+      </c>
+      <c r="D1093" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1094" t="n">
+        <v>55.93000030517578</v>
+      </c>
+      <c r="D1094" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1095" t="n">
+        <v>4.940000057220459</v>
+      </c>
+      <c r="D1095" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1096" t="n">
+        <v>64.34999847412109</v>
+      </c>
+      <c r="D1096" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1097" t="n">
+        <v>53.15000152587891</v>
+      </c>
+      <c r="D1097" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1098" t="n">
+        <v>21.31999969482422</v>
+      </c>
+      <c r="D1098" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1099" t="n">
+        <v>45.70000076293945</v>
+      </c>
+      <c r="D1099" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1100" t="n">
+        <v>139.7899932861328</v>
+      </c>
+      <c r="D1100" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1101" t="n">
+        <v>42.45000076293945</v>
+      </c>
+      <c r="D1101" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1102" t="n">
+        <v>7.360000133514404</v>
+      </c>
+      <c r="D1102" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1102" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1103" t="n">
+        <v>36.86999893188477</v>
+      </c>
+      <c r="D1103" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1103" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-12
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1103"/>
+  <dimension ref="A1:E1132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22926,7 +22926,7 @@
       </c>
     </row>
     <row r="1075">
-      <c r="A1075" s="2" t="n">
+      <c r="A1075" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1075" t="inlineStr">
@@ -22947,7 +22947,7 @@
       </c>
     </row>
     <row r="1076">
-      <c r="A1076" s="2" t="n">
+      <c r="A1076" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1076" t="inlineStr">
@@ -22968,7 +22968,7 @@
       </c>
     </row>
     <row r="1077">
-      <c r="A1077" s="2" t="n">
+      <c r="A1077" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1077" t="inlineStr">
@@ -22989,7 +22989,7 @@
       </c>
     </row>
     <row r="1078">
-      <c r="A1078" s="2" t="n">
+      <c r="A1078" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1078" t="inlineStr">
@@ -23010,7 +23010,7 @@
       </c>
     </row>
     <row r="1079">
-      <c r="A1079" s="2" t="n">
+      <c r="A1079" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1079" t="inlineStr">
@@ -23031,7 +23031,7 @@
       </c>
     </row>
     <row r="1080">
-      <c r="A1080" s="2" t="n">
+      <c r="A1080" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1080" t="inlineStr">
@@ -23052,7 +23052,7 @@
       </c>
     </row>
     <row r="1081">
-      <c r="A1081" s="2" t="n">
+      <c r="A1081" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1081" t="inlineStr">
@@ -23073,7 +23073,7 @@
       </c>
     </row>
     <row r="1082">
-      <c r="A1082" s="2" t="n">
+      <c r="A1082" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1082" t="inlineStr">
@@ -23094,7 +23094,7 @@
       </c>
     </row>
     <row r="1083">
-      <c r="A1083" s="2" t="n">
+      <c r="A1083" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1083" t="inlineStr">
@@ -23115,7 +23115,7 @@
       </c>
     </row>
     <row r="1084">
-      <c r="A1084" s="2" t="n">
+      <c r="A1084" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1084" t="inlineStr">
@@ -23136,7 +23136,7 @@
       </c>
     </row>
     <row r="1085">
-      <c r="A1085" s="2" t="n">
+      <c r="A1085" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1085" t="inlineStr">
@@ -23157,7 +23157,7 @@
       </c>
     </row>
     <row r="1086">
-      <c r="A1086" s="2" t="n">
+      <c r="A1086" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1086" t="inlineStr">
@@ -23178,7 +23178,7 @@
       </c>
     </row>
     <row r="1087">
-      <c r="A1087" s="2" t="n">
+      <c r="A1087" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1087" t="inlineStr">
@@ -23199,7 +23199,7 @@
       </c>
     </row>
     <row r="1088">
-      <c r="A1088" s="2" t="n">
+      <c r="A1088" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1088" t="inlineStr">
@@ -23220,7 +23220,7 @@
       </c>
     </row>
     <row r="1089">
-      <c r="A1089" s="2" t="n">
+      <c r="A1089" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1089" t="inlineStr">
@@ -23241,7 +23241,7 @@
       </c>
     </row>
     <row r="1090">
-      <c r="A1090" s="2" t="n">
+      <c r="A1090" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1090" t="inlineStr">
@@ -23262,7 +23262,7 @@
       </c>
     </row>
     <row r="1091">
-      <c r="A1091" s="2" t="n">
+      <c r="A1091" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1091" t="inlineStr">
@@ -23283,7 +23283,7 @@
       </c>
     </row>
     <row r="1092">
-      <c r="A1092" s="2" t="n">
+      <c r="A1092" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1092" t="inlineStr">
@@ -23304,7 +23304,7 @@
       </c>
     </row>
     <row r="1093">
-      <c r="A1093" s="2" t="n">
+      <c r="A1093" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1093" t="inlineStr">
@@ -23325,7 +23325,7 @@
       </c>
     </row>
     <row r="1094">
-      <c r="A1094" s="2" t="n">
+      <c r="A1094" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1094" t="inlineStr">
@@ -23346,7 +23346,7 @@
       </c>
     </row>
     <row r="1095">
-      <c r="A1095" s="2" t="n">
+      <c r="A1095" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1095" t="inlineStr">
@@ -23367,7 +23367,7 @@
       </c>
     </row>
     <row r="1096">
-      <c r="A1096" s="2" t="n">
+      <c r="A1096" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1096" t="inlineStr">
@@ -23388,7 +23388,7 @@
       </c>
     </row>
     <row r="1097">
-      <c r="A1097" s="2" t="n">
+      <c r="A1097" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1097" t="inlineStr">
@@ -23409,7 +23409,7 @@
       </c>
     </row>
     <row r="1098">
-      <c r="A1098" s="2" t="n">
+      <c r="A1098" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1098" t="inlineStr">
@@ -23430,7 +23430,7 @@
       </c>
     </row>
     <row r="1099">
-      <c r="A1099" s="2" t="n">
+      <c r="A1099" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1099" t="inlineStr">
@@ -23451,7 +23451,7 @@
       </c>
     </row>
     <row r="1100">
-      <c r="A1100" s="2" t="n">
+      <c r="A1100" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1100" t="inlineStr">
@@ -23472,7 +23472,7 @@
       </c>
     </row>
     <row r="1101">
-      <c r="A1101" s="2" t="n">
+      <c r="A1101" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1101" t="inlineStr">
@@ -23493,7 +23493,7 @@
       </c>
     </row>
     <row r="1102">
-      <c r="A1102" s="2" t="n">
+      <c r="A1102" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1102" t="inlineStr">
@@ -23514,7 +23514,7 @@
       </c>
     </row>
     <row r="1103">
-      <c r="A1103" s="2" t="n">
+      <c r="A1103" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="B1103" t="inlineStr">
@@ -23529,6 +23529,615 @@
         <v>48</v>
       </c>
       <c r="E1103" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1104" t="n">
+        <v>35.83000183105469</v>
+      </c>
+      <c r="D1104" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1104" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1105" t="n">
+        <v>16.67000007629395</v>
+      </c>
+      <c r="D1105" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1105" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1106" t="n">
+        <v>24.63999938964844</v>
+      </c>
+      <c r="D1106" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1106" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1107" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D1107" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1108" t="n">
+        <v>1.600000023841858</v>
+      </c>
+      <c r="D1108" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1109" t="n">
+        <v>205.5500030517578</v>
+      </c>
+      <c r="D1109" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1110" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="D1110" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1111" t="n">
+        <v>4.369999885559082</v>
+      </c>
+      <c r="D1111" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1112" t="n">
+        <v>5.010000228881836</v>
+      </c>
+      <c r="D1112" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1113" t="n">
+        <v>6.610000133514404</v>
+      </c>
+      <c r="D1113" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1113" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1114" t="n">
+        <v>20.8700008392334</v>
+      </c>
+      <c r="D1114" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1114" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1115" t="n">
+        <v>31.40999984741211</v>
+      </c>
+      <c r="D1115" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1115" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1116" t="n">
+        <v>19.76000022888184</v>
+      </c>
+      <c r="D1116" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1117" t="n">
+        <v>5.699999809265137</v>
+      </c>
+      <c r="D1117" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1118" t="n">
+        <v>26.93000030517578</v>
+      </c>
+      <c r="D1118" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1119" t="n">
+        <v>14.59000015258789</v>
+      </c>
+      <c r="D1119" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1120" t="n">
+        <v>12.22000026702881</v>
+      </c>
+      <c r="D1120" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1121" t="n">
+        <v>18.94000053405762</v>
+      </c>
+      <c r="D1121" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1122" t="n">
+        <v>7.820000171661377</v>
+      </c>
+      <c r="D1122" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1123" t="n">
+        <v>56</v>
+      </c>
+      <c r="D1123" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1124" t="n">
+        <v>4.940000057220459</v>
+      </c>
+      <c r="D1124" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1125" t="n">
+        <v>64.44999694824219</v>
+      </c>
+      <c r="D1125" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1126" t="n">
+        <v>53.15999984741211</v>
+      </c>
+      <c r="D1126" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1127" t="n">
+        <v>21.45999908447266</v>
+      </c>
+      <c r="D1127" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1128" t="n">
+        <v>45.75</v>
+      </c>
+      <c r="D1128" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1129" t="n">
+        <v>139.8000030517578</v>
+      </c>
+      <c r="D1129" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1130" t="n">
+        <v>42.66999816894531</v>
+      </c>
+      <c r="D1130" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1131" t="n">
+        <v>7.300000190734863</v>
+      </c>
+      <c r="D1131" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1132" t="n">
+        <v>36.88000106811523</v>
+      </c>
+      <c r="D1132" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1132" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-13
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1132"/>
+  <dimension ref="A1:E1161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23535,7 +23535,7 @@
       </c>
     </row>
     <row r="1104">
-      <c r="A1104" s="2" t="n">
+      <c r="A1104" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1104" t="inlineStr">
@@ -23556,7 +23556,7 @@
       </c>
     </row>
     <row r="1105">
-      <c r="A1105" s="2" t="n">
+      <c r="A1105" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1105" t="inlineStr">
@@ -23577,7 +23577,7 @@
       </c>
     </row>
     <row r="1106">
-      <c r="A1106" s="2" t="n">
+      <c r="A1106" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1106" t="inlineStr">
@@ -23598,7 +23598,7 @@
       </c>
     </row>
     <row r="1107">
-      <c r="A1107" s="2" t="n">
+      <c r="A1107" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1107" t="inlineStr">
@@ -23619,7 +23619,7 @@
       </c>
     </row>
     <row r="1108">
-      <c r="A1108" s="2" t="n">
+      <c r="A1108" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1108" t="inlineStr">
@@ -23640,7 +23640,7 @@
       </c>
     </row>
     <row r="1109">
-      <c r="A1109" s="2" t="n">
+      <c r="A1109" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1109" t="inlineStr">
@@ -23661,7 +23661,7 @@
       </c>
     </row>
     <row r="1110">
-      <c r="A1110" s="2" t="n">
+      <c r="A1110" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1110" t="inlineStr">
@@ -23682,7 +23682,7 @@
       </c>
     </row>
     <row r="1111">
-      <c r="A1111" s="2" t="n">
+      <c r="A1111" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1111" t="inlineStr">
@@ -23703,7 +23703,7 @@
       </c>
     </row>
     <row r="1112">
-      <c r="A1112" s="2" t="n">
+      <c r="A1112" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1112" t="inlineStr">
@@ -23724,7 +23724,7 @@
       </c>
     </row>
     <row r="1113">
-      <c r="A1113" s="2" t="n">
+      <c r="A1113" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1113" t="inlineStr">
@@ -23745,7 +23745,7 @@
       </c>
     </row>
     <row r="1114">
-      <c r="A1114" s="2" t="n">
+      <c r="A1114" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1114" t="inlineStr">
@@ -23766,7 +23766,7 @@
       </c>
     </row>
     <row r="1115">
-      <c r="A1115" s="2" t="n">
+      <c r="A1115" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1115" t="inlineStr">
@@ -23787,7 +23787,7 @@
       </c>
     </row>
     <row r="1116">
-      <c r="A1116" s="2" t="n">
+      <c r="A1116" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1116" t="inlineStr">
@@ -23808,7 +23808,7 @@
       </c>
     </row>
     <row r="1117">
-      <c r="A1117" s="2" t="n">
+      <c r="A1117" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1117" t="inlineStr">
@@ -23829,7 +23829,7 @@
       </c>
     </row>
     <row r="1118">
-      <c r="A1118" s="2" t="n">
+      <c r="A1118" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1118" t="inlineStr">
@@ -23850,7 +23850,7 @@
       </c>
     </row>
     <row r="1119">
-      <c r="A1119" s="2" t="n">
+      <c r="A1119" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1119" t="inlineStr">
@@ -23871,7 +23871,7 @@
       </c>
     </row>
     <row r="1120">
-      <c r="A1120" s="2" t="n">
+      <c r="A1120" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1120" t="inlineStr">
@@ -23892,7 +23892,7 @@
       </c>
     </row>
     <row r="1121">
-      <c r="A1121" s="2" t="n">
+      <c r="A1121" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1121" t="inlineStr">
@@ -23913,7 +23913,7 @@
       </c>
     </row>
     <row r="1122">
-      <c r="A1122" s="2" t="n">
+      <c r="A1122" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1122" t="inlineStr">
@@ -23934,7 +23934,7 @@
       </c>
     </row>
     <row r="1123">
-      <c r="A1123" s="2" t="n">
+      <c r="A1123" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1123" t="inlineStr">
@@ -23955,7 +23955,7 @@
       </c>
     </row>
     <row r="1124">
-      <c r="A1124" s="2" t="n">
+      <c r="A1124" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1124" t="inlineStr">
@@ -23976,7 +23976,7 @@
       </c>
     </row>
     <row r="1125">
-      <c r="A1125" s="2" t="n">
+      <c r="A1125" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1125" t="inlineStr">
@@ -23997,7 +23997,7 @@
       </c>
     </row>
     <row r="1126">
-      <c r="A1126" s="2" t="n">
+      <c r="A1126" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1126" t="inlineStr">
@@ -24018,7 +24018,7 @@
       </c>
     </row>
     <row r="1127">
-      <c r="A1127" s="2" t="n">
+      <c r="A1127" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1127" t="inlineStr">
@@ -24039,7 +24039,7 @@
       </c>
     </row>
     <row r="1128">
-      <c r="A1128" s="2" t="n">
+      <c r="A1128" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1128" t="inlineStr">
@@ -24060,7 +24060,7 @@
       </c>
     </row>
     <row r="1129">
-      <c r="A1129" s="2" t="n">
+      <c r="A1129" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1129" t="inlineStr">
@@ -24081,7 +24081,7 @@
       </c>
     </row>
     <row r="1130">
-      <c r="A1130" s="2" t="n">
+      <c r="A1130" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1130" t="inlineStr">
@@ -24102,7 +24102,7 @@
       </c>
     </row>
     <row r="1131">
-      <c r="A1131" s="2" t="n">
+      <c r="A1131" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1131" t="inlineStr">
@@ -24123,7 +24123,7 @@
       </c>
     </row>
     <row r="1132">
-      <c r="A1132" s="2" t="n">
+      <c r="A1132" s="1" t="n">
         <v>46307</v>
       </c>
       <c r="B1132" t="inlineStr">
@@ -24138,6 +24138,615 @@
         <v>48</v>
       </c>
       <c r="E1132" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1133" t="n">
+        <v>34.66999816894531</v>
+      </c>
+      <c r="D1133" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1134" t="n">
+        <v>17.28000068664551</v>
+      </c>
+      <c r="D1134" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1135" t="n">
+        <v>24.22999954223633</v>
+      </c>
+      <c r="D1135" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1136" t="n">
+        <v>4.400000095367432</v>
+      </c>
+      <c r="D1136" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1137" t="n">
+        <v>1.450000047683716</v>
+      </c>
+      <c r="D1137" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1138" t="n">
+        <v>203.75</v>
+      </c>
+      <c r="D1138" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1139" t="n">
+        <v>80.06999969482422</v>
+      </c>
+      <c r="D1139" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1140" t="n">
+        <v>4.46999979019165</v>
+      </c>
+      <c r="D1140" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1141" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1141" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1142" t="n">
+        <v>6.519999980926514</v>
+      </c>
+      <c r="D1142" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1143" t="n">
+        <v>20.92000007629395</v>
+      </c>
+      <c r="D1143" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1144" t="n">
+        <v>31.29999923706055</v>
+      </c>
+      <c r="D1144" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1145" t="n">
+        <v>18.85000038146973</v>
+      </c>
+      <c r="D1145" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1146" t="n">
+        <v>5.429999828338623</v>
+      </c>
+      <c r="D1146" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1147" t="n">
+        <v>25.92000007629395</v>
+      </c>
+      <c r="D1147" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1148" t="n">
+        <v>13.67000007629395</v>
+      </c>
+      <c r="D1148" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1149" t="n">
+        <v>11.36999988555908</v>
+      </c>
+      <c r="D1149" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1150" t="n">
+        <v>17.43000030517578</v>
+      </c>
+      <c r="D1150" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1151" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D1151" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1152" t="n">
+        <v>56.7400016784668</v>
+      </c>
+      <c r="D1152" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1153" t="n">
+        <v>4.789999961853027</v>
+      </c>
+      <c r="D1153" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1154" t="n">
+        <v>66.66999816894531</v>
+      </c>
+      <c r="D1154" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1155" t="n">
+        <v>52.58000183105469</v>
+      </c>
+      <c r="D1155" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1156" t="n">
+        <v>20.70000076293945</v>
+      </c>
+      <c r="D1156" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1157" t="n">
+        <v>44.25</v>
+      </c>
+      <c r="D1157" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1158" t="n">
+        <v>134.9600067138672</v>
+      </c>
+      <c r="D1158" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1159" t="n">
+        <v>43.18000030517578</v>
+      </c>
+      <c r="D1159" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1160" t="n">
+        <v>7.150000095367432</v>
+      </c>
+      <c r="D1160" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1161" t="n">
+        <v>36.45999908447266</v>
+      </c>
+      <c r="D1161" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1161" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-15
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1161"/>
+  <dimension ref="A1:E1190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24144,7 +24144,7 @@
       </c>
     </row>
     <row r="1133">
-      <c r="A1133" s="2" t="n">
+      <c r="A1133" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1133" t="inlineStr">
@@ -24165,7 +24165,7 @@
       </c>
     </row>
     <row r="1134">
-      <c r="A1134" s="2" t="n">
+      <c r="A1134" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1134" t="inlineStr">
@@ -24186,7 +24186,7 @@
       </c>
     </row>
     <row r="1135">
-      <c r="A1135" s="2" t="n">
+      <c r="A1135" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1135" t="inlineStr">
@@ -24207,7 +24207,7 @@
       </c>
     </row>
     <row r="1136">
-      <c r="A1136" s="2" t="n">
+      <c r="A1136" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1136" t="inlineStr">
@@ -24228,7 +24228,7 @@
       </c>
     </row>
     <row r="1137">
-      <c r="A1137" s="2" t="n">
+      <c r="A1137" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1137" t="inlineStr">
@@ -24249,7 +24249,7 @@
       </c>
     </row>
     <row r="1138">
-      <c r="A1138" s="2" t="n">
+      <c r="A1138" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1138" t="inlineStr">
@@ -24270,7 +24270,7 @@
       </c>
     </row>
     <row r="1139">
-      <c r="A1139" s="2" t="n">
+      <c r="A1139" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1139" t="inlineStr">
@@ -24291,7 +24291,7 @@
       </c>
     </row>
     <row r="1140">
-      <c r="A1140" s="2" t="n">
+      <c r="A1140" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1140" t="inlineStr">
@@ -24312,7 +24312,7 @@
       </c>
     </row>
     <row r="1141">
-      <c r="A1141" s="2" t="n">
+      <c r="A1141" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1141" t="inlineStr">
@@ -24333,7 +24333,7 @@
       </c>
     </row>
     <row r="1142">
-      <c r="A1142" s="2" t="n">
+      <c r="A1142" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1142" t="inlineStr">
@@ -24354,7 +24354,7 @@
       </c>
     </row>
     <row r="1143">
-      <c r="A1143" s="2" t="n">
+      <c r="A1143" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1143" t="inlineStr">
@@ -24375,7 +24375,7 @@
       </c>
     </row>
     <row r="1144">
-      <c r="A1144" s="2" t="n">
+      <c r="A1144" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1144" t="inlineStr">
@@ -24396,7 +24396,7 @@
       </c>
     </row>
     <row r="1145">
-      <c r="A1145" s="2" t="n">
+      <c r="A1145" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1145" t="inlineStr">
@@ -24417,7 +24417,7 @@
       </c>
     </row>
     <row r="1146">
-      <c r="A1146" s="2" t="n">
+      <c r="A1146" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1146" t="inlineStr">
@@ -24438,7 +24438,7 @@
       </c>
     </row>
     <row r="1147">
-      <c r="A1147" s="2" t="n">
+      <c r="A1147" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1147" t="inlineStr">
@@ -24459,7 +24459,7 @@
       </c>
     </row>
     <row r="1148">
-      <c r="A1148" s="2" t="n">
+      <c r="A1148" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1148" t="inlineStr">
@@ -24480,7 +24480,7 @@
       </c>
     </row>
     <row r="1149">
-      <c r="A1149" s="2" t="n">
+      <c r="A1149" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1149" t="inlineStr">
@@ -24501,7 +24501,7 @@
       </c>
     </row>
     <row r="1150">
-      <c r="A1150" s="2" t="n">
+      <c r="A1150" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1150" t="inlineStr">
@@ -24522,7 +24522,7 @@
       </c>
     </row>
     <row r="1151">
-      <c r="A1151" s="2" t="n">
+      <c r="A1151" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1151" t="inlineStr">
@@ -24543,7 +24543,7 @@
       </c>
     </row>
     <row r="1152">
-      <c r="A1152" s="2" t="n">
+      <c r="A1152" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1152" t="inlineStr">
@@ -24564,7 +24564,7 @@
       </c>
     </row>
     <row r="1153">
-      <c r="A1153" s="2" t="n">
+      <c r="A1153" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1153" t="inlineStr">
@@ -24585,7 +24585,7 @@
       </c>
     </row>
     <row r="1154">
-      <c r="A1154" s="2" t="n">
+      <c r="A1154" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1154" t="inlineStr">
@@ -24606,7 +24606,7 @@
       </c>
     </row>
     <row r="1155">
-      <c r="A1155" s="2" t="n">
+      <c r="A1155" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1155" t="inlineStr">
@@ -24627,7 +24627,7 @@
       </c>
     </row>
     <row r="1156">
-      <c r="A1156" s="2" t="n">
+      <c r="A1156" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1156" t="inlineStr">
@@ -24648,7 +24648,7 @@
       </c>
     </row>
     <row r="1157">
-      <c r="A1157" s="2" t="n">
+      <c r="A1157" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1157" t="inlineStr">
@@ -24669,7 +24669,7 @@
       </c>
     </row>
     <row r="1158">
-      <c r="A1158" s="2" t="n">
+      <c r="A1158" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1158" t="inlineStr">
@@ -24690,7 +24690,7 @@
       </c>
     </row>
     <row r="1159">
-      <c r="A1159" s="2" t="n">
+      <c r="A1159" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1159" t="inlineStr">
@@ -24711,7 +24711,7 @@
       </c>
     </row>
     <row r="1160">
-      <c r="A1160" s="2" t="n">
+      <c r="A1160" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1160" t="inlineStr">
@@ -24732,7 +24732,7 @@
       </c>
     </row>
     <row r="1161">
-      <c r="A1161" s="2" t="n">
+      <c r="A1161" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="B1161" t="inlineStr">
@@ -24747,6 +24747,615 @@
         <v>48</v>
       </c>
       <c r="E1161" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1162" t="n">
+        <v>34.45000076293945</v>
+      </c>
+      <c r="D1162" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1163" t="n">
+        <v>18.06999969482422</v>
+      </c>
+      <c r="D1163" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1164" t="n">
+        <v>23.79999923706055</v>
+      </c>
+      <c r="D1164" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1165" t="n">
+        <v>4.110000133514404</v>
+      </c>
+      <c r="D1165" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1166" t="n">
+        <v>1.120000004768372</v>
+      </c>
+      <c r="D1166" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1167" t="n">
+        <v>200.7799987792969</v>
+      </c>
+      <c r="D1167" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1168" t="n">
+        <v>76.90000152587891</v>
+      </c>
+      <c r="D1168" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1169" t="n">
+        <v>4.360000133514404</v>
+      </c>
+      <c r="D1169" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1170" t="n">
+        <v>4.860000133514404</v>
+      </c>
+      <c r="D1170" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1171" t="n">
+        <v>6.019999980926514</v>
+      </c>
+      <c r="D1171" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1172" t="n">
+        <v>21.14999961853027</v>
+      </c>
+      <c r="D1172" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1173" t="n">
+        <v>31.28000068664551</v>
+      </c>
+      <c r="D1173" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1174" t="n">
+        <v>18.14999961853027</v>
+      </c>
+      <c r="D1174" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1175" t="n">
+        <v>5.150000095367432</v>
+      </c>
+      <c r="D1175" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1176" t="n">
+        <v>25.56999969482422</v>
+      </c>
+      <c r="D1176" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1177" t="n">
+        <v>13.07999992370605</v>
+      </c>
+      <c r="D1177" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1178" t="n">
+        <v>10.36999988555908</v>
+      </c>
+      <c r="D1178" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1179" t="n">
+        <v>16.19000053405762</v>
+      </c>
+      <c r="D1179" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1180" t="n">
+        <v>7.110000133514404</v>
+      </c>
+      <c r="D1180" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1181" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="D1181" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1182" t="n">
+        <v>4.670000076293945</v>
+      </c>
+      <c r="D1182" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1183" t="n">
+        <v>68.26999664306641</v>
+      </c>
+      <c r="D1183" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1183" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1184" t="n">
+        <v>52.7400016784668</v>
+      </c>
+      <c r="D1184" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1184" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1185" t="n">
+        <v>20.48999977111816</v>
+      </c>
+      <c r="D1185" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1185" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1186" t="n">
+        <v>42.68000030517578</v>
+      </c>
+      <c r="D1186" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1186" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1187" t="n">
+        <v>130.1799926757812</v>
+      </c>
+      <c r="D1187" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1187" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1188" t="n">
+        <v>42.40000152587891</v>
+      </c>
+      <c r="D1188" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1188" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1189" t="n">
+        <v>6.710000038146973</v>
+      </c>
+      <c r="D1189" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1189" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1190" t="n">
+        <v>36.25</v>
+      </c>
+      <c r="D1190" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1190" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-16
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1190"/>
+  <dimension ref="A1:E1219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24753,7 +24753,7 @@
       </c>
     </row>
     <row r="1162">
-      <c r="A1162" s="2" t="n">
+      <c r="A1162" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1162" t="inlineStr">
@@ -24774,7 +24774,7 @@
       </c>
     </row>
     <row r="1163">
-      <c r="A1163" s="2" t="n">
+      <c r="A1163" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1163" t="inlineStr">
@@ -24795,7 +24795,7 @@
       </c>
     </row>
     <row r="1164">
-      <c r="A1164" s="2" t="n">
+      <c r="A1164" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1164" t="inlineStr">
@@ -24816,7 +24816,7 @@
       </c>
     </row>
     <row r="1165">
-      <c r="A1165" s="2" t="n">
+      <c r="A1165" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1165" t="inlineStr">
@@ -24837,7 +24837,7 @@
       </c>
     </row>
     <row r="1166">
-      <c r="A1166" s="2" t="n">
+      <c r="A1166" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1166" t="inlineStr">
@@ -24858,7 +24858,7 @@
       </c>
     </row>
     <row r="1167">
-      <c r="A1167" s="2" t="n">
+      <c r="A1167" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1167" t="inlineStr">
@@ -24879,7 +24879,7 @@
       </c>
     </row>
     <row r="1168">
-      <c r="A1168" s="2" t="n">
+      <c r="A1168" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1168" t="inlineStr">
@@ -24900,7 +24900,7 @@
       </c>
     </row>
     <row r="1169">
-      <c r="A1169" s="2" t="n">
+      <c r="A1169" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1169" t="inlineStr">
@@ -24921,7 +24921,7 @@
       </c>
     </row>
     <row r="1170">
-      <c r="A1170" s="2" t="n">
+      <c r="A1170" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1170" t="inlineStr">
@@ -24942,7 +24942,7 @@
       </c>
     </row>
     <row r="1171">
-      <c r="A1171" s="2" t="n">
+      <c r="A1171" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1171" t="inlineStr">
@@ -24963,7 +24963,7 @@
       </c>
     </row>
     <row r="1172">
-      <c r="A1172" s="2" t="n">
+      <c r="A1172" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1172" t="inlineStr">
@@ -24984,7 +24984,7 @@
       </c>
     </row>
     <row r="1173">
-      <c r="A1173" s="2" t="n">
+      <c r="A1173" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1173" t="inlineStr">
@@ -25005,7 +25005,7 @@
       </c>
     </row>
     <row r="1174">
-      <c r="A1174" s="2" t="n">
+      <c r="A1174" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1174" t="inlineStr">
@@ -25026,7 +25026,7 @@
       </c>
     </row>
     <row r="1175">
-      <c r="A1175" s="2" t="n">
+      <c r="A1175" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1175" t="inlineStr">
@@ -25047,7 +25047,7 @@
       </c>
     </row>
     <row r="1176">
-      <c r="A1176" s="2" t="n">
+      <c r="A1176" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1176" t="inlineStr">
@@ -25068,7 +25068,7 @@
       </c>
     </row>
     <row r="1177">
-      <c r="A1177" s="2" t="n">
+      <c r="A1177" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1177" t="inlineStr">
@@ -25089,7 +25089,7 @@
       </c>
     </row>
     <row r="1178">
-      <c r="A1178" s="2" t="n">
+      <c r="A1178" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1178" t="inlineStr">
@@ -25110,7 +25110,7 @@
       </c>
     </row>
     <row r="1179">
-      <c r="A1179" s="2" t="n">
+      <c r="A1179" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1179" t="inlineStr">
@@ -25131,7 +25131,7 @@
       </c>
     </row>
     <row r="1180">
-      <c r="A1180" s="2" t="n">
+      <c r="A1180" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1180" t="inlineStr">
@@ -25152,7 +25152,7 @@
       </c>
     </row>
     <row r="1181">
-      <c r="A1181" s="2" t="n">
+      <c r="A1181" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1181" t="inlineStr">
@@ -25173,7 +25173,7 @@
       </c>
     </row>
     <row r="1182">
-      <c r="A1182" s="2" t="n">
+      <c r="A1182" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1182" t="inlineStr">
@@ -25194,7 +25194,7 @@
       </c>
     </row>
     <row r="1183">
-      <c r="A1183" s="2" t="n">
+      <c r="A1183" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1183" t="inlineStr">
@@ -25215,7 +25215,7 @@
       </c>
     </row>
     <row r="1184">
-      <c r="A1184" s="2" t="n">
+      <c r="A1184" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1184" t="inlineStr">
@@ -25236,7 +25236,7 @@
       </c>
     </row>
     <row r="1185">
-      <c r="A1185" s="2" t="n">
+      <c r="A1185" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1185" t="inlineStr">
@@ -25257,7 +25257,7 @@
       </c>
     </row>
     <row r="1186">
-      <c r="A1186" s="2" t="n">
+      <c r="A1186" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1186" t="inlineStr">
@@ -25278,7 +25278,7 @@
       </c>
     </row>
     <row r="1187">
-      <c r="A1187" s="2" t="n">
+      <c r="A1187" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1187" t="inlineStr">
@@ -25299,7 +25299,7 @@
       </c>
     </row>
     <row r="1188">
-      <c r="A1188" s="2" t="n">
+      <c r="A1188" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1188" t="inlineStr">
@@ -25320,7 +25320,7 @@
       </c>
     </row>
     <row r="1189">
-      <c r="A1189" s="2" t="n">
+      <c r="A1189" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1189" t="inlineStr">
@@ -25341,7 +25341,7 @@
       </c>
     </row>
     <row r="1190">
-      <c r="A1190" s="2" t="n">
+      <c r="A1190" s="1" t="n">
         <v>46310</v>
       </c>
       <c r="B1190" t="inlineStr">
@@ -25356,6 +25356,615 @@
         <v>48</v>
       </c>
       <c r="E1190" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1191" t="n">
+        <v>34.5099983215332</v>
+      </c>
+      <c r="D1191" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1191" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1192" t="n">
+        <v>17.84000015258789</v>
+      </c>
+      <c r="D1192" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1193" t="n">
+        <v>23.54999923706055</v>
+      </c>
+      <c r="D1193" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1194" t="n">
+        <v>4.199999809265137</v>
+      </c>
+      <c r="D1194" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1195" t="n">
+        <v>1.129999995231628</v>
+      </c>
+      <c r="D1195" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1196" t="n">
+        <v>202.3500061035156</v>
+      </c>
+      <c r="D1196" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1197" t="n">
+        <v>76.48999786376953</v>
+      </c>
+      <c r="D1197" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1197" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1198" t="n">
+        <v>4.130000114440918</v>
+      </c>
+      <c r="D1198" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1198" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1199" t="n">
+        <v>4.869999885559082</v>
+      </c>
+      <c r="D1199" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1199" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1200" t="n">
+        <v>5.820000171661377</v>
+      </c>
+      <c r="D1200" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1200" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1201" t="n">
+        <v>21.80999946594238</v>
+      </c>
+      <c r="D1201" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1201" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1202" t="n">
+        <v>31.60000038146973</v>
+      </c>
+      <c r="D1202" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1202" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1203" t="n">
+        <v>18.10000038146973</v>
+      </c>
+      <c r="D1203" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1203" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1204" t="n">
+        <v>5.159999847412109</v>
+      </c>
+      <c r="D1204" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1204" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1205" t="n">
+        <v>25.77000045776367</v>
+      </c>
+      <c r="D1205" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1205" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1206" t="n">
+        <v>12.90999984741211</v>
+      </c>
+      <c r="D1206" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1206" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1207" t="n">
+        <v>11.0600004196167</v>
+      </c>
+      <c r="D1207" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1208" t="n">
+        <v>16.46999931335449</v>
+      </c>
+      <c r="D1208" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1209" t="n">
+        <v>7.239999771118164</v>
+      </c>
+      <c r="D1209" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1210" t="n">
+        <v>59.2400016784668</v>
+      </c>
+      <c r="D1210" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1211" t="n">
+        <v>4.630000114440918</v>
+      </c>
+      <c r="D1211" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1212" t="n">
+        <v>70.44999694824219</v>
+      </c>
+      <c r="D1212" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1213" t="n">
+        <v>53.06000137329102</v>
+      </c>
+      <c r="D1213" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1214" t="n">
+        <v>20.61000061035156</v>
+      </c>
+      <c r="D1214" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1215" t="n">
+        <v>42.45000076293945</v>
+      </c>
+      <c r="D1215" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1216" t="n">
+        <v>131</v>
+      </c>
+      <c r="D1216" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1217" t="n">
+        <v>43</v>
+      </c>
+      <c r="D1217" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1217" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1218" t="n">
+        <v>6.71999979019165</v>
+      </c>
+      <c r="D1218" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1218" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1219" t="n">
+        <v>36.54999923706055</v>
+      </c>
+      <c r="D1219" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1219" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-19
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1219"/>
+  <dimension ref="A1:E1248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25362,7 +25362,7 @@
       </c>
     </row>
     <row r="1191">
-      <c r="A1191" s="2" t="n">
+      <c r="A1191" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1191" t="inlineStr">
@@ -25383,7 +25383,7 @@
       </c>
     </row>
     <row r="1192">
-      <c r="A1192" s="2" t="n">
+      <c r="A1192" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1192" t="inlineStr">
@@ -25404,7 +25404,7 @@
       </c>
     </row>
     <row r="1193">
-      <c r="A1193" s="2" t="n">
+      <c r="A1193" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1193" t="inlineStr">
@@ -25425,7 +25425,7 @@
       </c>
     </row>
     <row r="1194">
-      <c r="A1194" s="2" t="n">
+      <c r="A1194" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1194" t="inlineStr">
@@ -25446,7 +25446,7 @@
       </c>
     </row>
     <row r="1195">
-      <c r="A1195" s="2" t="n">
+      <c r="A1195" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1195" t="inlineStr">
@@ -25467,7 +25467,7 @@
       </c>
     </row>
     <row r="1196">
-      <c r="A1196" s="2" t="n">
+      <c r="A1196" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1196" t="inlineStr">
@@ -25488,7 +25488,7 @@
       </c>
     </row>
     <row r="1197">
-      <c r="A1197" s="2" t="n">
+      <c r="A1197" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1197" t="inlineStr">
@@ -25509,7 +25509,7 @@
       </c>
     </row>
     <row r="1198">
-      <c r="A1198" s="2" t="n">
+      <c r="A1198" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1198" t="inlineStr">
@@ -25530,7 +25530,7 @@
       </c>
     </row>
     <row r="1199">
-      <c r="A1199" s="2" t="n">
+      <c r="A1199" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1199" t="inlineStr">
@@ -25551,7 +25551,7 @@
       </c>
     </row>
     <row r="1200">
-      <c r="A1200" s="2" t="n">
+      <c r="A1200" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1200" t="inlineStr">
@@ -25572,7 +25572,7 @@
       </c>
     </row>
     <row r="1201">
-      <c r="A1201" s="2" t="n">
+      <c r="A1201" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1201" t="inlineStr">
@@ -25593,7 +25593,7 @@
       </c>
     </row>
     <row r="1202">
-      <c r="A1202" s="2" t="n">
+      <c r="A1202" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1202" t="inlineStr">
@@ -25614,7 +25614,7 @@
       </c>
     </row>
     <row r="1203">
-      <c r="A1203" s="2" t="n">
+      <c r="A1203" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1203" t="inlineStr">
@@ -25635,7 +25635,7 @@
       </c>
     </row>
     <row r="1204">
-      <c r="A1204" s="2" t="n">
+      <c r="A1204" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1204" t="inlineStr">
@@ -25656,7 +25656,7 @@
       </c>
     </row>
     <row r="1205">
-      <c r="A1205" s="2" t="n">
+      <c r="A1205" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1205" t="inlineStr">
@@ -25677,7 +25677,7 @@
       </c>
     </row>
     <row r="1206">
-      <c r="A1206" s="2" t="n">
+      <c r="A1206" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1206" t="inlineStr">
@@ -25698,7 +25698,7 @@
       </c>
     </row>
     <row r="1207">
-      <c r="A1207" s="2" t="n">
+      <c r="A1207" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1207" t="inlineStr">
@@ -25719,7 +25719,7 @@
       </c>
     </row>
     <row r="1208">
-      <c r="A1208" s="2" t="n">
+      <c r="A1208" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1208" t="inlineStr">
@@ -25740,7 +25740,7 @@
       </c>
     </row>
     <row r="1209">
-      <c r="A1209" s="2" t="n">
+      <c r="A1209" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1209" t="inlineStr">
@@ -25761,7 +25761,7 @@
       </c>
     </row>
     <row r="1210">
-      <c r="A1210" s="2" t="n">
+      <c r="A1210" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1210" t="inlineStr">
@@ -25782,7 +25782,7 @@
       </c>
     </row>
     <row r="1211">
-      <c r="A1211" s="2" t="n">
+      <c r="A1211" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1211" t="inlineStr">
@@ -25803,7 +25803,7 @@
       </c>
     </row>
     <row r="1212">
-      <c r="A1212" s="2" t="n">
+      <c r="A1212" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1212" t="inlineStr">
@@ -25824,7 +25824,7 @@
       </c>
     </row>
     <row r="1213">
-      <c r="A1213" s="2" t="n">
+      <c r="A1213" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1213" t="inlineStr">
@@ -25845,7 +25845,7 @@
       </c>
     </row>
     <row r="1214">
-      <c r="A1214" s="2" t="n">
+      <c r="A1214" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1214" t="inlineStr">
@@ -25866,7 +25866,7 @@
       </c>
     </row>
     <row r="1215">
-      <c r="A1215" s="2" t="n">
+      <c r="A1215" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1215" t="inlineStr">
@@ -25887,7 +25887,7 @@
       </c>
     </row>
     <row r="1216">
-      <c r="A1216" s="2" t="n">
+      <c r="A1216" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1216" t="inlineStr">
@@ -25908,7 +25908,7 @@
       </c>
     </row>
     <row r="1217">
-      <c r="A1217" s="2" t="n">
+      <c r="A1217" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1217" t="inlineStr">
@@ -25929,7 +25929,7 @@
       </c>
     </row>
     <row r="1218">
-      <c r="A1218" s="2" t="n">
+      <c r="A1218" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1218" t="inlineStr">
@@ -25950,7 +25950,7 @@
       </c>
     </row>
     <row r="1219">
-      <c r="A1219" s="2" t="n">
+      <c r="A1219" s="1" t="n">
         <v>46311</v>
       </c>
       <c r="B1219" t="inlineStr">
@@ -25965,6 +25965,615 @@
         <v>48</v>
       </c>
       <c r="E1219" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1220" t="n">
+        <v>34.95999908447266</v>
+      </c>
+      <c r="D1220" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1221" t="n">
+        <v>18.38999938964844</v>
+      </c>
+      <c r="D1221" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1222" t="n">
+        <v>23.89999961853027</v>
+      </c>
+      <c r="D1222" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1223" t="n">
+        <v>4.329999923706055</v>
+      </c>
+      <c r="D1223" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1224" t="n">
+        <v>1.179999947547913</v>
+      </c>
+      <c r="D1224" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1224" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1225" t="n">
+        <v>201.9100036621094</v>
+      </c>
+      <c r="D1225" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1225" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1226" t="n">
+        <v>78.01000213623047</v>
+      </c>
+      <c r="D1226" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1226" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1227" t="n">
+        <v>4.190000057220459</v>
+      </c>
+      <c r="D1227" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1227" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1228" t="n">
+        <v>4.96999979019165</v>
+      </c>
+      <c r="D1228" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1228" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1229" t="n">
+        <v>5.940000057220459</v>
+      </c>
+      <c r="D1229" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1229" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1230" t="n">
+        <v>21.1200008392334</v>
+      </c>
+      <c r="D1230" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1230" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1231" t="n">
+        <v>31.44000053405762</v>
+      </c>
+      <c r="D1231" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1231" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1232" t="n">
+        <v>18.20000076293945</v>
+      </c>
+      <c r="D1232" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1232" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1233" t="n">
+        <v>5.420000076293945</v>
+      </c>
+      <c r="D1233" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1233" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1234" t="n">
+        <v>26.34000015258789</v>
+      </c>
+      <c r="D1234" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1234" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1235" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D1235" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1235" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1236" t="n">
+        <v>11.82999992370605</v>
+      </c>
+      <c r="D1236" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1236" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1237" t="n">
+        <v>17.6200008392334</v>
+      </c>
+      <c r="D1237" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1237" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1238" t="n">
+        <v>7.96999979019165</v>
+      </c>
+      <c r="D1238" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1238" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1239" t="n">
+        <v>58.15000152587891</v>
+      </c>
+      <c r="D1239" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1239" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1240" t="n">
+        <v>4.699999809265137</v>
+      </c>
+      <c r="D1240" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1240" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1241" t="n">
+        <v>71.06999969482422</v>
+      </c>
+      <c r="D1241" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1241" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1242" t="n">
+        <v>51.40000152587891</v>
+      </c>
+      <c r="D1242" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1242" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1243" t="n">
+        <v>21.31999969482422</v>
+      </c>
+      <c r="D1243" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1243" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1244" t="n">
+        <v>43.31999969482422</v>
+      </c>
+      <c r="D1244" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1244" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1245" t="n">
+        <v>134</v>
+      </c>
+      <c r="D1245" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1245" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1246" t="n">
+        <v>42.79000091552734</v>
+      </c>
+      <c r="D1246" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1246" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1247" t="n">
+        <v>6.650000095367432</v>
+      </c>
+      <c r="D1247" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1247" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1248" t="n">
+        <v>36.20000076293945</v>
+      </c>
+      <c r="D1248" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1248" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-20
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1248"/>
+  <dimension ref="A1:E1277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25971,7 +25971,7 @@
       </c>
     </row>
     <row r="1220">
-      <c r="A1220" s="2" t="n">
+      <c r="A1220" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1220" t="inlineStr">
@@ -25992,7 +25992,7 @@
       </c>
     </row>
     <row r="1221">
-      <c r="A1221" s="2" t="n">
+      <c r="A1221" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1221" t="inlineStr">
@@ -26013,7 +26013,7 @@
       </c>
     </row>
     <row r="1222">
-      <c r="A1222" s="2" t="n">
+      <c r="A1222" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1222" t="inlineStr">
@@ -26034,7 +26034,7 @@
       </c>
     </row>
     <row r="1223">
-      <c r="A1223" s="2" t="n">
+      <c r="A1223" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1223" t="inlineStr">
@@ -26055,7 +26055,7 @@
       </c>
     </row>
     <row r="1224">
-      <c r="A1224" s="2" t="n">
+      <c r="A1224" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1224" t="inlineStr">
@@ -26076,7 +26076,7 @@
       </c>
     </row>
     <row r="1225">
-      <c r="A1225" s="2" t="n">
+      <c r="A1225" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1225" t="inlineStr">
@@ -26097,7 +26097,7 @@
       </c>
     </row>
     <row r="1226">
-      <c r="A1226" s="2" t="n">
+      <c r="A1226" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1226" t="inlineStr">
@@ -26118,7 +26118,7 @@
       </c>
     </row>
     <row r="1227">
-      <c r="A1227" s="2" t="n">
+      <c r="A1227" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1227" t="inlineStr">
@@ -26139,7 +26139,7 @@
       </c>
     </row>
     <row r="1228">
-      <c r="A1228" s="2" t="n">
+      <c r="A1228" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1228" t="inlineStr">
@@ -26160,7 +26160,7 @@
       </c>
     </row>
     <row r="1229">
-      <c r="A1229" s="2" t="n">
+      <c r="A1229" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1229" t="inlineStr">
@@ -26181,7 +26181,7 @@
       </c>
     </row>
     <row r="1230">
-      <c r="A1230" s="2" t="n">
+      <c r="A1230" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1230" t="inlineStr">
@@ -26202,7 +26202,7 @@
       </c>
     </row>
     <row r="1231">
-      <c r="A1231" s="2" t="n">
+      <c r="A1231" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1231" t="inlineStr">
@@ -26223,7 +26223,7 @@
       </c>
     </row>
     <row r="1232">
-      <c r="A1232" s="2" t="n">
+      <c r="A1232" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1232" t="inlineStr">
@@ -26244,7 +26244,7 @@
       </c>
     </row>
     <row r="1233">
-      <c r="A1233" s="2" t="n">
+      <c r="A1233" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1233" t="inlineStr">
@@ -26265,7 +26265,7 @@
       </c>
     </row>
     <row r="1234">
-      <c r="A1234" s="2" t="n">
+      <c r="A1234" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1234" t="inlineStr">
@@ -26286,7 +26286,7 @@
       </c>
     </row>
     <row r="1235">
-      <c r="A1235" s="2" t="n">
+      <c r="A1235" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1235" t="inlineStr">
@@ -26307,7 +26307,7 @@
       </c>
     </row>
     <row r="1236">
-      <c r="A1236" s="2" t="n">
+      <c r="A1236" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1236" t="inlineStr">
@@ -26328,7 +26328,7 @@
       </c>
     </row>
     <row r="1237">
-      <c r="A1237" s="2" t="n">
+      <c r="A1237" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1237" t="inlineStr">
@@ -26349,7 +26349,7 @@
       </c>
     </row>
     <row r="1238">
-      <c r="A1238" s="2" t="n">
+      <c r="A1238" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1238" t="inlineStr">
@@ -26370,7 +26370,7 @@
       </c>
     </row>
     <row r="1239">
-      <c r="A1239" s="2" t="n">
+      <c r="A1239" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1239" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
     </row>
     <row r="1240">
-      <c r="A1240" s="2" t="n">
+      <c r="A1240" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1240" t="inlineStr">
@@ -26412,7 +26412,7 @@
       </c>
     </row>
     <row r="1241">
-      <c r="A1241" s="2" t="n">
+      <c r="A1241" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1241" t="inlineStr">
@@ -26433,7 +26433,7 @@
       </c>
     </row>
     <row r="1242">
-      <c r="A1242" s="2" t="n">
+      <c r="A1242" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1242" t="inlineStr">
@@ -26454,7 +26454,7 @@
       </c>
     </row>
     <row r="1243">
-      <c r="A1243" s="2" t="n">
+      <c r="A1243" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1243" t="inlineStr">
@@ -26475,7 +26475,7 @@
       </c>
     </row>
     <row r="1244">
-      <c r="A1244" s="2" t="n">
+      <c r="A1244" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1244" t="inlineStr">
@@ -26496,7 +26496,7 @@
       </c>
     </row>
     <row r="1245">
-      <c r="A1245" s="2" t="n">
+      <c r="A1245" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1245" t="inlineStr">
@@ -26517,7 +26517,7 @@
       </c>
     </row>
     <row r="1246">
-      <c r="A1246" s="2" t="n">
+      <c r="A1246" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1246" t="inlineStr">
@@ -26538,7 +26538,7 @@
       </c>
     </row>
     <row r="1247">
-      <c r="A1247" s="2" t="n">
+      <c r="A1247" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1247" t="inlineStr">
@@ -26559,7 +26559,7 @@
       </c>
     </row>
     <row r="1248">
-      <c r="A1248" s="2" t="n">
+      <c r="A1248" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="B1248" t="inlineStr">
@@ -26574,6 +26574,615 @@
         <v>48</v>
       </c>
       <c r="E1248" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1249" t="n">
+        <v>35.59999847412109</v>
+      </c>
+      <c r="D1249" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1249" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1250" t="n">
+        <v>17.95000076293945</v>
+      </c>
+      <c r="D1250" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1250" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1251" t="n">
+        <v>24.22999954223633</v>
+      </c>
+      <c r="D1251" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1251" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1252" t="n">
+        <v>4.329999923706055</v>
+      </c>
+      <c r="D1252" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1252" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1253" t="n">
+        <v>1.450000047683716</v>
+      </c>
+      <c r="D1253" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1253" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1254" t="n">
+        <v>204.8099975585938</v>
+      </c>
+      <c r="D1254" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1254" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1255" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="D1255" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1255" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1256" t="n">
+        <v>4.159999847412109</v>
+      </c>
+      <c r="D1256" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1256" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1257" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1257" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1257" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1258" t="n">
+        <v>5.980000019073486</v>
+      </c>
+      <c r="D1258" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1258" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1259" t="n">
+        <v>21.20000076293945</v>
+      </c>
+      <c r="D1259" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1259" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1260" t="n">
+        <v>32</v>
+      </c>
+      <c r="D1260" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1260" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1261" t="n">
+        <v>18.94000053405762</v>
+      </c>
+      <c r="D1261" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1261" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1262" t="n">
+        <v>5.650000095367432</v>
+      </c>
+      <c r="D1262" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1262" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1263" t="n">
+        <v>27.14999961853027</v>
+      </c>
+      <c r="D1263" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1263" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1264" t="n">
+        <v>14.15999984741211</v>
+      </c>
+      <c r="D1264" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1265" t="n">
+        <v>13.53999996185303</v>
+      </c>
+      <c r="D1265" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1266" t="n">
+        <v>19.86000061035156</v>
+      </c>
+      <c r="D1266" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1267" t="n">
+        <v>8.260000228881836</v>
+      </c>
+      <c r="D1267" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1268" t="n">
+        <v>58.06999969482422</v>
+      </c>
+      <c r="D1268" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1269" t="n">
+        <v>4.980000019073486</v>
+      </c>
+      <c r="D1269" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1270" t="n">
+        <v>71.09999847412109</v>
+      </c>
+      <c r="D1270" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1271" t="n">
+        <v>52.59000015258789</v>
+      </c>
+      <c r="D1271" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1272" t="n">
+        <v>21.57999992370605</v>
+      </c>
+      <c r="D1272" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1273" t="n">
+        <v>44.09000015258789</v>
+      </c>
+      <c r="D1273" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1274" t="n">
+        <v>138.3699951171875</v>
+      </c>
+      <c r="D1274" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1275" t="n">
+        <v>42.36000061035156</v>
+      </c>
+      <c r="D1275" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1276" t="n">
+        <v>6.78000020980835</v>
+      </c>
+      <c r="D1276" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1277" t="n">
+        <v>36.59000015258789</v>
+      </c>
+      <c r="D1277" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1277" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-21
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1248"/>
+  <dimension ref="A1:E1277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26576,6 +26576,615 @@
         </is>
       </c>
     </row>
+    <row r="1249">
+      <c r="A1249" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1249" t="n">
+        <v>35.27000045776367</v>
+      </c>
+      <c r="D1249" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1249" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1250" t="n">
+        <v>17.45000076293945</v>
+      </c>
+      <c r="D1250" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1250" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1251" t="n">
+        <v>24.05999946594238</v>
+      </c>
+      <c r="D1251" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1251" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1252" t="n">
+        <v>4.289999961853027</v>
+      </c>
+      <c r="D1252" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1252" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1253" t="n">
+        <v>1.409999966621399</v>
+      </c>
+      <c r="D1253" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1253" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1254" t="n">
+        <v>203.3000030517578</v>
+      </c>
+      <c r="D1254" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1254" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1255" t="n">
+        <v>80.40000152587891</v>
+      </c>
+      <c r="D1255" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1255" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1256" t="n">
+        <v>4.079999923706055</v>
+      </c>
+      <c r="D1256" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1256" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1257" t="n">
+        <v>4.940000057220459</v>
+      </c>
+      <c r="D1257" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1257" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1258" t="n">
+        <v>5.739999771118164</v>
+      </c>
+      <c r="D1258" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1258" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1259" t="n">
+        <v>21.3799991607666</v>
+      </c>
+      <c r="D1259" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1259" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1260" t="n">
+        <v>32.04000091552734</v>
+      </c>
+      <c r="D1260" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1260" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1261" t="n">
+        <v>19.13999938964844</v>
+      </c>
+      <c r="D1261" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1261" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1262" t="n">
+        <v>5.420000076293945</v>
+      </c>
+      <c r="D1262" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1262" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1263" t="n">
+        <v>26.69000053405762</v>
+      </c>
+      <c r="D1263" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1263" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1264" t="n">
+        <v>14.23999977111816</v>
+      </c>
+      <c r="D1264" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1265" t="n">
+        <v>13.10000038146973</v>
+      </c>
+      <c r="D1265" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1266" t="n">
+        <v>18.77000045776367</v>
+      </c>
+      <c r="D1266" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1267" t="n">
+        <v>8.229999542236328</v>
+      </c>
+      <c r="D1267" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1268" t="n">
+        <v>57.79999923706055</v>
+      </c>
+      <c r="D1268" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1269" t="n">
+        <v>4.659999847412109</v>
+      </c>
+      <c r="D1269" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1270" t="n">
+        <v>71.30000305175781</v>
+      </c>
+      <c r="D1270" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1271" t="n">
+        <v>51.84999847412109</v>
+      </c>
+      <c r="D1271" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1272" t="n">
+        <v>21.09000015258789</v>
+      </c>
+      <c r="D1272" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1273" t="n">
+        <v>43.47999954223633</v>
+      </c>
+      <c r="D1273" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1274" t="n">
+        <v>135.7899932861328</v>
+      </c>
+      <c r="D1274" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1275" t="n">
+        <v>42.63999938964844</v>
+      </c>
+      <c r="D1275" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1276" t="n">
+        <v>6.610000133514404</v>
+      </c>
+      <c r="D1276" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1277" t="n">
+        <v>36.65000152587891</v>
+      </c>
+      <c r="D1277" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-22
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1277"/>
+  <dimension ref="A1:E1306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27185,6 +27185,615 @@
         </is>
       </c>
     </row>
+    <row r="1278">
+      <c r="A1278" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1278" t="n">
+        <v>34.70000076293945</v>
+      </c>
+      <c r="D1278" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1279" t="n">
+        <v>16.65999984741211</v>
+      </c>
+      <c r="D1279" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1280" t="n">
+        <v>23.82999992370605</v>
+      </c>
+      <c r="D1280" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1281" t="n">
+        <v>4.210000038146973</v>
+      </c>
+      <c r="D1281" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1282" t="n">
+        <v>1.309999942779541</v>
+      </c>
+      <c r="D1282" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1283" t="n">
+        <v>200.7299957275391</v>
+      </c>
+      <c r="D1283" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1284" t="n">
+        <v>79.40000152587891</v>
+      </c>
+      <c r="D1284" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1285" t="n">
+        <v>3.990000009536743</v>
+      </c>
+      <c r="D1285" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1286" t="n">
+        <v>4.980000019073486</v>
+      </c>
+      <c r="D1286" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1287" t="n">
+        <v>5.429999828338623</v>
+      </c>
+      <c r="D1287" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1288" t="n">
+        <v>21.29999923706055</v>
+      </c>
+      <c r="D1288" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1289" t="n">
+        <v>31.97999954223633</v>
+      </c>
+      <c r="D1289" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1290" t="n">
+        <v>18.81999969482422</v>
+      </c>
+      <c r="D1290" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1291" t="n">
+        <v>5.21999979019165</v>
+      </c>
+      <c r="D1291" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1292" t="n">
+        <v>26.44000053405762</v>
+      </c>
+      <c r="D1292" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1293" t="n">
+        <v>13.60000038146973</v>
+      </c>
+      <c r="D1293" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1294" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="D1294" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1295" t="n">
+        <v>18.26000022888184</v>
+      </c>
+      <c r="D1295" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1296" t="n">
+        <v>8.260000228881836</v>
+      </c>
+      <c r="D1296" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1297" t="n">
+        <v>57.7599983215332</v>
+      </c>
+      <c r="D1297" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1298" t="n">
+        <v>4.739999771118164</v>
+      </c>
+      <c r="D1298" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1299" t="n">
+        <v>72.62999725341797</v>
+      </c>
+      <c r="D1299" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1300" t="n">
+        <v>51.59000015258789</v>
+      </c>
+      <c r="D1300" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1301" t="n">
+        <v>20.26000022888184</v>
+      </c>
+      <c r="D1301" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1302" t="n">
+        <v>43.93999862670898</v>
+      </c>
+      <c r="D1302" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1303" t="n">
+        <v>134.6499938964844</v>
+      </c>
+      <c r="D1303" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1304" t="n">
+        <v>42.90000152587891</v>
+      </c>
+      <c r="D1304" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1305" t="n">
+        <v>6.329999923706055</v>
+      </c>
+      <c r="D1305" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1306" t="n">
+        <v>36.77999877929688</v>
+      </c>
+      <c r="D1306" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-23
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1306"/>
+  <dimension ref="A1:E1335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27794,6 +27794,615 @@
         </is>
       </c>
     </row>
+    <row r="1307">
+      <c r="A1307" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1307" t="n">
+        <v>35.13000106811523</v>
+      </c>
+      <c r="D1307" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1308" t="n">
+        <v>16.86000061035156</v>
+      </c>
+      <c r="D1308" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1309" t="n">
+        <v>24.85000038146973</v>
+      </c>
+      <c r="D1309" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1310" t="n">
+        <v>4.260000228881836</v>
+      </c>
+      <c r="D1310" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1311" t="n">
+        <v>1.440000057220459</v>
+      </c>
+      <c r="D1311" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1312" t="n">
+        <v>202.3699951171875</v>
+      </c>
+      <c r="D1312" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1313" t="n">
+        <v>80.09999847412109</v>
+      </c>
+      <c r="D1313" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1314" t="n">
+        <v>4.210000038146973</v>
+      </c>
+      <c r="D1314" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1315" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1315" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1316" t="n">
+        <v>6.039999961853027</v>
+      </c>
+      <c r="D1316" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1317" t="n">
+        <v>21.45999908447266</v>
+      </c>
+      <c r="D1317" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1318" t="n">
+        <v>31.46999931335449</v>
+      </c>
+      <c r="D1318" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1319" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="D1319" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1320" t="n">
+        <v>5.320000171661377</v>
+      </c>
+      <c r="D1320" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1321" t="n">
+        <v>27.21999931335449</v>
+      </c>
+      <c r="D1321" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1322" t="n">
+        <v>13.92000007629395</v>
+      </c>
+      <c r="D1322" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1323" t="n">
+        <v>12.76000022888184</v>
+      </c>
+      <c r="D1323" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1324" t="n">
+        <v>18.95000076293945</v>
+      </c>
+      <c r="D1324" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1325" t="n">
+        <v>8.300000190734863</v>
+      </c>
+      <c r="D1325" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1326" t="n">
+        <v>58.83000183105469</v>
+      </c>
+      <c r="D1326" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1327" t="n">
+        <v>4.78000020980835</v>
+      </c>
+      <c r="D1327" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1328" t="n">
+        <v>73.87000274658203</v>
+      </c>
+      <c r="D1328" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1329" t="n">
+        <v>51.52000045776367</v>
+      </c>
+      <c r="D1329" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1330" t="n">
+        <v>20.35000038146973</v>
+      </c>
+      <c r="D1330" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1331" t="n">
+        <v>43.66999816894531</v>
+      </c>
+      <c r="D1331" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1332" t="n">
+        <v>137.5899963378906</v>
+      </c>
+      <c r="D1332" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1333" t="n">
+        <v>42.84999847412109</v>
+      </c>
+      <c r="D1333" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1334" t="n">
+        <v>6.670000076293945</v>
+      </c>
+      <c r="D1334" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1335" t="n">
+        <v>35.90000152587891</v>
+      </c>
+      <c r="D1335" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-26
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1335"/>
+  <dimension ref="A1:E1364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28403,6 +28403,615 @@
         </is>
       </c>
     </row>
+    <row r="1336">
+      <c r="A1336" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1336" t="n">
+        <v>26.48999977111816</v>
+      </c>
+      <c r="D1336" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1337" t="n">
+        <v>13.27000045776367</v>
+      </c>
+      <c r="D1337" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1338" t="n">
+        <v>17.96999931335449</v>
+      </c>
+      <c r="D1338" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1339" t="n">
+        <v>3.319999933242798</v>
+      </c>
+      <c r="D1339" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1340" t="n">
+        <v>0.8999999761581421</v>
+      </c>
+      <c r="D1340" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1341" t="n">
+        <v>174.1000061035156</v>
+      </c>
+      <c r="D1341" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1342" t="n">
+        <v>60.4900016784668</v>
+      </c>
+      <c r="D1342" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1343" t="n">
+        <v>3.099999904632568</v>
+      </c>
+      <c r="D1343" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1344" t="n">
+        <v>4.739999771118164</v>
+      </c>
+      <c r="D1344" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1345" t="n">
+        <v>5.039999961853027</v>
+      </c>
+      <c r="D1345" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1346" t="n">
+        <v>21.04999923706055</v>
+      </c>
+      <c r="D1346" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1347" t="n">
+        <v>26.80999946594238</v>
+      </c>
+      <c r="D1347" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1348" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="D1348" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1349" t="n">
+        <v>3.660000085830688</v>
+      </c>
+      <c r="D1349" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1350" t="n">
+        <v>20.55999946594238</v>
+      </c>
+      <c r="D1350" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1351" t="n">
+        <v>10.89999961853027</v>
+      </c>
+      <c r="D1351" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1352" t="n">
+        <v>5.380000114440918</v>
+      </c>
+      <c r="D1352" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1353" t="n">
+        <v>7.710000038146973</v>
+      </c>
+      <c r="D1353" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1354" t="n">
+        <v>4.699999809265137</v>
+      </c>
+      <c r="D1354" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1355" t="n">
+        <v>53.72000122070312</v>
+      </c>
+      <c r="D1355" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1356" t="n">
+        <v>4.090000152587891</v>
+      </c>
+      <c r="D1356" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1357" t="n">
+        <v>71.19999694824219</v>
+      </c>
+      <c r="D1357" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1358" t="n">
+        <v>48.2400016784668</v>
+      </c>
+      <c r="D1358" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1359" t="n">
+        <v>15.72000026702881</v>
+      </c>
+      <c r="D1359" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1360" t="n">
+        <v>35.02999877929688</v>
+      </c>
+      <c r="D1360" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1361" t="n">
+        <v>99.81999969482422</v>
+      </c>
+      <c r="D1361" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1362" t="n">
+        <v>47.63000106811523</v>
+      </c>
+      <c r="D1362" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1363" t="n">
+        <v>5.940000057220459</v>
+      </c>
+      <c r="D1363" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1364" t="n">
+        <v>32.18000030517578</v>
+      </c>
+      <c r="D1364" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-27
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1364"/>
+  <dimension ref="A1:E1393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29012,6 +29012,615 @@
         </is>
       </c>
     </row>
+    <row r="1365">
+      <c r="A1365" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1365" t="n">
+        <v>25.79000091552734</v>
+      </c>
+      <c r="D1365" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1366" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="D1366" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1367" t="n">
+        <v>17.42000007629395</v>
+      </c>
+      <c r="D1367" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1367" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1368" t="n">
+        <v>3.180000066757202</v>
+      </c>
+      <c r="D1368" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1369" t="n">
+        <v>0.9200000166893005</v>
+      </c>
+      <c r="D1369" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1370" t="n">
+        <v>172.9600067138672</v>
+      </c>
+      <c r="D1370" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1371" t="n">
+        <v>60.15999984741211</v>
+      </c>
+      <c r="D1371" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1372" t="n">
+        <v>3.799999952316284</v>
+      </c>
+      <c r="D1372" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1373" t="n">
+        <v>4.559999942779541</v>
+      </c>
+      <c r="D1373" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1374" t="n">
+        <v>4.769999980926514</v>
+      </c>
+      <c r="D1374" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1375" t="n">
+        <v>21.52000045776367</v>
+      </c>
+      <c r="D1375" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1376" t="n">
+        <v>27.06999969482422</v>
+      </c>
+      <c r="D1376" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1377" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D1377" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1378" t="n">
+        <v>3.809999942779541</v>
+      </c>
+      <c r="D1378" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1379" t="n">
+        <v>21.54999923706055</v>
+      </c>
+      <c r="D1379" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1380" t="n">
+        <v>10.4399995803833</v>
+      </c>
+      <c r="D1380" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1381" t="n">
+        <v>5.710000038146973</v>
+      </c>
+      <c r="D1381" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1382" t="n">
+        <v>7.789999961853027</v>
+      </c>
+      <c r="D1382" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1383" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D1383" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1384" t="n">
+        <v>52.91999816894531</v>
+      </c>
+      <c r="D1384" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1385" t="n">
+        <v>4.050000190734863</v>
+      </c>
+      <c r="D1385" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1386" t="n">
+        <v>70.61000061035156</v>
+      </c>
+      <c r="D1386" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1387" t="n">
+        <v>48.04999923706055</v>
+      </c>
+      <c r="D1387" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1388" t="n">
+        <v>16.10000038146973</v>
+      </c>
+      <c r="D1388" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1389" t="n">
+        <v>34.88999938964844</v>
+      </c>
+      <c r="D1389" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1390" t="n">
+        <v>99.30000305175781</v>
+      </c>
+      <c r="D1390" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1391" t="n">
+        <v>47.52000045776367</v>
+      </c>
+      <c r="D1391" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1392" t="n">
+        <v>5.71999979019165</v>
+      </c>
+      <c r="D1392" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1393" t="n">
+        <v>32.09999847412109</v>
+      </c>
+      <c r="D1393" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-28
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1393"/>
+  <dimension ref="A1:E1422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29621,6 +29621,615 @@
         </is>
       </c>
     </row>
+    <row r="1394">
+      <c r="A1394" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1394" t="n">
+        <v>24.44000053405762</v>
+      </c>
+      <c r="D1394" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1395" t="n">
+        <v>13.44999980926514</v>
+      </c>
+      <c r="D1395" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1396" t="n">
+        <v>16.82999992370605</v>
+      </c>
+      <c r="D1396" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1397" t="n">
+        <v>2.890000104904175</v>
+      </c>
+      <c r="D1397" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1398" t="n">
+        <v>0.7400000095367432</v>
+      </c>
+      <c r="D1398" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1399" t="n">
+        <v>168.1999969482422</v>
+      </c>
+      <c r="D1399" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1400" t="n">
+        <v>56.43999862670898</v>
+      </c>
+      <c r="D1400" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1400" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1401" t="n">
+        <v>3.299999952316284</v>
+      </c>
+      <c r="D1401" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1402" t="n">
+        <v>4.429999828338623</v>
+      </c>
+      <c r="D1402" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1403" t="n">
+        <v>4.349999904632568</v>
+      </c>
+      <c r="D1403" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1404" t="n">
+        <v>21.13999938964844</v>
+      </c>
+      <c r="D1404" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1404" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1405" t="n">
+        <v>26.45999908447266</v>
+      </c>
+      <c r="D1405" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1405" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1406" t="n">
+        <v>9.670000076293945</v>
+      </c>
+      <c r="D1406" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1406" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1407" t="n">
+        <v>3.539999961853027</v>
+      </c>
+      <c r="D1407" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1407" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1408" t="n">
+        <v>21.53000068664551</v>
+      </c>
+      <c r="D1408" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1408" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1409" t="n">
+        <v>9.670000076293945</v>
+      </c>
+      <c r="D1409" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1409" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1410" t="n">
+        <v>5.179999828338623</v>
+      </c>
+      <c r="D1410" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1410" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1411" t="n">
+        <v>6.630000114440918</v>
+      </c>
+      <c r="D1411" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1411" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1412" t="n">
+        <v>4.300000190734863</v>
+      </c>
+      <c r="D1412" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1412" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1413" t="n">
+        <v>52.72999954223633</v>
+      </c>
+      <c r="D1413" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1413" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1414" t="n">
+        <v>3.900000095367432</v>
+      </c>
+      <c r="D1414" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1414" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1415" t="n">
+        <v>72</v>
+      </c>
+      <c r="D1415" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1415" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1416" t="n">
+        <v>46.84000015258789</v>
+      </c>
+      <c r="D1416" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1416" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1417" t="n">
+        <v>15.69999980926514</v>
+      </c>
+      <c r="D1417" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1417" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1418" t="n">
+        <v>33.84000015258789</v>
+      </c>
+      <c r="D1418" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1418" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1419" t="n">
+        <v>95.25</v>
+      </c>
+      <c r="D1419" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1419" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1420" t="n">
+        <v>48.15000152587891</v>
+      </c>
+      <c r="D1420" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1420" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1421" t="n">
+        <v>5.670000076293945</v>
+      </c>
+      <c r="D1421" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1421" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1422" t="n">
+        <v>30.65999984741211</v>
+      </c>
+      <c r="D1422" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1422" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-29
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1422"/>
+  <dimension ref="A1:E1451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30230,6 +30230,615 @@
         </is>
       </c>
     </row>
+    <row r="1423">
+      <c r="A1423" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1423" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="D1423" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1423" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1424" t="n">
+        <v>12.9399995803833</v>
+      </c>
+      <c r="D1424" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1424" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1425" t="n">
+        <v>16.46999931335449</v>
+      </c>
+      <c r="D1425" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1425" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1426" t="n">
+        <v>2.660000085830688</v>
+      </c>
+      <c r="D1426" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1426" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1427" t="n">
+        <v>0.6399999856948853</v>
+      </c>
+      <c r="D1427" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1427" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1428" t="n">
+        <v>166.7799987792969</v>
+      </c>
+      <c r="D1428" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1428" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1429" t="n">
+        <v>54.27999877929688</v>
+      </c>
+      <c r="D1429" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1429" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1430" t="n">
+        <v>2.940000057220459</v>
+      </c>
+      <c r="D1430" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1430" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1431" t="n">
+        <v>4.559999942779541</v>
+      </c>
+      <c r="D1431" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1431" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1432" t="n">
+        <v>4.230000019073486</v>
+      </c>
+      <c r="D1432" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1432" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1433" t="n">
+        <v>21.46999931335449</v>
+      </c>
+      <c r="D1433" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1433" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1434" t="n">
+        <v>25.86000061035156</v>
+      </c>
+      <c r="D1434" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1434" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1435" t="n">
+        <v>9.130000114440918</v>
+      </c>
+      <c r="D1435" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1435" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1436" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1436" t="n">
+        <v>3.539999961853027</v>
+      </c>
+      <c r="D1436" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1436" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1437" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1437" t="n">
+        <v>21.40999984741211</v>
+      </c>
+      <c r="D1437" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1437" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1438" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1438" t="n">
+        <v>8.680000305175781</v>
+      </c>
+      <c r="D1438" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1438" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1439" t="n">
+        <v>5.130000114440918</v>
+      </c>
+      <c r="D1439" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1439" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1440" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1440" t="n">
+        <v>5.940000057220459</v>
+      </c>
+      <c r="D1440" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1440" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1441" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1441" t="n">
+        <v>4.070000171661377</v>
+      </c>
+      <c r="D1441" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1441" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1442" t="n">
+        <v>52.40000152587891</v>
+      </c>
+      <c r="D1442" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1442" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1443" t="n">
+        <v>3.829999923706055</v>
+      </c>
+      <c r="D1443" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1443" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1444" t="n">
+        <v>70.25</v>
+      </c>
+      <c r="D1444" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1444" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1445" t="n">
+        <v>45.95000076293945</v>
+      </c>
+      <c r="D1445" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1445" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1446" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="D1446" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1446" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1447" t="n">
+        <v>32.20999908447266</v>
+      </c>
+      <c r="D1447" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1447" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1448" t="n">
+        <v>93.02999877929688</v>
+      </c>
+      <c r="D1448" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1448" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1449" t="n">
+        <v>49.88000106811523</v>
+      </c>
+      <c r="D1449" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1449" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1450" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D1450" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1450" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1451" t="n">
+        <v>30.48999977111816</v>
+      </c>
+      <c r="D1451" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1451" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-10-30
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1451"/>
+  <dimension ref="A1:E1480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30839,6 +30839,615 @@
         </is>
       </c>
     </row>
+    <row r="1452">
+      <c r="A1452" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C1452" t="n">
+        <v>23.6200008392334</v>
+      </c>
+      <c r="D1452" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1452" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C1453" t="n">
+        <v>12.44999980926514</v>
+      </c>
+      <c r="D1453" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1453" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C1454" t="n">
+        <v>16.54999923706055</v>
+      </c>
+      <c r="D1454" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1454" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C1455" t="n">
+        <v>2.539999961853027</v>
+      </c>
+      <c r="D1455" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1455" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C1456" t="n">
+        <v>0.6899999976158142</v>
+      </c>
+      <c r="D1456" t="n">
+        <v>12</v>
+      </c>
+      <c r="E1456" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C1457" t="n">
+        <v>165.3899993896484</v>
+      </c>
+      <c r="D1457" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1457" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C1458" t="n">
+        <v>51.40000152587891</v>
+      </c>
+      <c r="D1458" t="n">
+        <v>45</v>
+      </c>
+      <c r="E1458" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C1459" t="n">
+        <v>2.970000028610229</v>
+      </c>
+      <c r="D1459" t="n">
+        <v>61</v>
+      </c>
+      <c r="E1459" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C1460" t="n">
+        <v>4.650000095367432</v>
+      </c>
+      <c r="D1460" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1460" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C1461" t="n">
+        <v>3.920000076293945</v>
+      </c>
+      <c r="D1461" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1461" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C1462" t="n">
+        <v>21.3700008392334</v>
+      </c>
+      <c r="D1462" t="n">
+        <v>49</v>
+      </c>
+      <c r="E1462" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C1463" t="n">
+        <v>25.68000030517578</v>
+      </c>
+      <c r="D1463" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1463" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C1464" t="n">
+        <v>8.979999542236328</v>
+      </c>
+      <c r="D1464" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1464" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C1465" t="n">
+        <v>3.480000019073486</v>
+      </c>
+      <c r="D1465" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1465" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C1466" t="n">
+        <v>21.3700008392334</v>
+      </c>
+      <c r="D1466" t="n">
+        <v>27</v>
+      </c>
+      <c r="E1466" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C1467" t="n">
+        <v>9.050000190734863</v>
+      </c>
+      <c r="D1467" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1467" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C1468" t="n">
+        <v>5.309999942779541</v>
+      </c>
+      <c r="D1468" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1468" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C1469" t="n">
+        <v>5.630000114440918</v>
+      </c>
+      <c r="D1469" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1469" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C1470" t="n">
+        <v>4.039999961853027</v>
+      </c>
+      <c r="D1470" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1470" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C1471" t="n">
+        <v>52.97000122070312</v>
+      </c>
+      <c r="D1471" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1471" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C1472" t="n">
+        <v>3.730000019073486</v>
+      </c>
+      <c r="D1472" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1472" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C1473" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="D1473" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1473" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1474" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C1474" t="n">
+        <v>44.9900016784668</v>
+      </c>
+      <c r="D1474" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1474" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C1475" t="n">
+        <v>15.15999984741211</v>
+      </c>
+      <c r="D1475" t="n">
+        <v>63</v>
+      </c>
+      <c r="E1475" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1476" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C1476" t="n">
+        <v>31.59000015258789</v>
+      </c>
+      <c r="D1476" t="n">
+        <v>35</v>
+      </c>
+      <c r="E1476" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1477" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C1477" t="n">
+        <v>92.44999694824219</v>
+      </c>
+      <c r="D1477" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1477" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1478" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C1478" t="n">
+        <v>50.40000152587891</v>
+      </c>
+      <c r="D1478" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1478" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1479" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C1479" t="n">
+        <v>5.019999980926514</v>
+      </c>
+      <c r="D1479" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1479" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1480" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C1480" t="n">
+        <v>29.52000045776367</v>
+      </c>
+      <c r="D1480" t="n">
+        <v>48</v>
+      </c>
+      <c r="E1480" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>